<commit_message>
Zeitplan, Doku, Readme aktu..., imageView delete
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA124D1-5080-4545-BEBE-4EA4CAA21AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5EA8FE-3CF0-4EEC-A5E8-294CF2E89915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
   <si>
     <t>IPERKA Phase</t>
   </si>
@@ -153,12 +153,33 @@
   <si>
     <t>Benutzerverwaltung</t>
   </si>
+  <si>
+    <t>Login System</t>
+  </si>
+  <si>
+    <t>Benutzerrechte implementieren</t>
+  </si>
+  <si>
+    <t>Mockups</t>
+  </si>
+  <si>
+    <t>ERM-Diagramm</t>
+  </si>
+  <si>
+    <t>Actifity Diagramm</t>
+  </si>
+  <si>
+    <t>Klassendiagramm</t>
+  </si>
+  <si>
+    <t>0.166667</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -218,6 +239,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -751,7 +778,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -814,44 +841,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -862,8 +862,86 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -886,72 +964,36 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -1269,7 +1311,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BC55"/>
+  <dimension ref="A1:BC73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
@@ -1286,162 +1328,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="91" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65" t="s">
+      <c r="B1" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="68" t="s">
+      <c r="C1" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="69"/>
-      <c r="E1" s="48" t="s">
+      <c r="D1" s="86"/>
+      <c r="E1" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="48" t="s">
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="48" t="s">
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="49"/>
-      <c r="O1" s="49"/>
-      <c r="P1" s="50"/>
-      <c r="Q1" s="48" t="s">
+      <c r="N1" s="76"/>
+      <c r="O1" s="76"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="49"/>
-      <c r="S1" s="49"/>
-      <c r="T1" s="50"/>
-      <c r="U1" s="48" t="s">
+      <c r="R1" s="76"/>
+      <c r="S1" s="76"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="49"/>
-      <c r="W1" s="49"/>
-      <c r="X1" s="50"/>
-      <c r="Y1" s="48" t="s">
+      <c r="V1" s="76"/>
+      <c r="W1" s="76"/>
+      <c r="X1" s="77"/>
+      <c r="Y1" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="49"/>
-      <c r="AA1" s="49"/>
-      <c r="AB1" s="50"/>
-      <c r="AC1" s="48" t="s">
+      <c r="Z1" s="76"/>
+      <c r="AA1" s="76"/>
+      <c r="AB1" s="77"/>
+      <c r="AC1" s="75" t="s">
         <v>29</v>
       </c>
-      <c r="AD1" s="49"/>
-      <c r="AE1" s="49"/>
-      <c r="AF1" s="50"/>
-      <c r="AG1" s="48" t="s">
+      <c r="AD1" s="76"/>
+      <c r="AE1" s="76"/>
+      <c r="AF1" s="77"/>
+      <c r="AG1" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="49"/>
-      <c r="AI1" s="49"/>
-      <c r="AJ1" s="50"/>
-      <c r="AK1" s="48" t="s">
+      <c r="AH1" s="76"/>
+      <c r="AI1" s="76"/>
+      <c r="AJ1" s="77"/>
+      <c r="AK1" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="AL1" s="49"/>
-      <c r="AM1" s="49"/>
-      <c r="AN1" s="50"/>
-      <c r="AO1" s="48" t="s">
+      <c r="AL1" s="76"/>
+      <c r="AM1" s="76"/>
+      <c r="AN1" s="77"/>
+      <c r="AO1" s="75" t="s">
         <v>27</v>
       </c>
-      <c r="AP1" s="49"/>
-      <c r="AQ1" s="49"/>
-      <c r="AR1" s="50"/>
-      <c r="AS1" s="48"/>
-      <c r="AT1" s="49"/>
-      <c r="AU1" s="49"/>
-      <c r="AV1" s="50"/>
-      <c r="AW1" s="48"/>
-      <c r="AX1" s="49"/>
-      <c r="AY1" s="49"/>
-      <c r="AZ1" s="50"/>
+      <c r="AP1" s="76"/>
+      <c r="AQ1" s="76"/>
+      <c r="AR1" s="77"/>
+      <c r="AS1" s="75"/>
+      <c r="AT1" s="76"/>
+      <c r="AU1" s="76"/>
+      <c r="AV1" s="77"/>
+      <c r="AW1" s="75"/>
+      <c r="AX1" s="76"/>
+      <c r="AY1" s="76"/>
+      <c r="AZ1" s="77"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="59"/>
-      <c r="B2" s="66"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="55">
+      <c r="A2" s="92"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="79">
         <v>44781</v>
       </c>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="55">
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="79">
         <v>44782</v>
       </c>
-      <c r="J2" s="56"/>
-      <c r="K2" s="56"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="55">
+      <c r="J2" s="80"/>
+      <c r="K2" s="80"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="79">
         <v>44783</v>
       </c>
-      <c r="N2" s="56"/>
-      <c r="O2" s="56"/>
-      <c r="P2" s="57"/>
-      <c r="Q2" s="55">
+      <c r="N2" s="80"/>
+      <c r="O2" s="80"/>
+      <c r="P2" s="81"/>
+      <c r="Q2" s="79">
         <v>44784</v>
       </c>
-      <c r="R2" s="56"/>
-      <c r="S2" s="56"/>
-      <c r="T2" s="57"/>
-      <c r="U2" s="55">
+      <c r="R2" s="80"/>
+      <c r="S2" s="80"/>
+      <c r="T2" s="81"/>
+      <c r="U2" s="79">
         <v>44785</v>
       </c>
-      <c r="V2" s="56"/>
-      <c r="W2" s="56"/>
-      <c r="X2" s="57"/>
-      <c r="Y2" s="55">
+      <c r="V2" s="80"/>
+      <c r="W2" s="80"/>
+      <c r="X2" s="81"/>
+      <c r="Y2" s="79">
         <v>44789</v>
       </c>
-      <c r="Z2" s="56"/>
-      <c r="AA2" s="56"/>
-      <c r="AB2" s="57"/>
-      <c r="AC2" s="55">
+      <c r="Z2" s="80"/>
+      <c r="AA2" s="80"/>
+      <c r="AB2" s="81"/>
+      <c r="AC2" s="79">
         <v>44790</v>
       </c>
-      <c r="AD2" s="56"/>
-      <c r="AE2" s="56"/>
-      <c r="AF2" s="57"/>
-      <c r="AG2" s="55">
+      <c r="AD2" s="80"/>
+      <c r="AE2" s="80"/>
+      <c r="AF2" s="81"/>
+      <c r="AG2" s="79">
         <v>44791</v>
       </c>
-      <c r="AH2" s="56"/>
-      <c r="AI2" s="56"/>
-      <c r="AJ2" s="57"/>
-      <c r="AK2" s="55">
+      <c r="AH2" s="80"/>
+      <c r="AI2" s="80"/>
+      <c r="AJ2" s="81"/>
+      <c r="AK2" s="79">
         <v>44792</v>
       </c>
-      <c r="AL2" s="56"/>
-      <c r="AM2" s="56"/>
-      <c r="AN2" s="57"/>
-      <c r="AO2" s="55">
+      <c r="AL2" s="80"/>
+      <c r="AM2" s="80"/>
+      <c r="AN2" s="81"/>
+      <c r="AO2" s="79">
         <v>44795</v>
       </c>
-      <c r="AP2" s="56"/>
-      <c r="AQ2" s="56"/>
-      <c r="AR2" s="57"/>
-      <c r="AS2" s="55"/>
-      <c r="AT2" s="56"/>
-      <c r="AU2" s="56"/>
-      <c r="AV2" s="57"/>
-      <c r="AW2" s="55"/>
-      <c r="AX2" s="56"/>
-      <c r="AY2" s="56"/>
-      <c r="AZ2" s="57"/>
+      <c r="AP2" s="80"/>
+      <c r="AQ2" s="80"/>
+      <c r="AR2" s="81"/>
+      <c r="AS2" s="79"/>
+      <c r="AT2" s="80"/>
+      <c r="AU2" s="80"/>
+      <c r="AV2" s="81"/>
+      <c r="AW2" s="79"/>
+      <c r="AX2" s="80"/>
+      <c r="AY2" s="80"/>
+      <c r="AZ2" s="81"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="60"/>
-      <c r="B3" s="67"/>
+      <c r="A3" s="93"/>
+      <c r="B3" s="84"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
@@ -1579,11 +1621,11 @@
     </row>
     <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="77" t="s">
+      <c r="B4" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="53"/>
-      <c r="D4" s="88"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="67"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1639,9 +1681,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="72"/>
-      <c r="C5" s="64"/>
-      <c r="D5" s="87"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="66"/>
+      <c r="D5" s="68"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1697,9 +1739,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="79"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="51"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="51"/>
+      <c r="D6" s="59"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1744,9 +1786,9 @@
     </row>
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="76"/>
-      <c r="C7" s="64"/>
-      <c r="D7" s="87"/>
+      <c r="B7" s="48"/>
+      <c r="C7" s="66"/>
+      <c r="D7" s="68"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1801,16 +1843,16 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="61" t="s">
+      <c r="A8" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="81" t="s">
+      <c r="B8" s="55" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="83">
+      <c r="C8" s="57">
         <v>0.1</v>
       </c>
-      <c r="D8" s="92">
+      <c r="D8" s="73">
         <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
@@ -1867,10 +1909,10 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="62"/>
-      <c r="B9" s="52"/>
-      <c r="C9" s="54"/>
-      <c r="D9" s="93"/>
+      <c r="A9" s="53"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="51"/>
+      <c r="D9" s="74"/>
       <c r="E9" s="42"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -1921,14 +1963,14 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="62"/>
-      <c r="B10" s="52" t="s">
+      <c r="A10" s="53"/>
+      <c r="B10" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="53">
+      <c r="C10" s="65">
         <v>1</v>
       </c>
-      <c r="D10" s="53">
+      <c r="D10" s="65">
         <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
@@ -1981,10 +2023,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="62"/>
-      <c r="B11" s="52"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
+      <c r="A11" s="53"/>
+      <c r="B11" s="56"/>
+      <c r="C11" s="51"/>
+      <c r="D11" s="51"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2035,12 +2077,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="62"/>
-      <c r="B12" s="52" t="s">
+      <c r="A12" s="53"/>
+      <c r="B12" s="56" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="53"/>
-      <c r="D12" s="53"/>
+      <c r="C12" s="65"/>
+      <c r="D12" s="65"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2091,10 +2133,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="62"/>
-      <c r="B13" s="52"/>
-      <c r="C13" s="54"/>
-      <c r="D13" s="54"/>
+      <c r="A13" s="53"/>
+      <c r="B13" s="56"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="51"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2145,14 +2187,14 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="62"/>
-      <c r="B14" s="52" t="s">
+      <c r="A14" s="53"/>
+      <c r="B14" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="C14" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="53" t="s">
+      <c r="D14" s="65" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="42"/>
@@ -2205,10 +2247,10 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="62"/>
-      <c r="B15" s="52"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
+      <c r="A15" s="53"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
       <c r="E15" s="42"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -2259,14 +2301,14 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="62"/>
-      <c r="B16" s="72" t="s">
+      <c r="A16" s="53"/>
+      <c r="B16" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="54" t="s">
+      <c r="C16" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="51" t="s">
+      <c r="D16" s="59" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="20"/>
@@ -2319,10 +2361,10 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="63"/>
-      <c r="B17" s="73"/>
-      <c r="C17" s="74"/>
-      <c r="D17" s="75"/>
+      <c r="A17" s="54"/>
+      <c r="B17" s="89"/>
+      <c r="C17" s="61"/>
+      <c r="D17" s="62"/>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
@@ -2373,14 +2415,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="61" t="s">
+      <c r="A18" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="85" t="s">
+      <c r="B18" s="78" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="83"/>
-      <c r="D18" s="84"/>
+      <c r="C18" s="57"/>
+      <c r="D18" s="58"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2431,10 +2473,10 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="62"/>
-      <c r="B19" s="86"/>
-      <c r="C19" s="54"/>
-      <c r="D19" s="51"/>
+      <c r="A19" s="53"/>
+      <c r="B19" s="63"/>
+      <c r="C19" s="51"/>
+      <c r="D19" s="59"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2485,12 +2527,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="62"/>
-      <c r="B20" s="52" t="s">
+      <c r="A20" s="53"/>
+      <c r="B20" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="54"/>
-      <c r="D20" s="51"/>
+      <c r="C20" s="51"/>
+      <c r="D20" s="59"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2530,10 +2572,10 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="62"/>
-      <c r="B21" s="52"/>
-      <c r="C21" s="54"/>
-      <c r="D21" s="51"/>
+      <c r="A21" s="53"/>
+      <c r="B21" s="56"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="59"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2584,14 +2626,14 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="62"/>
-      <c r="B22" s="52" t="s">
+      <c r="A22" s="53"/>
+      <c r="B22" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="54">
+      <c r="C22" s="51">
         <v>0.1</v>
       </c>
-      <c r="D22" s="51">
+      <c r="D22" s="59">
         <v>0.1</v>
       </c>
       <c r="E22" s="11"/>
@@ -2644,10 +2686,10 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="62"/>
-      <c r="B23" s="52"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="51"/>
+      <c r="A23" s="53"/>
+      <c r="B23" s="56"/>
+      <c r="C23" s="51"/>
+      <c r="D23" s="59"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2698,10 +2740,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="62"/>
-      <c r="B24" s="72"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="89"/>
+      <c r="A24" s="53"/>
+      <c r="B24" s="64"/>
+      <c r="C24" s="66"/>
+      <c r="D24" s="70"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2752,10 +2794,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="62"/>
-      <c r="B25" s="77"/>
-      <c r="C25" s="53"/>
-      <c r="D25" s="90"/>
+      <c r="A25" s="53"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="65"/>
+      <c r="D25" s="71"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2806,12 +2848,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="62"/>
-      <c r="B26" s="52" t="s">
+      <c r="A26" s="53"/>
+      <c r="B26" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="64"/>
-      <c r="D26" s="89">
+      <c r="C26" s="66"/>
+      <c r="D26" s="70">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2864,10 +2906,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="63"/>
-      <c r="B27" s="52"/>
-      <c r="C27" s="78"/>
-      <c r="D27" s="91"/>
+      <c r="A27" s="54"/>
+      <c r="B27" s="56"/>
+      <c r="C27" s="90"/>
+      <c r="D27" s="72"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2918,14 +2960,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="61" t="s">
+      <c r="A28" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="81" t="s">
+      <c r="B28" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="83"/>
-      <c r="D28" s="84"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="58"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -2976,10 +3018,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="62"/>
-      <c r="B29" s="82"/>
-      <c r="C29" s="74"/>
-      <c r="D29" s="75"/>
+      <c r="A29" s="53"/>
+      <c r="B29" s="60"/>
+      <c r="C29" s="61"/>
+      <c r="D29" s="62"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3030,18 +3072,22 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="61" t="s">
+      <c r="A30" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="81" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="83"/>
-      <c r="D30" s="84"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="10"/>
+      <c r="B30" s="55" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="57">
+        <v>2</v>
+      </c>
+      <c r="D30" s="58">
+        <v>2</v>
+      </c>
+      <c r="E30" s="99"/>
+      <c r="F30" s="100"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="94"/>
       <c r="I30" s="8"/>
       <c r="J30" s="9"/>
       <c r="K30" s="9"/>
@@ -3088,14 +3134,14 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="62"/>
-      <c r="B31" s="52"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="51"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="13"/>
+      <c r="A31" s="53"/>
+      <c r="B31" s="56"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="59"/>
+      <c r="E31" s="105"/>
+      <c r="F31" s="106"/>
+      <c r="G31" s="43"/>
+      <c r="H31" s="95"/>
       <c r="I31" s="11"/>
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
@@ -3142,17 +3188,21 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="62"/>
-      <c r="B32" s="76" t="s">
-        <v>37</v>
-      </c>
-      <c r="C32" s="54"/>
-      <c r="D32" s="51"/>
+      <c r="A32" s="53"/>
+      <c r="B32" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="C32" s="51">
+        <v>4</v>
+      </c>
+      <c r="D32" s="51">
+        <v>7</v>
+      </c>
       <c r="E32" s="11"/>
       <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="11"/>
+      <c r="G32" s="101"/>
+      <c r="H32" s="102"/>
+      <c r="I32" s="103"/>
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
       <c r="L32" s="13"/>
@@ -3198,16 +3248,16 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="62"/>
-      <c r="B33" s="77"/>
-      <c r="C33" s="54"/>
+      <c r="A33" s="53"/>
+      <c r="B33" s="49"/>
+      <c r="C33" s="51"/>
       <c r="D33" s="51"/>
       <c r="E33" s="11"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="12"/>
+      <c r="F33" s="106"/>
+      <c r="G33" s="106"/>
+      <c r="H33" s="107"/>
+      <c r="I33" s="105"/>
+      <c r="J33" s="106"/>
       <c r="K33" s="12"/>
       <c r="L33" s="13"/>
       <c r="M33" s="11"/>
@@ -3251,19 +3301,23 @@
       <c r="AY33" s="12"/>
       <c r="AZ33" s="13"/>
     </row>
-    <row r="34" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A34" s="62"/>
-      <c r="B34" s="76" t="s">
-        <v>38</v>
-      </c>
-      <c r="C34" s="80"/>
-      <c r="D34" s="51"/>
+    <row r="34" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="53"/>
+      <c r="B34" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="51" t="s">
+        <v>34</v>
+      </c>
+      <c r="D34" s="51" t="s">
+        <v>34</v>
+      </c>
       <c r="E34" s="11"/>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
       <c r="H34" s="13"/>
-      <c r="I34" s="11"/>
-      <c r="J34" s="12"/>
+      <c r="I34" s="103"/>
+      <c r="J34" s="43"/>
       <c r="K34" s="12"/>
       <c r="L34" s="13"/>
       <c r="M34" s="11"/>
@@ -3307,16 +3361,16 @@
       <c r="AY34" s="12"/>
       <c r="AZ34" s="13"/>
     </row>
-    <row r="35" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A35" s="62"/>
-      <c r="B35" s="77"/>
-      <c r="C35" s="80"/>
+    <row r="35" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="53"/>
+      <c r="B35" s="49"/>
+      <c r="C35" s="51"/>
       <c r="D35" s="51"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
       <c r="H35" s="13"/>
-      <c r="I35" s="11"/>
+      <c r="I35" s="108"/>
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
       <c r="L35" s="13"/>
@@ -3361,19 +3415,23 @@
       <c r="AY35" s="12"/>
       <c r="AZ35" s="13"/>
     </row>
-    <row r="36" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A36" s="62"/>
-      <c r="B36" s="76" t="s">
-        <v>39</v>
-      </c>
-      <c r="C36" s="80"/>
-      <c r="D36" s="51"/>
+    <row r="36" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="53"/>
+      <c r="B36" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="C36" s="51">
+        <v>1.5</v>
+      </c>
+      <c r="D36" s="51">
+        <v>2</v>
+      </c>
       <c r="E36" s="11"/>
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
       <c r="H36" s="13"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="12"/>
+      <c r="I36" s="104"/>
+      <c r="J36" s="101"/>
       <c r="K36" s="12"/>
       <c r="L36" s="13"/>
       <c r="M36" s="11"/>
@@ -3417,18 +3475,18 @@
       <c r="AY36" s="12"/>
       <c r="AZ36" s="13"/>
     </row>
-    <row r="37" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A37" s="62"/>
-      <c r="B37" s="77"/>
-      <c r="C37" s="80"/>
+    <row r="37" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="53"/>
+      <c r="B37" s="49"/>
+      <c r="C37" s="51"/>
       <c r="D37" s="51"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
       <c r="H37" s="13"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
+      <c r="I37" s="96"/>
+      <c r="J37" s="106"/>
+      <c r="K37" s="97"/>
       <c r="L37" s="13"/>
       <c r="M37" s="11"/>
       <c r="N37" s="12"/>
@@ -3471,21 +3529,27 @@
       <c r="AY37" s="12"/>
       <c r="AZ37" s="13"/>
     </row>
-    <row r="38" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A38" s="62"/>
-      <c r="B38" s="76"/>
-      <c r="C38" s="80"/>
-      <c r="D38" s="51"/>
+    <row r="38" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="53"/>
+      <c r="B38" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="C38" s="51">
+        <v>7</v>
+      </c>
+      <c r="D38" s="59">
+        <v>4</v>
+      </c>
       <c r="E38" s="11"/>
       <c r="F38" s="12"/>
       <c r="G38" s="12"/>
       <c r="H38" s="13"/>
       <c r="I38" s="11"/>
       <c r="J38" s="12"/>
-      <c r="K38" s="12"/>
-      <c r="L38" s="13"/>
-      <c r="M38" s="11"/>
-      <c r="N38" s="12"/>
+      <c r="K38" s="101"/>
+      <c r="L38" s="102"/>
+      <c r="M38" s="103"/>
+      <c r="N38" s="101"/>
       <c r="O38" s="12"/>
       <c r="P38" s="13"/>
       <c r="Q38" s="11"/>
@@ -3525,25 +3589,25 @@
       <c r="AY38" s="12"/>
       <c r="AZ38" s="13"/>
     </row>
-    <row r="39" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A39" s="62"/>
-      <c r="B39" s="77"/>
-      <c r="C39" s="54"/>
-      <c r="D39" s="51"/>
+    <row r="39" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="53"/>
+      <c r="B39" s="49"/>
+      <c r="C39" s="51"/>
+      <c r="D39" s="59"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
       <c r="H39" s="13"/>
       <c r="I39" s="11"/>
-      <c r="J39" s="12"/>
-      <c r="K39" s="12"/>
+      <c r="J39" s="106"/>
+      <c r="K39" s="43"/>
       <c r="L39" s="13"/>
       <c r="M39" s="11"/>
       <c r="N39" s="12"/>
       <c r="O39" s="12"/>
       <c r="P39" s="13"/>
-      <c r="Q39" s="11"/>
-      <c r="R39" s="12"/>
+      <c r="Q39" s="105"/>
+      <c r="R39" s="106"/>
       <c r="S39" s="12"/>
       <c r="T39" s="13"/>
       <c r="U39" s="11"/>
@@ -3579,22 +3643,24 @@
       <c r="AY39" s="12"/>
       <c r="AZ39" s="13"/>
     </row>
-    <row r="40" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A40" s="62"/>
-      <c r="B40" s="79" t="s">
-        <v>26</v>
-      </c>
-      <c r="C40" s="54"/>
-      <c r="D40" s="51"/>
+    <row r="40" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="53"/>
+      <c r="B40" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="C40" s="51">
+        <v>6</v>
+      </c>
+      <c r="D40" s="59"/>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
       <c r="H40" s="13"/>
       <c r="I40" s="11"/>
       <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
-      <c r="L40" s="13"/>
-      <c r="M40" s="11"/>
+      <c r="K40" s="101"/>
+      <c r="L40" s="102"/>
+      <c r="M40" s="103"/>
       <c r="N40" s="12"/>
       <c r="O40" s="12"/>
       <c r="P40" s="13"/>
@@ -3635,27 +3701,27 @@
       <c r="AY40" s="12"/>
       <c r="AZ40" s="13"/>
     </row>
-    <row r="41" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A41" s="62"/>
-      <c r="B41" s="79"/>
-      <c r="C41" s="54"/>
-      <c r="D41" s="51"/>
+    <row r="41" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="53"/>
+      <c r="B41" s="49"/>
+      <c r="C41" s="51"/>
+      <c r="D41" s="59"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
       <c r="H41" s="13"/>
       <c r="I41" s="11"/>
       <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
-      <c r="L41" s="13"/>
-      <c r="M41" s="11"/>
-      <c r="N41" s="12"/>
-      <c r="O41" s="12"/>
-      <c r="P41" s="13"/>
-      <c r="Q41" s="11"/>
-      <c r="R41" s="12"/>
-      <c r="S41" s="12"/>
-      <c r="T41" s="13"/>
+      <c r="K41" s="106"/>
+      <c r="L41" s="107"/>
+      <c r="M41" s="105"/>
+      <c r="N41" s="43"/>
+      <c r="O41" s="97"/>
+      <c r="P41" s="107"/>
+      <c r="Q41" s="42"/>
+      <c r="R41" s="43"/>
+      <c r="S41" s="106"/>
+      <c r="T41" s="107"/>
       <c r="U41" s="11"/>
       <c r="V41" s="12"/>
       <c r="W41" s="12"/>
@@ -3690,26 +3756,28 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="62"/>
-      <c r="B42" s="52" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="54"/>
-      <c r="D42" s="51">
-        <v>0</v>
+      <c r="A42" s="53"/>
+      <c r="B42" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="C42" s="51">
+        <v>4</v>
+      </c>
+      <c r="D42" s="59">
+        <v>2</v>
       </c>
       <c r="E42" s="11"/>
       <c r="F42" s="12"/>
       <c r="G42" s="12"/>
       <c r="H42" s="13"/>
       <c r="I42" s="11"/>
-      <c r="J42" s="12"/>
-      <c r="K42" s="12"/>
-      <c r="L42" s="13"/>
-      <c r="M42" s="11"/>
-      <c r="N42" s="12"/>
-      <c r="O42" s="12"/>
-      <c r="P42" s="13"/>
+      <c r="J42" s="101"/>
+      <c r="K42" s="101"/>
+      <c r="L42" s="95"/>
+      <c r="M42" s="42"/>
+      <c r="N42" s="43"/>
+      <c r="O42" s="43"/>
+      <c r="P42" s="95"/>
       <c r="Q42" s="11"/>
       <c r="R42" s="12"/>
       <c r="S42" s="12"/>
@@ -3747,27 +3815,27 @@
       <c r="AY42" s="12"/>
       <c r="AZ42" s="13"/>
     </row>
-    <row r="43" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="62"/>
-      <c r="B43" s="52"/>
-      <c r="C43" s="54"/>
-      <c r="D43" s="51"/>
+    <row r="43" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A43" s="53"/>
+      <c r="B43" s="49"/>
+      <c r="C43" s="51"/>
+      <c r="D43" s="59"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
       <c r="H43" s="13"/>
       <c r="I43" s="11"/>
-      <c r="J43" s="12"/>
-      <c r="K43" s="12"/>
-      <c r="L43" s="13"/>
-      <c r="M43" s="11"/>
-      <c r="N43" s="12"/>
-      <c r="O43" s="12"/>
-      <c r="P43" s="13"/>
-      <c r="Q43" s="11"/>
-      <c r="R43" s="12"/>
-      <c r="S43" s="12"/>
-      <c r="T43" s="13"/>
+      <c r="J43" s="106"/>
+      <c r="K43" s="106"/>
+      <c r="L43" s="98"/>
+      <c r="M43" s="42"/>
+      <c r="N43" s="43"/>
+      <c r="O43" s="43"/>
+      <c r="P43" s="95"/>
+      <c r="Q43" s="42"/>
+      <c r="R43" s="43"/>
+      <c r="S43" s="43"/>
+      <c r="T43" s="95"/>
       <c r="U43" s="11"/>
       <c r="V43" s="12"/>
       <c r="W43" s="12"/>
@@ -3801,81 +3869,77 @@
       <c r="AY43" s="12"/>
       <c r="AZ43" s="13"/>
     </row>
-    <row r="44" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A44" s="61" t="s">
-        <v>14</v>
-      </c>
-      <c r="B44" s="81" t="s">
-        <v>22</v>
-      </c>
-      <c r="C44" s="83"/>
-      <c r="D44" s="84"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="9"/>
-      <c r="G44" s="9"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="8"/>
-      <c r="J44" s="9"/>
-      <c r="K44" s="9"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="8"/>
-      <c r="N44" s="9"/>
-      <c r="O44" s="9"/>
-      <c r="P44" s="10"/>
-      <c r="Q44" s="8"/>
-      <c r="R44" s="9"/>
-      <c r="S44" s="9"/>
-      <c r="T44" s="10"/>
-      <c r="U44" s="8"/>
-      <c r="V44" s="9"/>
-      <c r="W44" s="9"/>
-      <c r="X44" s="10"/>
-      <c r="Y44" s="8"/>
-      <c r="Z44" s="9"/>
-      <c r="AA44" s="9"/>
-      <c r="AB44" s="10"/>
-      <c r="AC44" s="8"/>
-      <c r="AD44" s="9"/>
-      <c r="AE44" s="9"/>
-      <c r="AF44" s="10"/>
-      <c r="AG44" s="8"/>
-      <c r="AH44" s="9"/>
-      <c r="AI44" s="9"/>
-      <c r="AJ44" s="10"/>
-      <c r="AK44" s="8"/>
-      <c r="AL44" s="9"/>
-      <c r="AM44" s="9"/>
-      <c r="AN44" s="10"/>
-      <c r="AO44" s="8"/>
-      <c r="AP44" s="9"/>
-      <c r="AQ44" s="9"/>
-      <c r="AR44" s="10"/>
-      <c r="AS44" s="8"/>
-      <c r="AT44" s="9"/>
-      <c r="AU44" s="9"/>
-      <c r="AV44" s="10"/>
-      <c r="AW44" s="8"/>
-      <c r="AX44" s="9"/>
-      <c r="AY44" s="9"/>
-      <c r="AZ44" s="10"/>
-    </row>
-    <row r="45" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A45" s="62"/>
-      <c r="B45" s="52"/>
-      <c r="C45" s="54"/>
-      <c r="D45" s="51"/>
+    <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="53"/>
+      <c r="B44" s="48"/>
+      <c r="C44" s="51"/>
+      <c r="D44" s="59"/>
+      <c r="E44" s="11"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="13"/>
+      <c r="I44" s="11"/>
+      <c r="J44" s="12"/>
+      <c r="K44" s="43"/>
+      <c r="L44" s="95"/>
+      <c r="M44" s="42"/>
+      <c r="N44" s="43"/>
+      <c r="O44" s="43"/>
+      <c r="P44" s="95"/>
+      <c r="Q44" s="11"/>
+      <c r="R44" s="12"/>
+      <c r="S44" s="12"/>
+      <c r="T44" s="13"/>
+      <c r="U44" s="11"/>
+      <c r="V44" s="12"/>
+      <c r="W44" s="12"/>
+      <c r="X44" s="13"/>
+      <c r="Y44" s="11"/>
+      <c r="Z44" s="12"/>
+      <c r="AA44" s="12"/>
+      <c r="AB44" s="13"/>
+      <c r="AC44" s="11"/>
+      <c r="AD44" s="12"/>
+      <c r="AE44" s="12"/>
+      <c r="AF44" s="13"/>
+      <c r="AG44" s="11"/>
+      <c r="AH44" s="12"/>
+      <c r="AI44" s="12"/>
+      <c r="AJ44" s="13"/>
+      <c r="AK44" s="11"/>
+      <c r="AL44" s="12"/>
+      <c r="AM44" s="12"/>
+      <c r="AN44" s="13"/>
+      <c r="AO44" s="11"/>
+      <c r="AP44" s="12"/>
+      <c r="AQ44" s="12"/>
+      <c r="AR44" s="13"/>
+      <c r="AS44" s="11"/>
+      <c r="AT44" s="12"/>
+      <c r="AU44" s="12"/>
+      <c r="AV44" s="13"/>
+      <c r="AW44" s="11"/>
+      <c r="AX44" s="12"/>
+      <c r="AY44" s="12"/>
+      <c r="AZ44" s="13"/>
+    </row>
+    <row r="45" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="53"/>
+      <c r="B45" s="49"/>
+      <c r="C45" s="51"/>
+      <c r="D45" s="59"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
       <c r="H45" s="13"/>
       <c r="I45" s="11"/>
       <c r="J45" s="12"/>
-      <c r="K45" s="12"/>
-      <c r="L45" s="13"/>
-      <c r="M45" s="11"/>
-      <c r="N45" s="12"/>
-      <c r="O45" s="12"/>
-      <c r="P45" s="13"/>
+      <c r="K45" s="43"/>
+      <c r="L45" s="95"/>
+      <c r="M45" s="42"/>
+      <c r="N45" s="43"/>
+      <c r="O45" s="43"/>
+      <c r="P45" s="95"/>
       <c r="Q45" s="11"/>
       <c r="R45" s="12"/>
       <c r="S45" s="12"/>
@@ -3913,25 +3977,23 @@
       <c r="AY45" s="12"/>
       <c r="AZ45" s="13"/>
     </row>
-    <row r="46" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="62"/>
-      <c r="B46" s="76" t="s">
-        <v>23</v>
-      </c>
-      <c r="C46" s="80"/>
-      <c r="D46" s="80"/>
+    <row r="46" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A46" s="53"/>
+      <c r="B46" s="48"/>
+      <c r="C46" s="50"/>
+      <c r="D46" s="59"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
       <c r="H46" s="13"/>
       <c r="I46" s="11"/>
       <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
-      <c r="L46" s="13"/>
-      <c r="M46" s="11"/>
-      <c r="N46" s="12"/>
-      <c r="O46" s="12"/>
-      <c r="P46" s="13"/>
+      <c r="K46" s="43"/>
+      <c r="L46" s="95"/>
+      <c r="M46" s="42"/>
+      <c r="N46" s="43"/>
+      <c r="O46" s="43"/>
+      <c r="P46" s="95"/>
       <c r="Q46" s="11"/>
       <c r="R46" s="12"/>
       <c r="S46" s="12"/>
@@ -3969,11 +4031,11 @@
       <c r="AY46" s="12"/>
       <c r="AZ46" s="13"/>
     </row>
-    <row r="47" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="62"/>
-      <c r="B47" s="77"/>
-      <c r="C47" s="54"/>
-      <c r="D47" s="54"/>
+    <row r="47" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A47" s="53"/>
+      <c r="B47" s="49"/>
+      <c r="C47" s="50"/>
+      <c r="D47" s="59"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -4024,11 +4086,9 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="62"/>
-      <c r="B48" s="52" t="s">
-        <v>24</v>
-      </c>
-      <c r="C48" s="54"/>
+      <c r="A48" s="53"/>
+      <c r="B48" s="48"/>
+      <c r="C48" s="51"/>
       <c r="D48" s="51"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
@@ -4079,71 +4139,67 @@
       <c r="AY48" s="12"/>
       <c r="AZ48" s="13"/>
     </row>
-    <row r="49" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="63"/>
-      <c r="B49" s="82"/>
-      <c r="C49" s="74"/>
-      <c r="D49" s="75"/>
-      <c r="E49" s="17"/>
-      <c r="F49" s="18"/>
-      <c r="G49" s="18"/>
-      <c r="H49" s="19"/>
-      <c r="I49" s="17"/>
-      <c r="J49" s="18"/>
-      <c r="K49" s="18"/>
-      <c r="L49" s="19"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="18"/>
-      <c r="O49" s="18"/>
-      <c r="P49" s="19"/>
-      <c r="Q49" s="17"/>
-      <c r="R49" s="18"/>
-      <c r="S49" s="18"/>
-      <c r="T49" s="19"/>
-      <c r="U49" s="17"/>
-      <c r="V49" s="18"/>
-      <c r="W49" s="18"/>
-      <c r="X49" s="19"/>
-      <c r="Y49" s="17"/>
-      <c r="Z49" s="18"/>
-      <c r="AA49" s="18"/>
-      <c r="AB49" s="19"/>
-      <c r="AC49" s="17"/>
-      <c r="AD49" s="18"/>
-      <c r="AE49" s="18"/>
-      <c r="AF49" s="19"/>
-      <c r="AG49" s="17"/>
-      <c r="AH49" s="18"/>
-      <c r="AI49" s="18"/>
-      <c r="AJ49" s="19"/>
-      <c r="AK49" s="17"/>
-      <c r="AL49" s="18"/>
-      <c r="AM49" s="18"/>
-      <c r="AN49" s="19"/>
-      <c r="AO49" s="17"/>
-      <c r="AP49" s="18"/>
-      <c r="AQ49" s="18"/>
-      <c r="AR49" s="19"/>
-      <c r="AS49" s="17"/>
-      <c r="AT49" s="18"/>
-      <c r="AU49" s="18"/>
-      <c r="AV49" s="19"/>
-      <c r="AW49" s="17"/>
-      <c r="AX49" s="18"/>
-      <c r="AY49" s="18"/>
-      <c r="AZ49" s="19"/>
-    </row>
-    <row r="50" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="61" t="s">
-        <v>15</v>
-      </c>
-      <c r="B50" s="76" t="s">
-        <v>25</v>
-      </c>
-      <c r="C50" s="80"/>
-      <c r="D50" s="80"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="12"/>
+    <row r="49" spans="1:52" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="53"/>
+      <c r="B49" s="49"/>
+      <c r="C49" s="51"/>
+      <c r="D49" s="51"/>
+      <c r="E49" s="11"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="12"/>
+      <c r="H49" s="13"/>
+      <c r="I49" s="11"/>
+      <c r="J49" s="12"/>
+      <c r="K49" s="12"/>
+      <c r="L49" s="13"/>
+      <c r="M49" s="11"/>
+      <c r="N49" s="12"/>
+      <c r="O49" s="12"/>
+      <c r="P49" s="13"/>
+      <c r="Q49" s="11"/>
+      <c r="R49" s="12"/>
+      <c r="S49" s="12"/>
+      <c r="T49" s="13"/>
+      <c r="U49" s="11"/>
+      <c r="V49" s="12"/>
+      <c r="W49" s="12"/>
+      <c r="X49" s="13"/>
+      <c r="Y49" s="11"/>
+      <c r="Z49" s="12"/>
+      <c r="AA49" s="12"/>
+      <c r="AB49" s="13"/>
+      <c r="AC49" s="11"/>
+      <c r="AD49" s="12"/>
+      <c r="AE49" s="12"/>
+      <c r="AF49" s="13"/>
+      <c r="AG49" s="11"/>
+      <c r="AH49" s="12"/>
+      <c r="AI49" s="12"/>
+      <c r="AJ49" s="13"/>
+      <c r="AK49" s="11"/>
+      <c r="AL49" s="12"/>
+      <c r="AM49" s="12"/>
+      <c r="AN49" s="13"/>
+      <c r="AO49" s="11"/>
+      <c r="AP49" s="12"/>
+      <c r="AQ49" s="12"/>
+      <c r="AR49" s="13"/>
+      <c r="AS49" s="11"/>
+      <c r="AT49" s="12"/>
+      <c r="AU49" s="12"/>
+      <c r="AV49" s="13"/>
+      <c r="AW49" s="11"/>
+      <c r="AX49" s="12"/>
+      <c r="AY49" s="12"/>
+      <c r="AZ49" s="13"/>
+    </row>
+    <row r="50" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A50" s="53"/>
+      <c r="B50" s="48"/>
+      <c r="C50" s="51"/>
+      <c r="D50" s="51"/>
+      <c r="E50" s="42"/>
+      <c r="F50" s="43"/>
       <c r="G50" s="12"/>
       <c r="H50" s="13"/>
       <c r="I50" s="11"/>
@@ -4191,11 +4247,11 @@
       <c r="AY50" s="12"/>
       <c r="AZ50" s="13"/>
     </row>
-    <row r="51" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="62"/>
-      <c r="B51" s="77"/>
-      <c r="C51" s="54"/>
-      <c r="D51" s="54"/>
+    <row r="51" spans="1:52" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A51" s="53"/>
+      <c r="B51" s="49"/>
+      <c r="C51" s="51"/>
+      <c r="D51" s="51"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4245,14 +4301,16 @@
       <c r="AY51" s="12"/>
       <c r="AZ51" s="13"/>
     </row>
-    <row r="52" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="62"/>
-      <c r="B52" s="76" t="s">
-        <v>7</v>
-      </c>
-      <c r="C52" s="80"/>
-      <c r="D52" s="80">
-        <v>0</v>
+    <row r="52" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A52" s="53"/>
+      <c r="B52" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C52" s="51">
+        <v>2</v>
+      </c>
+      <c r="D52" s="51" t="s">
+        <v>46</v>
       </c>
       <c r="E52" s="11"/>
       <c r="F52" s="12"/>
@@ -4263,7 +4321,7 @@
       <c r="K52" s="12"/>
       <c r="L52" s="13"/>
       <c r="M52" s="11"/>
-      <c r="N52" s="12"/>
+      <c r="N52" s="101"/>
       <c r="O52" s="12"/>
       <c r="P52" s="13"/>
       <c r="Q52" s="11"/>
@@ -4303,210 +4361,1151 @@
       <c r="AY52" s="12"/>
       <c r="AZ52" s="13"/>
     </row>
-    <row r="53" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="63"/>
-      <c r="B53" s="86"/>
-      <c r="C53" s="54"/>
-      <c r="D53" s="54"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="18"/>
-      <c r="G53" s="18"/>
-      <c r="H53" s="19"/>
-      <c r="I53" s="17"/>
-      <c r="J53" s="18"/>
-      <c r="K53" s="18"/>
-      <c r="L53" s="19"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="18"/>
-      <c r="O53" s="18"/>
-      <c r="P53" s="19"/>
-      <c r="Q53" s="17"/>
-      <c r="R53" s="18"/>
-      <c r="S53" s="18"/>
-      <c r="T53" s="19"/>
-      <c r="U53" s="17"/>
-      <c r="V53" s="18"/>
-      <c r="W53" s="18"/>
-      <c r="X53" s="19"/>
-      <c r="Y53" s="17"/>
-      <c r="Z53" s="18"/>
-      <c r="AA53" s="18"/>
-      <c r="AB53" s="19"/>
-      <c r="AC53" s="17"/>
-      <c r="AD53" s="18"/>
-      <c r="AE53" s="18"/>
-      <c r="AF53" s="19"/>
-      <c r="AG53" s="17"/>
-      <c r="AH53" s="18"/>
-      <c r="AI53" s="18"/>
-      <c r="AJ53" s="19"/>
-      <c r="AK53" s="17"/>
-      <c r="AL53" s="18"/>
-      <c r="AM53" s="18"/>
-      <c r="AN53" s="19"/>
-      <c r="AO53" s="17"/>
-      <c r="AP53" s="18"/>
-      <c r="AQ53" s="18"/>
-      <c r="AR53" s="19"/>
-      <c r="AS53" s="17"/>
-      <c r="AT53" s="18"/>
-      <c r="AU53" s="18"/>
-      <c r="AV53" s="19"/>
-      <c r="AW53" s="17"/>
-      <c r="AX53" s="18"/>
-      <c r="AY53" s="18"/>
-      <c r="AZ53" s="19"/>
-    </row>
-    <row r="54" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="4" t="s">
+    <row r="53" spans="1:52" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A53" s="53"/>
+      <c r="B53" s="49"/>
+      <c r="C53" s="51"/>
+      <c r="D53" s="51"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="12"/>
+      <c r="G53" s="12"/>
+      <c r="H53" s="13"/>
+      <c r="I53" s="11"/>
+      <c r="J53" s="12"/>
+      <c r="K53" s="12"/>
+      <c r="L53" s="13"/>
+      <c r="M53" s="11"/>
+      <c r="N53" s="106"/>
+      <c r="O53" s="106"/>
+      <c r="P53" s="13"/>
+      <c r="Q53" s="11"/>
+      <c r="R53" s="12"/>
+      <c r="S53" s="12"/>
+      <c r="T53" s="13"/>
+      <c r="U53" s="11"/>
+      <c r="V53" s="12"/>
+      <c r="W53" s="12"/>
+      <c r="X53" s="13"/>
+      <c r="Y53" s="11"/>
+      <c r="Z53" s="12"/>
+      <c r="AA53" s="12"/>
+      <c r="AB53" s="13"/>
+      <c r="AC53" s="11"/>
+      <c r="AD53" s="12"/>
+      <c r="AE53" s="12"/>
+      <c r="AF53" s="13"/>
+      <c r="AG53" s="11"/>
+      <c r="AH53" s="12"/>
+      <c r="AI53" s="12"/>
+      <c r="AJ53" s="13"/>
+      <c r="AK53" s="11"/>
+      <c r="AL53" s="12"/>
+      <c r="AM53" s="12"/>
+      <c r="AN53" s="13"/>
+      <c r="AO53" s="11"/>
+      <c r="AP53" s="12"/>
+      <c r="AQ53" s="12"/>
+      <c r="AR53" s="13"/>
+      <c r="AS53" s="11"/>
+      <c r="AT53" s="12"/>
+      <c r="AU53" s="12"/>
+      <c r="AV53" s="13"/>
+      <c r="AW53" s="11"/>
+      <c r="AX53" s="12"/>
+      <c r="AY53" s="12"/>
+      <c r="AZ53" s="13"/>
+    </row>
+    <row r="54" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A54" s="53"/>
+      <c r="B54" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="C54" s="51"/>
+      <c r="D54" s="51"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="12"/>
+      <c r="H54" s="13"/>
+      <c r="I54" s="11"/>
+      <c r="J54" s="12"/>
+      <c r="K54" s="12"/>
+      <c r="L54" s="13"/>
+      <c r="M54" s="11"/>
+      <c r="N54" s="12"/>
+      <c r="O54" s="12"/>
+      <c r="P54" s="13"/>
+      <c r="Q54" s="11"/>
+      <c r="R54" s="12"/>
+      <c r="S54" s="12"/>
+      <c r="T54" s="13"/>
+      <c r="U54" s="11"/>
+      <c r="V54" s="12"/>
+      <c r="W54" s="12"/>
+      <c r="X54" s="13"/>
+      <c r="Y54" s="11"/>
+      <c r="Z54" s="12"/>
+      <c r="AA54" s="12"/>
+      <c r="AB54" s="13"/>
+      <c r="AC54" s="11"/>
+      <c r="AD54" s="12"/>
+      <c r="AE54" s="12"/>
+      <c r="AF54" s="13"/>
+      <c r="AG54" s="11"/>
+      <c r="AH54" s="12"/>
+      <c r="AI54" s="12"/>
+      <c r="AJ54" s="13"/>
+      <c r="AK54" s="11"/>
+      <c r="AL54" s="12"/>
+      <c r="AM54" s="12"/>
+      <c r="AN54" s="13"/>
+      <c r="AO54" s="11"/>
+      <c r="AP54" s="12"/>
+      <c r="AQ54" s="12"/>
+      <c r="AR54" s="13"/>
+      <c r="AS54" s="11"/>
+      <c r="AT54" s="12"/>
+      <c r="AU54" s="12"/>
+      <c r="AV54" s="13"/>
+      <c r="AW54" s="11"/>
+      <c r="AX54" s="12"/>
+      <c r="AY54" s="12"/>
+      <c r="AZ54" s="13"/>
+    </row>
+    <row r="55" spans="1:52" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A55" s="53"/>
+      <c r="B55" s="49"/>
+      <c r="C55" s="51"/>
+      <c r="D55" s="51"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="12"/>
+      <c r="G55" s="12"/>
+      <c r="H55" s="13"/>
+      <c r="I55" s="11"/>
+      <c r="J55" s="12"/>
+      <c r="K55" s="12"/>
+      <c r="L55" s="13"/>
+      <c r="M55" s="11"/>
+      <c r="N55" s="12"/>
+      <c r="O55" s="12"/>
+      <c r="P55" s="13"/>
+      <c r="Q55" s="11"/>
+      <c r="R55" s="12"/>
+      <c r="S55" s="12"/>
+      <c r="T55" s="13"/>
+      <c r="U55" s="11"/>
+      <c r="V55" s="12"/>
+      <c r="W55" s="12"/>
+      <c r="X55" s="13"/>
+      <c r="Y55" s="11"/>
+      <c r="Z55" s="12"/>
+      <c r="AA55" s="12"/>
+      <c r="AB55" s="13"/>
+      <c r="AC55" s="11"/>
+      <c r="AD55" s="12"/>
+      <c r="AE55" s="12"/>
+      <c r="AF55" s="13"/>
+      <c r="AG55" s="11"/>
+      <c r="AH55" s="12"/>
+      <c r="AI55" s="12"/>
+      <c r="AJ55" s="13"/>
+      <c r="AK55" s="11"/>
+      <c r="AL55" s="12"/>
+      <c r="AM55" s="12"/>
+      <c r="AN55" s="13"/>
+      <c r="AO55" s="11"/>
+      <c r="AP55" s="12"/>
+      <c r="AQ55" s="12"/>
+      <c r="AR55" s="13"/>
+      <c r="AS55" s="11"/>
+      <c r="AT55" s="12"/>
+      <c r="AU55" s="12"/>
+      <c r="AV55" s="13"/>
+      <c r="AW55" s="11"/>
+      <c r="AX55" s="12"/>
+      <c r="AY55" s="12"/>
+      <c r="AZ55" s="13"/>
+    </row>
+    <row r="56" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="53"/>
+      <c r="B56" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="C56" s="50"/>
+      <c r="D56" s="59"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="12"/>
+      <c r="G56" s="12"/>
+      <c r="H56" s="13"/>
+      <c r="I56" s="11"/>
+      <c r="J56" s="12"/>
+      <c r="K56" s="12"/>
+      <c r="L56" s="13"/>
+      <c r="M56" s="11"/>
+      <c r="N56" s="12"/>
+      <c r="O56" s="12"/>
+      <c r="P56" s="13"/>
+      <c r="Q56" s="11"/>
+      <c r="R56" s="12"/>
+      <c r="S56" s="12"/>
+      <c r="T56" s="13"/>
+      <c r="U56" s="11"/>
+      <c r="V56" s="12"/>
+      <c r="W56" s="12"/>
+      <c r="X56" s="13"/>
+      <c r="Y56" s="11"/>
+      <c r="Z56" s="12"/>
+      <c r="AA56" s="12"/>
+      <c r="AB56" s="13"/>
+      <c r="AC56" s="11"/>
+      <c r="AD56" s="12"/>
+      <c r="AE56" s="12"/>
+      <c r="AF56" s="13"/>
+      <c r="AG56" s="11"/>
+      <c r="AH56" s="12"/>
+      <c r="AI56" s="12"/>
+      <c r="AJ56" s="13"/>
+      <c r="AK56" s="11"/>
+      <c r="AL56" s="12"/>
+      <c r="AM56" s="12"/>
+      <c r="AN56" s="13"/>
+      <c r="AO56" s="11"/>
+      <c r="AP56" s="12"/>
+      <c r="AQ56" s="12"/>
+      <c r="AR56" s="13"/>
+      <c r="AS56" s="11"/>
+      <c r="AT56" s="12"/>
+      <c r="AU56" s="12"/>
+      <c r="AV56" s="13"/>
+      <c r="AW56" s="11"/>
+      <c r="AX56" s="12"/>
+      <c r="AY56" s="12"/>
+      <c r="AZ56" s="13"/>
+    </row>
+    <row r="57" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="53"/>
+      <c r="B57" s="49"/>
+      <c r="C57" s="51"/>
+      <c r="D57" s="59"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="13"/>
+      <c r="I57" s="11"/>
+      <c r="J57" s="12"/>
+      <c r="K57" s="12"/>
+      <c r="L57" s="13"/>
+      <c r="M57" s="11"/>
+      <c r="N57" s="12"/>
+      <c r="O57" s="12"/>
+      <c r="P57" s="13"/>
+      <c r="Q57" s="11"/>
+      <c r="R57" s="12"/>
+      <c r="S57" s="12"/>
+      <c r="T57" s="13"/>
+      <c r="U57" s="11"/>
+      <c r="V57" s="12"/>
+      <c r="W57" s="12"/>
+      <c r="X57" s="13"/>
+      <c r="Y57" s="11"/>
+      <c r="Z57" s="12"/>
+      <c r="AA57" s="12"/>
+      <c r="AB57" s="13"/>
+      <c r="AC57" s="11"/>
+      <c r="AD57" s="12"/>
+      <c r="AE57" s="12"/>
+      <c r="AF57" s="13"/>
+      <c r="AG57" s="11"/>
+      <c r="AH57" s="12"/>
+      <c r="AI57" s="12"/>
+      <c r="AJ57" s="13"/>
+      <c r="AK57" s="11"/>
+      <c r="AL57" s="12"/>
+      <c r="AM57" s="12"/>
+      <c r="AN57" s="13"/>
+      <c r="AO57" s="11"/>
+      <c r="AP57" s="12"/>
+      <c r="AQ57" s="12"/>
+      <c r="AR57" s="13"/>
+      <c r="AS57" s="11"/>
+      <c r="AT57" s="12"/>
+      <c r="AU57" s="12"/>
+      <c r="AV57" s="13"/>
+      <c r="AW57" s="11"/>
+      <c r="AX57" s="12"/>
+      <c r="AY57" s="12"/>
+      <c r="AZ57" s="13"/>
+    </row>
+    <row r="58" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A58" s="53"/>
+      <c r="B58" s="69" t="s">
+        <v>26</v>
+      </c>
+      <c r="C58" s="51"/>
+      <c r="D58" s="59"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="12"/>
+      <c r="H58" s="13"/>
+      <c r="I58" s="11"/>
+      <c r="J58" s="12"/>
+      <c r="K58" s="12"/>
+      <c r="L58" s="13"/>
+      <c r="M58" s="11"/>
+      <c r="N58" s="12"/>
+      <c r="O58" s="12"/>
+      <c r="P58" s="13"/>
+      <c r="Q58" s="11"/>
+      <c r="R58" s="12"/>
+      <c r="S58" s="12"/>
+      <c r="T58" s="13"/>
+      <c r="U58" s="11"/>
+      <c r="V58" s="12"/>
+      <c r="W58" s="12"/>
+      <c r="X58" s="13"/>
+      <c r="Y58" s="11"/>
+      <c r="Z58" s="12"/>
+      <c r="AA58" s="12"/>
+      <c r="AB58" s="13"/>
+      <c r="AC58" s="11"/>
+      <c r="AD58" s="12"/>
+      <c r="AE58" s="12"/>
+      <c r="AF58" s="13"/>
+      <c r="AG58" s="11"/>
+      <c r="AH58" s="12"/>
+      <c r="AI58" s="12"/>
+      <c r="AJ58" s="13"/>
+      <c r="AK58" s="11"/>
+      <c r="AL58" s="12"/>
+      <c r="AM58" s="12"/>
+      <c r="AN58" s="13"/>
+      <c r="AO58" s="11"/>
+      <c r="AP58" s="12"/>
+      <c r="AQ58" s="12"/>
+      <c r="AR58" s="13"/>
+      <c r="AS58" s="11"/>
+      <c r="AT58" s="12"/>
+      <c r="AU58" s="12"/>
+      <c r="AV58" s="13"/>
+      <c r="AW58" s="11"/>
+      <c r="AX58" s="12"/>
+      <c r="AY58" s="12"/>
+      <c r="AZ58" s="13"/>
+    </row>
+    <row r="59" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A59" s="53"/>
+      <c r="B59" s="69"/>
+      <c r="C59" s="51"/>
+      <c r="D59" s="59"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="12"/>
+      <c r="H59" s="13"/>
+      <c r="I59" s="11"/>
+      <c r="J59" s="12"/>
+      <c r="K59" s="12"/>
+      <c r="L59" s="13"/>
+      <c r="M59" s="11"/>
+      <c r="N59" s="12"/>
+      <c r="O59" s="12"/>
+      <c r="P59" s="13"/>
+      <c r="Q59" s="11"/>
+      <c r="R59" s="12"/>
+      <c r="S59" s="12"/>
+      <c r="T59" s="13"/>
+      <c r="U59" s="11"/>
+      <c r="V59" s="12"/>
+      <c r="W59" s="12"/>
+      <c r="X59" s="13"/>
+      <c r="Y59" s="11"/>
+      <c r="Z59" s="12"/>
+      <c r="AA59" s="12"/>
+      <c r="AB59" s="13"/>
+      <c r="AC59" s="11"/>
+      <c r="AD59" s="12"/>
+      <c r="AE59" s="12"/>
+      <c r="AF59" s="13"/>
+      <c r="AG59" s="11"/>
+      <c r="AH59" s="12"/>
+      <c r="AI59" s="12"/>
+      <c r="AJ59" s="13"/>
+      <c r="AK59" s="11"/>
+      <c r="AL59" s="12"/>
+      <c r="AM59" s="12"/>
+      <c r="AN59" s="13"/>
+      <c r="AO59" s="11"/>
+      <c r="AP59" s="12"/>
+      <c r="AQ59" s="12"/>
+      <c r="AR59" s="13"/>
+      <c r="AS59" s="11"/>
+      <c r="AT59" s="12"/>
+      <c r="AU59" s="12"/>
+      <c r="AV59" s="13"/>
+      <c r="AW59" s="11"/>
+      <c r="AX59" s="12"/>
+      <c r="AY59" s="12"/>
+      <c r="AZ59" s="13"/>
+    </row>
+    <row r="60" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A60" s="53"/>
+      <c r="B60" s="56" t="s">
+        <v>7</v>
+      </c>
+      <c r="C60" s="51"/>
+      <c r="D60" s="59">
+        <v>0</v>
+      </c>
+      <c r="E60" s="11"/>
+      <c r="F60" s="12"/>
+      <c r="G60" s="12"/>
+      <c r="H60" s="13"/>
+      <c r="I60" s="11"/>
+      <c r="J60" s="12"/>
+      <c r="K60" s="12"/>
+      <c r="L60" s="13"/>
+      <c r="M60" s="11"/>
+      <c r="N60" s="12"/>
+      <c r="O60" s="12"/>
+      <c r="P60" s="13"/>
+      <c r="Q60" s="11"/>
+      <c r="R60" s="12"/>
+      <c r="S60" s="12"/>
+      <c r="T60" s="13"/>
+      <c r="U60" s="11"/>
+      <c r="V60" s="12"/>
+      <c r="W60" s="12"/>
+      <c r="X60" s="13"/>
+      <c r="Y60" s="11"/>
+      <c r="Z60" s="12"/>
+      <c r="AA60" s="12"/>
+      <c r="AB60" s="13"/>
+      <c r="AC60" s="11"/>
+      <c r="AD60" s="12"/>
+      <c r="AE60" s="12"/>
+      <c r="AF60" s="13"/>
+      <c r="AG60" s="11"/>
+      <c r="AH60" s="12"/>
+      <c r="AI60" s="12"/>
+      <c r="AJ60" s="13"/>
+      <c r="AK60" s="11"/>
+      <c r="AL60" s="12"/>
+      <c r="AM60" s="12"/>
+      <c r="AN60" s="13"/>
+      <c r="AO60" s="11"/>
+      <c r="AP60" s="12"/>
+      <c r="AQ60" s="12"/>
+      <c r="AR60" s="13"/>
+      <c r="AS60" s="11"/>
+      <c r="AT60" s="12"/>
+      <c r="AU60" s="12"/>
+      <c r="AV60" s="13"/>
+      <c r="AW60" s="11"/>
+      <c r="AX60" s="12"/>
+      <c r="AY60" s="12"/>
+      <c r="AZ60" s="13"/>
+    </row>
+    <row r="61" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="53"/>
+      <c r="B61" s="56"/>
+      <c r="C61" s="51"/>
+      <c r="D61" s="59"/>
+      <c r="E61" s="11"/>
+      <c r="F61" s="12"/>
+      <c r="G61" s="12"/>
+      <c r="H61" s="13"/>
+      <c r="I61" s="11"/>
+      <c r="J61" s="12"/>
+      <c r="K61" s="12"/>
+      <c r="L61" s="13"/>
+      <c r="M61" s="11"/>
+      <c r="N61" s="12"/>
+      <c r="O61" s="12"/>
+      <c r="P61" s="13"/>
+      <c r="Q61" s="11"/>
+      <c r="R61" s="12"/>
+      <c r="S61" s="12"/>
+      <c r="T61" s="13"/>
+      <c r="U61" s="11"/>
+      <c r="V61" s="12"/>
+      <c r="W61" s="12"/>
+      <c r="X61" s="13"/>
+      <c r="Y61" s="11"/>
+      <c r="Z61" s="12"/>
+      <c r="AA61" s="12"/>
+      <c r="AB61" s="13"/>
+      <c r="AC61" s="11"/>
+      <c r="AD61" s="12"/>
+      <c r="AE61" s="12"/>
+      <c r="AF61" s="13"/>
+      <c r="AG61" s="11"/>
+      <c r="AH61" s="12"/>
+      <c r="AI61" s="12"/>
+      <c r="AJ61" s="13"/>
+      <c r="AK61" s="11"/>
+      <c r="AL61" s="12"/>
+      <c r="AM61" s="12"/>
+      <c r="AN61" s="13"/>
+      <c r="AO61" s="11"/>
+      <c r="AP61" s="12"/>
+      <c r="AQ61" s="12"/>
+      <c r="AR61" s="13"/>
+      <c r="AS61" s="11"/>
+      <c r="AT61" s="12"/>
+      <c r="AU61" s="12"/>
+      <c r="AV61" s="13"/>
+      <c r="AW61" s="11"/>
+      <c r="AX61" s="12"/>
+      <c r="AY61" s="12"/>
+      <c r="AZ61" s="13"/>
+    </row>
+    <row r="62" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A62" s="52" t="s">
+        <v>14</v>
+      </c>
+      <c r="B62" s="55" t="s">
+        <v>22</v>
+      </c>
+      <c r="C62" s="57"/>
+      <c r="D62" s="58"/>
+      <c r="E62" s="8"/>
+      <c r="F62" s="9"/>
+      <c r="G62" s="9"/>
+      <c r="H62" s="10"/>
+      <c r="I62" s="8"/>
+      <c r="J62" s="9"/>
+      <c r="K62" s="9"/>
+      <c r="L62" s="10"/>
+      <c r="M62" s="8"/>
+      <c r="N62" s="9"/>
+      <c r="O62" s="9"/>
+      <c r="P62" s="10"/>
+      <c r="Q62" s="8"/>
+      <c r="R62" s="9"/>
+      <c r="S62" s="9"/>
+      <c r="T62" s="10"/>
+      <c r="U62" s="8"/>
+      <c r="V62" s="9"/>
+      <c r="W62" s="9"/>
+      <c r="X62" s="10"/>
+      <c r="Y62" s="8"/>
+      <c r="Z62" s="9"/>
+      <c r="AA62" s="9"/>
+      <c r="AB62" s="10"/>
+      <c r="AC62" s="8"/>
+      <c r="AD62" s="9"/>
+      <c r="AE62" s="9"/>
+      <c r="AF62" s="10"/>
+      <c r="AG62" s="8"/>
+      <c r="AH62" s="9"/>
+      <c r="AI62" s="9"/>
+      <c r="AJ62" s="10"/>
+      <c r="AK62" s="8"/>
+      <c r="AL62" s="9"/>
+      <c r="AM62" s="9"/>
+      <c r="AN62" s="10"/>
+      <c r="AO62" s="8"/>
+      <c r="AP62" s="9"/>
+      <c r="AQ62" s="9"/>
+      <c r="AR62" s="10"/>
+      <c r="AS62" s="8"/>
+      <c r="AT62" s="9"/>
+      <c r="AU62" s="9"/>
+      <c r="AV62" s="10"/>
+      <c r="AW62" s="8"/>
+      <c r="AX62" s="9"/>
+      <c r="AY62" s="9"/>
+      <c r="AZ62" s="10"/>
+    </row>
+    <row r="63" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A63" s="53"/>
+      <c r="B63" s="56"/>
+      <c r="C63" s="51"/>
+      <c r="D63" s="59"/>
+      <c r="E63" s="11"/>
+      <c r="F63" s="12"/>
+      <c r="G63" s="12"/>
+      <c r="H63" s="13"/>
+      <c r="I63" s="11"/>
+      <c r="J63" s="12"/>
+      <c r="K63" s="12"/>
+      <c r="L63" s="13"/>
+      <c r="M63" s="11"/>
+      <c r="N63" s="12"/>
+      <c r="O63" s="12"/>
+      <c r="P63" s="13"/>
+      <c r="Q63" s="11"/>
+      <c r="R63" s="12"/>
+      <c r="S63" s="12"/>
+      <c r="T63" s="13"/>
+      <c r="U63" s="11"/>
+      <c r="V63" s="12"/>
+      <c r="W63" s="12"/>
+      <c r="X63" s="13"/>
+      <c r="Y63" s="11"/>
+      <c r="Z63" s="12"/>
+      <c r="AA63" s="12"/>
+      <c r="AB63" s="13"/>
+      <c r="AC63" s="11"/>
+      <c r="AD63" s="12"/>
+      <c r="AE63" s="12"/>
+      <c r="AF63" s="13"/>
+      <c r="AG63" s="11"/>
+      <c r="AH63" s="12"/>
+      <c r="AI63" s="12"/>
+      <c r="AJ63" s="13"/>
+      <c r="AK63" s="11"/>
+      <c r="AL63" s="12"/>
+      <c r="AM63" s="12"/>
+      <c r="AN63" s="13"/>
+      <c r="AO63" s="11"/>
+      <c r="AP63" s="12"/>
+      <c r="AQ63" s="12"/>
+      <c r="AR63" s="13"/>
+      <c r="AS63" s="11"/>
+      <c r="AT63" s="12"/>
+      <c r="AU63" s="12"/>
+      <c r="AV63" s="13"/>
+      <c r="AW63" s="11"/>
+      <c r="AX63" s="12"/>
+      <c r="AY63" s="12"/>
+      <c r="AZ63" s="13"/>
+    </row>
+    <row r="64" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="53"/>
+      <c r="B64" s="48" t="s">
+        <v>23</v>
+      </c>
+      <c r="C64" s="50"/>
+      <c r="D64" s="50"/>
+      <c r="E64" s="11"/>
+      <c r="F64" s="12"/>
+      <c r="G64" s="12"/>
+      <c r="H64" s="13"/>
+      <c r="I64" s="11"/>
+      <c r="J64" s="12"/>
+      <c r="K64" s="12"/>
+      <c r="L64" s="13"/>
+      <c r="M64" s="11"/>
+      <c r="N64" s="12"/>
+      <c r="O64" s="12"/>
+      <c r="P64" s="13"/>
+      <c r="Q64" s="11"/>
+      <c r="R64" s="12"/>
+      <c r="S64" s="12"/>
+      <c r="T64" s="13"/>
+      <c r="U64" s="11"/>
+      <c r="V64" s="12"/>
+      <c r="W64" s="12"/>
+      <c r="X64" s="13"/>
+      <c r="Y64" s="11"/>
+      <c r="Z64" s="12"/>
+      <c r="AA64" s="12"/>
+      <c r="AB64" s="13"/>
+      <c r="AC64" s="11"/>
+      <c r="AD64" s="12"/>
+      <c r="AE64" s="12"/>
+      <c r="AF64" s="13"/>
+      <c r="AG64" s="11"/>
+      <c r="AH64" s="12"/>
+      <c r="AI64" s="12"/>
+      <c r="AJ64" s="13"/>
+      <c r="AK64" s="11"/>
+      <c r="AL64" s="12"/>
+      <c r="AM64" s="12"/>
+      <c r="AN64" s="13"/>
+      <c r="AO64" s="11"/>
+      <c r="AP64" s="12"/>
+      <c r="AQ64" s="12"/>
+      <c r="AR64" s="13"/>
+      <c r="AS64" s="11"/>
+      <c r="AT64" s="12"/>
+      <c r="AU64" s="12"/>
+      <c r="AV64" s="13"/>
+      <c r="AW64" s="11"/>
+      <c r="AX64" s="12"/>
+      <c r="AY64" s="12"/>
+      <c r="AZ64" s="13"/>
+    </row>
+    <row r="65" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="53"/>
+      <c r="B65" s="49"/>
+      <c r="C65" s="51"/>
+      <c r="D65" s="51"/>
+      <c r="E65" s="11"/>
+      <c r="F65" s="12"/>
+      <c r="G65" s="12"/>
+      <c r="H65" s="13"/>
+      <c r="I65" s="11"/>
+      <c r="J65" s="12"/>
+      <c r="K65" s="12"/>
+      <c r="L65" s="13"/>
+      <c r="M65" s="11"/>
+      <c r="N65" s="12"/>
+      <c r="O65" s="12"/>
+      <c r="P65" s="13"/>
+      <c r="Q65" s="11"/>
+      <c r="R65" s="12"/>
+      <c r="S65" s="12"/>
+      <c r="T65" s="13"/>
+      <c r="U65" s="11"/>
+      <c r="V65" s="12"/>
+      <c r="W65" s="12"/>
+      <c r="X65" s="13"/>
+      <c r="Y65" s="11"/>
+      <c r="Z65" s="12"/>
+      <c r="AA65" s="12"/>
+      <c r="AB65" s="13"/>
+      <c r="AC65" s="11"/>
+      <c r="AD65" s="12"/>
+      <c r="AE65" s="12"/>
+      <c r="AF65" s="13"/>
+      <c r="AG65" s="11"/>
+      <c r="AH65" s="12"/>
+      <c r="AI65" s="12"/>
+      <c r="AJ65" s="13"/>
+      <c r="AK65" s="11"/>
+      <c r="AL65" s="12"/>
+      <c r="AM65" s="12"/>
+      <c r="AN65" s="13"/>
+      <c r="AO65" s="11"/>
+      <c r="AP65" s="12"/>
+      <c r="AQ65" s="12"/>
+      <c r="AR65" s="13"/>
+      <c r="AS65" s="11"/>
+      <c r="AT65" s="12"/>
+      <c r="AU65" s="12"/>
+      <c r="AV65" s="13"/>
+      <c r="AW65" s="11"/>
+      <c r="AX65" s="12"/>
+      <c r="AY65" s="12"/>
+      <c r="AZ65" s="13"/>
+    </row>
+    <row r="66" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A66" s="53"/>
+      <c r="B66" s="56" t="s">
+        <v>24</v>
+      </c>
+      <c r="C66" s="51"/>
+      <c r="D66" s="59"/>
+      <c r="E66" s="11"/>
+      <c r="F66" s="12"/>
+      <c r="G66" s="12"/>
+      <c r="H66" s="13"/>
+      <c r="I66" s="11"/>
+      <c r="J66" s="12"/>
+      <c r="K66" s="12"/>
+      <c r="L66" s="13"/>
+      <c r="M66" s="11"/>
+      <c r="N66" s="12"/>
+      <c r="O66" s="12"/>
+      <c r="P66" s="13"/>
+      <c r="Q66" s="11"/>
+      <c r="R66" s="12"/>
+      <c r="S66" s="12"/>
+      <c r="T66" s="13"/>
+      <c r="U66" s="11"/>
+      <c r="V66" s="12"/>
+      <c r="W66" s="12"/>
+      <c r="X66" s="13"/>
+      <c r="Y66" s="11"/>
+      <c r="Z66" s="12"/>
+      <c r="AA66" s="12"/>
+      <c r="AB66" s="13"/>
+      <c r="AC66" s="11"/>
+      <c r="AD66" s="12"/>
+      <c r="AE66" s="12"/>
+      <c r="AF66" s="13"/>
+      <c r="AG66" s="11"/>
+      <c r="AH66" s="12"/>
+      <c r="AI66" s="12"/>
+      <c r="AJ66" s="13"/>
+      <c r="AK66" s="11"/>
+      <c r="AL66" s="12"/>
+      <c r="AM66" s="12"/>
+      <c r="AN66" s="13"/>
+      <c r="AO66" s="11"/>
+      <c r="AP66" s="12"/>
+      <c r="AQ66" s="12"/>
+      <c r="AR66" s="13"/>
+      <c r="AS66" s="11"/>
+      <c r="AT66" s="12"/>
+      <c r="AU66" s="12"/>
+      <c r="AV66" s="13"/>
+      <c r="AW66" s="11"/>
+      <c r="AX66" s="12"/>
+      <c r="AY66" s="12"/>
+      <c r="AZ66" s="13"/>
+    </row>
+    <row r="67" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="54"/>
+      <c r="B67" s="60"/>
+      <c r="C67" s="61"/>
+      <c r="D67" s="62"/>
+      <c r="E67" s="17"/>
+      <c r="F67" s="18"/>
+      <c r="G67" s="18"/>
+      <c r="H67" s="19"/>
+      <c r="I67" s="17"/>
+      <c r="J67" s="18"/>
+      <c r="K67" s="18"/>
+      <c r="L67" s="19"/>
+      <c r="M67" s="17"/>
+      <c r="N67" s="18"/>
+      <c r="O67" s="18"/>
+      <c r="P67" s="19"/>
+      <c r="Q67" s="17"/>
+      <c r="R67" s="18"/>
+      <c r="S67" s="18"/>
+      <c r="T67" s="19"/>
+      <c r="U67" s="17"/>
+      <c r="V67" s="18"/>
+      <c r="W67" s="18"/>
+      <c r="X67" s="19"/>
+      <c r="Y67" s="17"/>
+      <c r="Z67" s="18"/>
+      <c r="AA67" s="18"/>
+      <c r="AB67" s="19"/>
+      <c r="AC67" s="17"/>
+      <c r="AD67" s="18"/>
+      <c r="AE67" s="18"/>
+      <c r="AF67" s="19"/>
+      <c r="AG67" s="17"/>
+      <c r="AH67" s="18"/>
+      <c r="AI67" s="18"/>
+      <c r="AJ67" s="19"/>
+      <c r="AK67" s="17"/>
+      <c r="AL67" s="18"/>
+      <c r="AM67" s="18"/>
+      <c r="AN67" s="19"/>
+      <c r="AO67" s="17"/>
+      <c r="AP67" s="18"/>
+      <c r="AQ67" s="18"/>
+      <c r="AR67" s="19"/>
+      <c r="AS67" s="17"/>
+      <c r="AT67" s="18"/>
+      <c r="AU67" s="18"/>
+      <c r="AV67" s="19"/>
+      <c r="AW67" s="17"/>
+      <c r="AX67" s="18"/>
+      <c r="AY67" s="18"/>
+      <c r="AZ67" s="19"/>
+    </row>
+    <row r="68" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="52" t="s">
+        <v>15</v>
+      </c>
+      <c r="B68" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="C68" s="50"/>
+      <c r="D68" s="50"/>
+      <c r="E68" s="11"/>
+      <c r="F68" s="12"/>
+      <c r="G68" s="12"/>
+      <c r="H68" s="13"/>
+      <c r="I68" s="11"/>
+      <c r="J68" s="12"/>
+      <c r="K68" s="12"/>
+      <c r="L68" s="13"/>
+      <c r="M68" s="11"/>
+      <c r="N68" s="12"/>
+      <c r="O68" s="12"/>
+      <c r="P68" s="13"/>
+      <c r="Q68" s="11"/>
+      <c r="R68" s="12"/>
+      <c r="S68" s="12"/>
+      <c r="T68" s="13"/>
+      <c r="U68" s="11"/>
+      <c r="V68" s="12"/>
+      <c r="W68" s="12"/>
+      <c r="X68" s="13"/>
+      <c r="Y68" s="11"/>
+      <c r="Z68" s="12"/>
+      <c r="AA68" s="12"/>
+      <c r="AB68" s="13"/>
+      <c r="AC68" s="11"/>
+      <c r="AD68" s="12"/>
+      <c r="AE68" s="12"/>
+      <c r="AF68" s="13"/>
+      <c r="AG68" s="11"/>
+      <c r="AH68" s="12"/>
+      <c r="AI68" s="12"/>
+      <c r="AJ68" s="13"/>
+      <c r="AK68" s="11"/>
+      <c r="AL68" s="12"/>
+      <c r="AM68" s="12"/>
+      <c r="AN68" s="13"/>
+      <c r="AO68" s="11"/>
+      <c r="AP68" s="12"/>
+      <c r="AQ68" s="12"/>
+      <c r="AR68" s="13"/>
+      <c r="AS68" s="11"/>
+      <c r="AT68" s="12"/>
+      <c r="AU68" s="12"/>
+      <c r="AV68" s="13"/>
+      <c r="AW68" s="11"/>
+      <c r="AX68" s="12"/>
+      <c r="AY68" s="12"/>
+      <c r="AZ68" s="13"/>
+    </row>
+    <row r="69" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="53"/>
+      <c r="B69" s="49"/>
+      <c r="C69" s="51"/>
+      <c r="D69" s="51"/>
+      <c r="E69" s="11"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="12"/>
+      <c r="H69" s="13"/>
+      <c r="I69" s="11"/>
+      <c r="J69" s="12"/>
+      <c r="K69" s="12"/>
+      <c r="L69" s="13"/>
+      <c r="M69" s="11"/>
+      <c r="N69" s="12"/>
+      <c r="O69" s="12"/>
+      <c r="P69" s="13"/>
+      <c r="Q69" s="11"/>
+      <c r="R69" s="12"/>
+      <c r="S69" s="12"/>
+      <c r="T69" s="13"/>
+      <c r="U69" s="11"/>
+      <c r="V69" s="12"/>
+      <c r="W69" s="12"/>
+      <c r="X69" s="13"/>
+      <c r="Y69" s="11"/>
+      <c r="Z69" s="12"/>
+      <c r="AA69" s="12"/>
+      <c r="AB69" s="13"/>
+      <c r="AC69" s="11"/>
+      <c r="AD69" s="12"/>
+      <c r="AE69" s="12"/>
+      <c r="AF69" s="13"/>
+      <c r="AG69" s="11"/>
+      <c r="AH69" s="12"/>
+      <c r="AI69" s="12"/>
+      <c r="AJ69" s="13"/>
+      <c r="AK69" s="11"/>
+      <c r="AL69" s="12"/>
+      <c r="AM69" s="12"/>
+      <c r="AN69" s="13"/>
+      <c r="AO69" s="11"/>
+      <c r="AP69" s="12"/>
+      <c r="AQ69" s="12"/>
+      <c r="AR69" s="13"/>
+      <c r="AS69" s="11"/>
+      <c r="AT69" s="12"/>
+      <c r="AU69" s="12"/>
+      <c r="AV69" s="13"/>
+      <c r="AW69" s="11"/>
+      <c r="AX69" s="12"/>
+      <c r="AY69" s="12"/>
+      <c r="AZ69" s="13"/>
+    </row>
+    <row r="70" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="53"/>
+      <c r="B70" s="48" t="s">
+        <v>7</v>
+      </c>
+      <c r="C70" s="50"/>
+      <c r="D70" s="50">
+        <v>0</v>
+      </c>
+      <c r="E70" s="11"/>
+      <c r="F70" s="12"/>
+      <c r="G70" s="12"/>
+      <c r="H70" s="13"/>
+      <c r="I70" s="11"/>
+      <c r="J70" s="12"/>
+      <c r="K70" s="12"/>
+      <c r="L70" s="13"/>
+      <c r="M70" s="11"/>
+      <c r="N70" s="12"/>
+      <c r="O70" s="12"/>
+      <c r="P70" s="13"/>
+      <c r="Q70" s="11"/>
+      <c r="R70" s="12"/>
+      <c r="S70" s="12"/>
+      <c r="T70" s="13"/>
+      <c r="U70" s="11"/>
+      <c r="V70" s="12"/>
+      <c r="W70" s="12"/>
+      <c r="X70" s="13"/>
+      <c r="Y70" s="11"/>
+      <c r="Z70" s="12"/>
+      <c r="AA70" s="12"/>
+      <c r="AB70" s="13"/>
+      <c r="AC70" s="11"/>
+      <c r="AD70" s="12"/>
+      <c r="AE70" s="12"/>
+      <c r="AF70" s="13"/>
+      <c r="AG70" s="11"/>
+      <c r="AH70" s="12"/>
+      <c r="AI70" s="12"/>
+      <c r="AJ70" s="13"/>
+      <c r="AK70" s="11"/>
+      <c r="AL70" s="12"/>
+      <c r="AM70" s="12"/>
+      <c r="AN70" s="13"/>
+      <c r="AO70" s="11"/>
+      <c r="AP70" s="12"/>
+      <c r="AQ70" s="12"/>
+      <c r="AR70" s="13"/>
+      <c r="AS70" s="11"/>
+      <c r="AT70" s="12"/>
+      <c r="AU70" s="12"/>
+      <c r="AV70" s="13"/>
+      <c r="AW70" s="11"/>
+      <c r="AX70" s="12"/>
+      <c r="AY70" s="12"/>
+      <c r="AZ70" s="13"/>
+    </row>
+    <row r="71" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="54"/>
+      <c r="B71" s="63"/>
+      <c r="C71" s="51"/>
+      <c r="D71" s="51"/>
+      <c r="E71" s="17"/>
+      <c r="F71" s="18"/>
+      <c r="G71" s="18"/>
+      <c r="H71" s="19"/>
+      <c r="I71" s="17"/>
+      <c r="J71" s="18"/>
+      <c r="K71" s="18"/>
+      <c r="L71" s="19"/>
+      <c r="M71" s="17"/>
+      <c r="N71" s="18"/>
+      <c r="O71" s="18"/>
+      <c r="P71" s="19"/>
+      <c r="Q71" s="17"/>
+      <c r="R71" s="18"/>
+      <c r="S71" s="18"/>
+      <c r="T71" s="19"/>
+      <c r="U71" s="17"/>
+      <c r="V71" s="18"/>
+      <c r="W71" s="18"/>
+      <c r="X71" s="19"/>
+      <c r="Y71" s="17"/>
+      <c r="Z71" s="18"/>
+      <c r="AA71" s="18"/>
+      <c r="AB71" s="19"/>
+      <c r="AC71" s="17"/>
+      <c r="AD71" s="18"/>
+      <c r="AE71" s="18"/>
+      <c r="AF71" s="19"/>
+      <c r="AG71" s="17"/>
+      <c r="AH71" s="18"/>
+      <c r="AI71" s="18"/>
+      <c r="AJ71" s="19"/>
+      <c r="AK71" s="17"/>
+      <c r="AL71" s="18"/>
+      <c r="AM71" s="18"/>
+      <c r="AN71" s="19"/>
+      <c r="AO71" s="17"/>
+      <c r="AP71" s="18"/>
+      <c r="AQ71" s="18"/>
+      <c r="AR71" s="19"/>
+      <c r="AS71" s="17"/>
+      <c r="AT71" s="18"/>
+      <c r="AU71" s="18"/>
+      <c r="AV71" s="19"/>
+      <c r="AW71" s="17"/>
+      <c r="AX71" s="18"/>
+      <c r="AY71" s="18"/>
+      <c r="AZ71" s="19"/>
+    </row>
+    <row r="72" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B72" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C54" s="5">
-        <f>SUM(C4:C53)</f>
-        <v>1.2000000000000002</v>
-      </c>
-      <c r="D54" s="5">
-        <f>SUM(D4:D53)</f>
-        <v>1.7000000000000002</v>
-      </c>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
-      <c r="J54" s="6"/>
-      <c r="K54" s="6"/>
-      <c r="L54" s="6"/>
-      <c r="M54" s="6"/>
-      <c r="N54" s="6"/>
-      <c r="O54" s="6"/>
-      <c r="P54" s="6"/>
-      <c r="Q54" s="6"/>
-      <c r="R54" s="6"/>
-      <c r="S54" s="6"/>
-      <c r="T54" s="6"/>
-      <c r="U54" s="6"/>
-      <c r="V54" s="6"/>
-      <c r="W54" s="6"/>
-      <c r="X54" s="6"/>
-      <c r="Y54" s="6"/>
-      <c r="Z54" s="6"/>
-      <c r="AA54" s="6"/>
-      <c r="AB54" s="6"/>
-      <c r="AC54" s="6"/>
-      <c r="AD54" s="6"/>
-      <c r="AE54" s="6"/>
-      <c r="AF54" s="6"/>
-      <c r="AG54" s="6"/>
-      <c r="AH54" s="6"/>
-      <c r="AI54" s="6"/>
-      <c r="AJ54" s="6"/>
-      <c r="AK54" s="6"/>
-      <c r="AL54" s="6"/>
-      <c r="AM54" s="6"/>
-      <c r="AN54" s="6"/>
-      <c r="AO54" s="6"/>
-      <c r="AP54" s="6"/>
-      <c r="AQ54" s="6"/>
-      <c r="AR54" s="6"/>
-      <c r="AS54" s="6"/>
-      <c r="AT54" s="6"/>
-      <c r="AU54" s="6"/>
-      <c r="AV54" s="6"/>
-      <c r="AW54" s="6"/>
-      <c r="AX54" s="6"/>
-      <c r="AY54" s="7"/>
-      <c r="AZ54" s="7"/>
-    </row>
-    <row r="55" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+      <c r="C72" s="5">
+        <f>SUM(C4:C71)</f>
+        <v>27.7</v>
+      </c>
+      <c r="D72" s="5">
+        <f>SUM(D4:D71)</f>
+        <v>18.7</v>
+      </c>
+      <c r="E72" s="6"/>
+      <c r="F72" s="6"/>
+      <c r="G72" s="6"/>
+      <c r="H72" s="6"/>
+      <c r="I72" s="6"/>
+      <c r="J72" s="6"/>
+      <c r="K72" s="6"/>
+      <c r="L72" s="6"/>
+      <c r="M72" s="6"/>
+      <c r="N72" s="6"/>
+      <c r="O72" s="6"/>
+      <c r="P72" s="6"/>
+      <c r="Q72" s="6"/>
+      <c r="R72" s="6"/>
+      <c r="S72" s="6"/>
+      <c r="T72" s="6"/>
+      <c r="U72" s="6"/>
+      <c r="V72" s="6"/>
+      <c r="W72" s="6"/>
+      <c r="X72" s="6"/>
+      <c r="Y72" s="6"/>
+      <c r="Z72" s="6"/>
+      <c r="AA72" s="6"/>
+      <c r="AB72" s="6"/>
+      <c r="AC72" s="6"/>
+      <c r="AD72" s="6"/>
+      <c r="AE72" s="6"/>
+      <c r="AF72" s="6"/>
+      <c r="AG72" s="6"/>
+      <c r="AH72" s="6"/>
+      <c r="AI72" s="6"/>
+      <c r="AJ72" s="6"/>
+      <c r="AK72" s="6"/>
+      <c r="AL72" s="6"/>
+      <c r="AM72" s="6"/>
+      <c r="AN72" s="6"/>
+      <c r="AO72" s="6"/>
+      <c r="AP72" s="6"/>
+      <c r="AQ72" s="6"/>
+      <c r="AR72" s="6"/>
+      <c r="AS72" s="6"/>
+      <c r="AT72" s="6"/>
+      <c r="AU72" s="6"/>
+      <c r="AV72" s="6"/>
+      <c r="AW72" s="6"/>
+      <c r="AX72" s="6"/>
+      <c r="AY72" s="7"/>
+      <c r="AZ72" s="7"/>
+    </row>
+    <row r="73" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="108">
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B44:B45"/>
+  <mergeCells count="135">
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
     <mergeCell ref="C44:C45"/>
     <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B44:B45"/>
     <mergeCell ref="B48:B49"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="B50:B51"/>
     <mergeCell ref="B52:B53"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="B32:B33"/>
     <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
     <mergeCell ref="C34:C35"/>
     <mergeCell ref="D34:D35"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AW1:AZ1"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A43"/>
-    <mergeCell ref="A44:A49"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
     <mergeCell ref="B40:B41"/>
     <mergeCell ref="C40:C41"/>
     <mergeCell ref="D40:D41"/>
-    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C52:C53"/>
     <mergeCell ref="U1:X1"/>
-    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="D46:D47"/>
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
@@ -4529,6 +5528,90 @@
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="U2:X2"/>
     <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A61"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="D70:D71"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
CSS verbessert, valid bearb, formular bearbeitung
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5EA8FE-3CF0-4EEC-A5E8-294CF2E89915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF0E3EB-F880-4624-95AF-1A90555C9DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
   <si>
     <t>IPERKA Phase</t>
   </si>
@@ -174,12 +174,21 @@
   <si>
     <t>0.166667</t>
   </si>
+  <si>
+    <t>Code refactoring</t>
+  </si>
+  <si>
+    <t>CSS verbessern</t>
+  </si>
+  <si>
+    <t>Projektstruktur verbessern</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -245,6 +254,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -778,7 +794,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -841,17 +857,65 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -862,86 +926,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -964,36 +950,68 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -1328,7 +1346,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="75" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="82" t="s">
@@ -1338,151 +1356,151 @@
         <v>2</v>
       </c>
       <c r="D1" s="86"/>
-      <c r="E1" s="75" t="s">
+      <c r="E1" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="75" t="s">
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="75" t="s">
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="76"/>
-      <c r="O1" s="76"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="75" t="s">
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="76"/>
-      <c r="S1" s="76"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="75" t="s">
+      <c r="R1" s="68"/>
+      <c r="S1" s="68"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="76"/>
-      <c r="W1" s="76"/>
-      <c r="X1" s="77"/>
-      <c r="Y1" s="75" t="s">
+      <c r="V1" s="68"/>
+      <c r="W1" s="68"/>
+      <c r="X1" s="69"/>
+      <c r="Y1" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="76"/>
-      <c r="AA1" s="76"/>
-      <c r="AB1" s="77"/>
-      <c r="AC1" s="75" t="s">
+      <c r="Z1" s="68"/>
+      <c r="AA1" s="68"/>
+      <c r="AB1" s="69"/>
+      <c r="AC1" s="67" t="s">
         <v>29</v>
       </c>
-      <c r="AD1" s="76"/>
-      <c r="AE1" s="76"/>
-      <c r="AF1" s="77"/>
-      <c r="AG1" s="75" t="s">
+      <c r="AD1" s="68"/>
+      <c r="AE1" s="68"/>
+      <c r="AF1" s="69"/>
+      <c r="AG1" s="67" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="76"/>
-      <c r="AI1" s="76"/>
-      <c r="AJ1" s="77"/>
-      <c r="AK1" s="75" t="s">
+      <c r="AH1" s="68"/>
+      <c r="AI1" s="68"/>
+      <c r="AJ1" s="69"/>
+      <c r="AK1" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="AL1" s="76"/>
-      <c r="AM1" s="76"/>
-      <c r="AN1" s="77"/>
-      <c r="AO1" s="75" t="s">
+      <c r="AL1" s="68"/>
+      <c r="AM1" s="68"/>
+      <c r="AN1" s="69"/>
+      <c r="AO1" s="67" t="s">
         <v>27</v>
       </c>
-      <c r="AP1" s="76"/>
-      <c r="AQ1" s="76"/>
-      <c r="AR1" s="77"/>
-      <c r="AS1" s="75"/>
-      <c r="AT1" s="76"/>
-      <c r="AU1" s="76"/>
-      <c r="AV1" s="77"/>
-      <c r="AW1" s="75"/>
-      <c r="AX1" s="76"/>
-      <c r="AY1" s="76"/>
-      <c r="AZ1" s="77"/>
+      <c r="AP1" s="68"/>
+      <c r="AQ1" s="68"/>
+      <c r="AR1" s="69"/>
+      <c r="AS1" s="67"/>
+      <c r="AT1" s="68"/>
+      <c r="AU1" s="68"/>
+      <c r="AV1" s="69"/>
+      <c r="AW1" s="67"/>
+      <c r="AX1" s="68"/>
+      <c r="AY1" s="68"/>
+      <c r="AZ1" s="69"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="92"/>
+      <c r="A2" s="76"/>
       <c r="B2" s="83"/>
       <c r="C2" s="87"/>
       <c r="D2" s="88"/>
-      <c r="E2" s="79">
+      <c r="E2" s="72">
         <v>44781</v>
       </c>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="81"/>
-      <c r="I2" s="79">
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="72">
         <v>44782</v>
       </c>
-      <c r="J2" s="80"/>
-      <c r="K2" s="80"/>
-      <c r="L2" s="81"/>
-      <c r="M2" s="79">
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="74"/>
+      <c r="M2" s="72">
         <v>44783</v>
       </c>
-      <c r="N2" s="80"/>
-      <c r="O2" s="80"/>
-      <c r="P2" s="81"/>
-      <c r="Q2" s="79">
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
+      <c r="P2" s="74"/>
+      <c r="Q2" s="72">
         <v>44784</v>
       </c>
-      <c r="R2" s="80"/>
-      <c r="S2" s="80"/>
-      <c r="T2" s="81"/>
-      <c r="U2" s="79">
+      <c r="R2" s="73"/>
+      <c r="S2" s="73"/>
+      <c r="T2" s="74"/>
+      <c r="U2" s="72">
         <v>44785</v>
       </c>
-      <c r="V2" s="80"/>
-      <c r="W2" s="80"/>
-      <c r="X2" s="81"/>
-      <c r="Y2" s="79">
+      <c r="V2" s="73"/>
+      <c r="W2" s="73"/>
+      <c r="X2" s="74"/>
+      <c r="Y2" s="72">
         <v>44789</v>
       </c>
-      <c r="Z2" s="80"/>
-      <c r="AA2" s="80"/>
-      <c r="AB2" s="81"/>
-      <c r="AC2" s="79">
+      <c r="Z2" s="73"/>
+      <c r="AA2" s="73"/>
+      <c r="AB2" s="74"/>
+      <c r="AC2" s="72">
         <v>44790</v>
       </c>
-      <c r="AD2" s="80"/>
-      <c r="AE2" s="80"/>
-      <c r="AF2" s="81"/>
-      <c r="AG2" s="79">
+      <c r="AD2" s="73"/>
+      <c r="AE2" s="73"/>
+      <c r="AF2" s="74"/>
+      <c r="AG2" s="72">
         <v>44791</v>
       </c>
-      <c r="AH2" s="80"/>
-      <c r="AI2" s="80"/>
-      <c r="AJ2" s="81"/>
-      <c r="AK2" s="79">
+      <c r="AH2" s="73"/>
+      <c r="AI2" s="73"/>
+      <c r="AJ2" s="74"/>
+      <c r="AK2" s="72">
         <v>44792</v>
       </c>
-      <c r="AL2" s="80"/>
-      <c r="AM2" s="80"/>
-      <c r="AN2" s="81"/>
-      <c r="AO2" s="79">
+      <c r="AL2" s="73"/>
+      <c r="AM2" s="73"/>
+      <c r="AN2" s="74"/>
+      <c r="AO2" s="72">
         <v>44795</v>
       </c>
-      <c r="AP2" s="80"/>
-      <c r="AQ2" s="80"/>
-      <c r="AR2" s="81"/>
-      <c r="AS2" s="79"/>
-      <c r="AT2" s="80"/>
-      <c r="AU2" s="80"/>
-      <c r="AV2" s="81"/>
-      <c r="AW2" s="79"/>
-      <c r="AX2" s="80"/>
-      <c r="AY2" s="80"/>
-      <c r="AZ2" s="81"/>
+      <c r="AP2" s="73"/>
+      <c r="AQ2" s="73"/>
+      <c r="AR2" s="74"/>
+      <c r="AS2" s="72"/>
+      <c r="AT2" s="73"/>
+      <c r="AU2" s="73"/>
+      <c r="AV2" s="74"/>
+      <c r="AW2" s="72"/>
+      <c r="AX2" s="73"/>
+      <c r="AY2" s="73"/>
+      <c r="AZ2" s="74"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="93"/>
+      <c r="A3" s="77"/>
       <c r="B3" s="84"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
@@ -1621,11 +1639,11 @@
     </row>
     <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="49" t="s">
+      <c r="B4" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="67"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="103"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1681,9 +1699,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="64"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="68"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="81"/>
+      <c r="D5" s="102"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1739,9 +1757,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="69"/>
-      <c r="C6" s="51"/>
-      <c r="D6" s="59"/>
+      <c r="B6" s="94"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="64"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1786,9 +1804,9 @@
     </row>
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="48"/>
-      <c r="C7" s="66"/>
-      <c r="D7" s="68"/>
+      <c r="B7" s="65"/>
+      <c r="C7" s="81"/>
+      <c r="D7" s="102"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1843,16 +1861,16 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="78" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="55" t="s">
+      <c r="B8" s="96" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="57">
+      <c r="C8" s="98">
         <v>0.1</v>
       </c>
-      <c r="D8" s="73">
+      <c r="D8" s="107">
         <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
@@ -1909,10 +1927,10 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="53"/>
-      <c r="B9" s="56"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="74"/>
+      <c r="A9" s="79"/>
+      <c r="B9" s="70"/>
+      <c r="C9" s="63"/>
+      <c r="D9" s="108"/>
       <c r="E9" s="42"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -1963,14 +1981,14 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="53"/>
-      <c r="B10" s="56" t="s">
+      <c r="A10" s="79"/>
+      <c r="B10" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="65">
+      <c r="C10" s="71">
         <v>1</v>
       </c>
-      <c r="D10" s="65">
+      <c r="D10" s="71">
         <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
@@ -2023,10 +2041,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="53"/>
-      <c r="B11" s="56"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
+      <c r="A11" s="79"/>
+      <c r="B11" s="70"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="63"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2077,12 +2095,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="56" t="s">
+      <c r="A12" s="79"/>
+      <c r="B12" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="65"/>
-      <c r="D12" s="65"/>
+      <c r="C12" s="71"/>
+      <c r="D12" s="71"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2133,10 +2151,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="53"/>
-      <c r="B13" s="56"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
+      <c r="A13" s="79"/>
+      <c r="B13" s="70"/>
+      <c r="C13" s="63"/>
+      <c r="D13" s="63"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2187,14 +2205,14 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="53"/>
-      <c r="B14" s="56" t="s">
+      <c r="A14" s="79"/>
+      <c r="B14" s="70" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="65" t="s">
+      <c r="C14" s="71" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="65" t="s">
+      <c r="D14" s="71" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="42"/>
@@ -2247,10 +2265,10 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="53"/>
-      <c r="B15" s="56"/>
-      <c r="C15" s="51"/>
-      <c r="D15" s="51"/>
+      <c r="A15" s="79"/>
+      <c r="B15" s="70"/>
+      <c r="C15" s="63"/>
+      <c r="D15" s="63"/>
       <c r="E15" s="42"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -2301,14 +2319,14 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="53"/>
-      <c r="B16" s="64" t="s">
+      <c r="A16" s="79"/>
+      <c r="B16" s="89" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="51" t="s">
+      <c r="C16" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="59" t="s">
+      <c r="D16" s="64" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="20"/>
@@ -2361,10 +2379,10 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="54"/>
-      <c r="B17" s="89"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="62"/>
+      <c r="A17" s="80"/>
+      <c r="B17" s="90"/>
+      <c r="C17" s="91"/>
+      <c r="D17" s="92"/>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
@@ -2415,14 +2433,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52" t="s">
+      <c r="A18" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="78" t="s">
+      <c r="B18" s="100" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="57"/>
-      <c r="D18" s="58"/>
+      <c r="C18" s="98"/>
+      <c r="D18" s="99"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2473,10 +2491,10 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="53"/>
-      <c r="B19" s="63"/>
-      <c r="C19" s="51"/>
-      <c r="D19" s="59"/>
+      <c r="A19" s="79"/>
+      <c r="B19" s="101"/>
+      <c r="C19" s="63"/>
+      <c r="D19" s="64"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2527,12 +2545,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="53"/>
-      <c r="B20" s="56" t="s">
+      <c r="A20" s="79"/>
+      <c r="B20" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="51"/>
-      <c r="D20" s="59"/>
+      <c r="C20" s="63"/>
+      <c r="D20" s="64"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2572,10 +2590,10 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="53"/>
-      <c r="B21" s="56"/>
-      <c r="C21" s="51"/>
-      <c r="D21" s="59"/>
+      <c r="A21" s="79"/>
+      <c r="B21" s="70"/>
+      <c r="C21" s="63"/>
+      <c r="D21" s="64"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2626,14 +2644,14 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="53"/>
-      <c r="B22" s="56" t="s">
+      <c r="A22" s="79"/>
+      <c r="B22" s="70" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="51">
+      <c r="C22" s="63">
         <v>0.1</v>
       </c>
-      <c r="D22" s="59">
+      <c r="D22" s="64">
         <v>0.1</v>
       </c>
       <c r="E22" s="11"/>
@@ -2686,10 +2704,10 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="53"/>
-      <c r="B23" s="56"/>
-      <c r="C23" s="51"/>
-      <c r="D23" s="59"/>
+      <c r="A23" s="79"/>
+      <c r="B23" s="70"/>
+      <c r="C23" s="63"/>
+      <c r="D23" s="64"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2740,10 +2758,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="53"/>
-      <c r="B24" s="64"/>
-      <c r="C24" s="66"/>
-      <c r="D24" s="70"/>
+      <c r="A24" s="79"/>
+      <c r="B24" s="89"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="104"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2794,10 +2812,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="49"/>
-      <c r="C25" s="65"/>
-      <c r="D25" s="71"/>
+      <c r="A25" s="79"/>
+      <c r="B25" s="66"/>
+      <c r="C25" s="71"/>
+      <c r="D25" s="105"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2848,12 +2866,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="53"/>
-      <c r="B26" s="56" t="s">
+      <c r="A26" s="79"/>
+      <c r="B26" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="66"/>
-      <c r="D26" s="70">
+      <c r="C26" s="81"/>
+      <c r="D26" s="104">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2906,10 +2924,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="54"/>
-      <c r="B27" s="56"/>
-      <c r="C27" s="90"/>
-      <c r="D27" s="72"/>
+      <c r="A27" s="80"/>
+      <c r="B27" s="70"/>
+      <c r="C27" s="93"/>
+      <c r="D27" s="106"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2960,14 +2978,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="52" t="s">
+      <c r="A28" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="55" t="s">
+      <c r="B28" s="96" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="57"/>
-      <c r="D28" s="58"/>
+      <c r="C28" s="98"/>
+      <c r="D28" s="99"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -3018,10 +3036,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="53"/>
-      <c r="B29" s="60"/>
-      <c r="C29" s="61"/>
-      <c r="D29" s="62"/>
+      <c r="A29" s="79"/>
+      <c r="B29" s="97"/>
+      <c r="C29" s="91"/>
+      <c r="D29" s="92"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3072,22 +3090,22 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="52" t="s">
+      <c r="A30" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="55" t="s">
+      <c r="B30" s="96" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="57">
+      <c r="C30" s="98">
         <v>2</v>
       </c>
-      <c r="D30" s="58">
+      <c r="D30" s="99">
         <v>2</v>
       </c>
-      <c r="E30" s="99"/>
-      <c r="F30" s="100"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="54"/>
       <c r="G30" s="47"/>
-      <c r="H30" s="94"/>
+      <c r="H30" s="48"/>
       <c r="I30" s="8"/>
       <c r="J30" s="9"/>
       <c r="K30" s="9"/>
@@ -3134,14 +3152,14 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="53"/>
-      <c r="B31" s="56"/>
-      <c r="C31" s="51"/>
-      <c r="D31" s="59"/>
-      <c r="E31" s="105"/>
-      <c r="F31" s="106"/>
+      <c r="A31" s="79"/>
+      <c r="B31" s="70"/>
+      <c r="C31" s="63"/>
+      <c r="D31" s="64"/>
+      <c r="E31" s="59"/>
+      <c r="F31" s="60"/>
       <c r="G31" s="43"/>
-      <c r="H31" s="95"/>
+      <c r="H31" s="49"/>
       <c r="I31" s="11"/>
       <c r="J31" s="12"/>
       <c r="K31" s="12"/>
@@ -3188,21 +3206,21 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="53"/>
-      <c r="B32" s="48" t="s">
+      <c r="A32" s="79"/>
+      <c r="B32" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="51">
+      <c r="C32" s="63">
         <v>4</v>
       </c>
-      <c r="D32" s="51">
+      <c r="D32" s="63">
         <v>7</v>
       </c>
       <c r="E32" s="11"/>
       <c r="F32" s="12"/>
-      <c r="G32" s="101"/>
-      <c r="H32" s="102"/>
-      <c r="I32" s="103"/>
+      <c r="G32" s="55"/>
+      <c r="H32" s="56"/>
+      <c r="I32" s="57"/>
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
       <c r="L32" s="13"/>
@@ -3248,16 +3266,16 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="53"/>
-      <c r="B33" s="49"/>
-      <c r="C33" s="51"/>
-      <c r="D33" s="51"/>
+      <c r="A33" s="79"/>
+      <c r="B33" s="66"/>
+      <c r="C33" s="63"/>
+      <c r="D33" s="63"/>
       <c r="E33" s="11"/>
-      <c r="F33" s="106"/>
-      <c r="G33" s="106"/>
-      <c r="H33" s="107"/>
-      <c r="I33" s="105"/>
-      <c r="J33" s="106"/>
+      <c r="F33" s="60"/>
+      <c r="G33" s="60"/>
+      <c r="H33" s="61"/>
+      <c r="I33" s="59"/>
+      <c r="J33" s="60"/>
       <c r="K33" s="12"/>
       <c r="L33" s="13"/>
       <c r="M33" s="11"/>
@@ -3302,21 +3320,21 @@
       <c r="AZ33" s="13"/>
     </row>
     <row r="34" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="53"/>
-      <c r="B34" s="48" t="s">
+      <c r="A34" s="79"/>
+      <c r="B34" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="51" t="s">
+      <c r="C34" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="51" t="s">
+      <c r="D34" s="63" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="11"/>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
       <c r="H34" s="13"/>
-      <c r="I34" s="103"/>
+      <c r="I34" s="57"/>
       <c r="J34" s="43"/>
       <c r="K34" s="12"/>
       <c r="L34" s="13"/>
@@ -3362,15 +3380,15 @@
       <c r="AZ34" s="13"/>
     </row>
     <row r="35" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="53"/>
-      <c r="B35" s="49"/>
-      <c r="C35" s="51"/>
-      <c r="D35" s="51"/>
+      <c r="A35" s="79"/>
+      <c r="B35" s="66"/>
+      <c r="C35" s="63"/>
+      <c r="D35" s="63"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
       <c r="H35" s="13"/>
-      <c r="I35" s="108"/>
+      <c r="I35" s="62"/>
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
       <c r="L35" s="13"/>
@@ -3416,22 +3434,22 @@
       <c r="AZ35" s="13"/>
     </row>
     <row r="36" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="53"/>
-      <c r="B36" s="48" t="s">
+      <c r="A36" s="79"/>
+      <c r="B36" s="65" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="51">
+      <c r="C36" s="63">
         <v>1.5</v>
       </c>
-      <c r="D36" s="51">
+      <c r="D36" s="63">
         <v>2</v>
       </c>
       <c r="E36" s="11"/>
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
       <c r="H36" s="13"/>
-      <c r="I36" s="104"/>
-      <c r="J36" s="101"/>
+      <c r="I36" s="58"/>
+      <c r="J36" s="55"/>
       <c r="K36" s="12"/>
       <c r="L36" s="13"/>
       <c r="M36" s="11"/>
@@ -3476,17 +3494,17 @@
       <c r="AZ36" s="13"/>
     </row>
     <row r="37" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="53"/>
-      <c r="B37" s="49"/>
-      <c r="C37" s="51"/>
-      <c r="D37" s="51"/>
+      <c r="A37" s="79"/>
+      <c r="B37" s="66"/>
+      <c r="C37" s="63"/>
+      <c r="D37" s="63"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
       <c r="H37" s="13"/>
-      <c r="I37" s="96"/>
-      <c r="J37" s="106"/>
-      <c r="K37" s="97"/>
+      <c r="I37" s="50"/>
+      <c r="J37" s="60"/>
+      <c r="K37" s="51"/>
       <c r="L37" s="13"/>
       <c r="M37" s="11"/>
       <c r="N37" s="12"/>
@@ -3530,15 +3548,15 @@
       <c r="AZ37" s="13"/>
     </row>
     <row r="38" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="48" t="s">
+      <c r="A38" s="79"/>
+      <c r="B38" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="51">
+      <c r="C38" s="63">
         <v>7</v>
       </c>
-      <c r="D38" s="59">
-        <v>4</v>
+      <c r="D38" s="64">
+        <v>6</v>
       </c>
       <c r="E38" s="11"/>
       <c r="F38" s="12"/>
@@ -3546,10 +3564,10 @@
       <c r="H38" s="13"/>
       <c r="I38" s="11"/>
       <c r="J38" s="12"/>
-      <c r="K38" s="101"/>
-      <c r="L38" s="102"/>
-      <c r="M38" s="103"/>
-      <c r="N38" s="101"/>
+      <c r="K38" s="55"/>
+      <c r="L38" s="56"/>
+      <c r="M38" s="57"/>
+      <c r="N38" s="55"/>
       <c r="O38" s="12"/>
       <c r="P38" s="13"/>
       <c r="Q38" s="11"/>
@@ -3590,25 +3608,25 @@
       <c r="AZ38" s="13"/>
     </row>
     <row r="39" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="53"/>
-      <c r="B39" s="49"/>
-      <c r="C39" s="51"/>
-      <c r="D39" s="59"/>
+      <c r="A39" s="79"/>
+      <c r="B39" s="66"/>
+      <c r="C39" s="63"/>
+      <c r="D39" s="64"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
       <c r="H39" s="13"/>
       <c r="I39" s="11"/>
-      <c r="J39" s="106"/>
+      <c r="J39" s="60"/>
       <c r="K39" s="43"/>
       <c r="L39" s="13"/>
       <c r="M39" s="11"/>
       <c r="N39" s="12"/>
       <c r="O39" s="12"/>
       <c r="P39" s="13"/>
-      <c r="Q39" s="105"/>
-      <c r="R39" s="106"/>
-      <c r="S39" s="12"/>
+      <c r="Q39" s="59"/>
+      <c r="R39" s="60"/>
+      <c r="S39" s="51"/>
       <c r="T39" s="13"/>
       <c r="U39" s="11"/>
       <c r="V39" s="12"/>
@@ -3644,30 +3662,30 @@
       <c r="AZ39" s="13"/>
     </row>
     <row r="40" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="53"/>
-      <c r="B40" s="48" t="s">
+      <c r="A40" s="79"/>
+      <c r="B40" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="51">
+      <c r="C40" s="63">
         <v>6</v>
       </c>
-      <c r="D40" s="59"/>
+      <c r="D40" s="64"/>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
       <c r="H40" s="13"/>
       <c r="I40" s="11"/>
       <c r="J40" s="12"/>
-      <c r="K40" s="101"/>
-      <c r="L40" s="102"/>
-      <c r="M40" s="103"/>
-      <c r="N40" s="12"/>
+      <c r="K40" s="55"/>
+      <c r="L40" s="56"/>
+      <c r="M40" s="57"/>
+      <c r="N40" s="55"/>
       <c r="O40" s="12"/>
       <c r="P40" s="13"/>
       <c r="Q40" s="11"/>
       <c r="R40" s="12"/>
-      <c r="S40" s="12"/>
-      <c r="T40" s="13"/>
+      <c r="S40" s="109"/>
+      <c r="T40" s="110"/>
       <c r="U40" s="11"/>
       <c r="V40" s="12"/>
       <c r="W40" s="12"/>
@@ -3702,26 +3720,26 @@
       <c r="AZ40" s="13"/>
     </row>
     <row r="41" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="53"/>
-      <c r="B41" s="49"/>
-      <c r="C41" s="51"/>
-      <c r="D41" s="59"/>
+      <c r="A41" s="79"/>
+      <c r="B41" s="66"/>
+      <c r="C41" s="63"/>
+      <c r="D41" s="64"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
       <c r="H41" s="13"/>
       <c r="I41" s="11"/>
       <c r="J41" s="12"/>
-      <c r="K41" s="106"/>
-      <c r="L41" s="107"/>
-      <c r="M41" s="105"/>
+      <c r="K41" s="60"/>
+      <c r="L41" s="61"/>
+      <c r="M41" s="59"/>
       <c r="N41" s="43"/>
-      <c r="O41" s="97"/>
-      <c r="P41" s="107"/>
+      <c r="O41" s="51"/>
+      <c r="P41" s="61"/>
       <c r="Q41" s="42"/>
       <c r="R41" s="43"/>
-      <c r="S41" s="106"/>
-      <c r="T41" s="107"/>
+      <c r="S41" s="43"/>
+      <c r="T41" s="49"/>
       <c r="U41" s="11"/>
       <c r="V41" s="12"/>
       <c r="W41" s="12"/>
@@ -3756,14 +3774,14 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="53"/>
-      <c r="B42" s="48" t="s">
+      <c r="A42" s="79"/>
+      <c r="B42" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="51">
+      <c r="C42" s="63">
         <v>4</v>
       </c>
-      <c r="D42" s="59">
+      <c r="D42" s="64">
         <v>2</v>
       </c>
       <c r="E42" s="11"/>
@@ -3771,13 +3789,13 @@
       <c r="G42" s="12"/>
       <c r="H42" s="13"/>
       <c r="I42" s="11"/>
-      <c r="J42" s="101"/>
-      <c r="K42" s="101"/>
-      <c r="L42" s="95"/>
+      <c r="J42" s="55"/>
+      <c r="K42" s="55"/>
+      <c r="L42" s="49"/>
       <c r="M42" s="42"/>
       <c r="N42" s="43"/>
       <c r="O42" s="43"/>
-      <c r="P42" s="95"/>
+      <c r="P42" s="49"/>
       <c r="Q42" s="11"/>
       <c r="R42" s="12"/>
       <c r="S42" s="12"/>
@@ -3816,26 +3834,26 @@
       <c r="AZ42" s="13"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A43" s="53"/>
-      <c r="B43" s="49"/>
-      <c r="C43" s="51"/>
-      <c r="D43" s="59"/>
+      <c r="A43" s="79"/>
+      <c r="B43" s="66"/>
+      <c r="C43" s="63"/>
+      <c r="D43" s="64"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
       <c r="H43" s="13"/>
       <c r="I43" s="11"/>
-      <c r="J43" s="106"/>
-      <c r="K43" s="106"/>
-      <c r="L43" s="98"/>
+      <c r="J43" s="60"/>
+      <c r="K43" s="60"/>
+      <c r="L43" s="52"/>
       <c r="M43" s="42"/>
       <c r="N43" s="43"/>
       <c r="O43" s="43"/>
-      <c r="P43" s="95"/>
+      <c r="P43" s="49"/>
       <c r="Q43" s="42"/>
       <c r="R43" s="43"/>
       <c r="S43" s="43"/>
-      <c r="T43" s="95"/>
+      <c r="T43" s="49"/>
       <c r="U43" s="11"/>
       <c r="V43" s="12"/>
       <c r="W43" s="12"/>
@@ -3870,10 +3888,12 @@
       <c r="AZ43" s="13"/>
     </row>
     <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="53"/>
-      <c r="B44" s="48"/>
-      <c r="C44" s="51"/>
-      <c r="D44" s="59"/>
+      <c r="A44" s="79"/>
+      <c r="B44" s="65" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="63"/>
+      <c r="D44" s="64"/>
       <c r="E44" s="11"/>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
@@ -3881,11 +3901,11 @@
       <c r="I44" s="11"/>
       <c r="J44" s="12"/>
       <c r="K44" s="43"/>
-      <c r="L44" s="95"/>
+      <c r="L44" s="49"/>
       <c r="M44" s="42"/>
       <c r="N44" s="43"/>
       <c r="O44" s="43"/>
-      <c r="P44" s="95"/>
+      <c r="P44" s="49"/>
       <c r="Q44" s="11"/>
       <c r="R44" s="12"/>
       <c r="S44" s="12"/>
@@ -3924,10 +3944,10 @@
       <c r="AZ44" s="13"/>
     </row>
     <row r="45" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="53"/>
-      <c r="B45" s="49"/>
-      <c r="C45" s="51"/>
-      <c r="D45" s="59"/>
+      <c r="A45" s="79"/>
+      <c r="B45" s="66"/>
+      <c r="C45" s="63"/>
+      <c r="D45" s="64"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
@@ -3935,15 +3955,15 @@
       <c r="I45" s="11"/>
       <c r="J45" s="12"/>
       <c r="K45" s="43"/>
-      <c r="L45" s="95"/>
+      <c r="L45" s="49"/>
       <c r="M45" s="42"/>
       <c r="N45" s="43"/>
       <c r="O45" s="43"/>
-      <c r="P45" s="95"/>
+      <c r="P45" s="49"/>
       <c r="Q45" s="11"/>
       <c r="R45" s="12"/>
       <c r="S45" s="12"/>
-      <c r="T45" s="13"/>
+      <c r="T45" s="61"/>
       <c r="U45" s="11"/>
       <c r="V45" s="12"/>
       <c r="W45" s="12"/>
@@ -3978,10 +3998,12 @@
       <c r="AZ45" s="13"/>
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A46" s="53"/>
-      <c r="B46" s="48"/>
-      <c r="C46" s="50"/>
-      <c r="D46" s="59"/>
+      <c r="A46" s="79"/>
+      <c r="B46" s="65" t="s">
+        <v>48</v>
+      </c>
+      <c r="C46" s="95"/>
+      <c r="D46" s="64"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -3989,11 +4011,11 @@
       <c r="I46" s="11"/>
       <c r="J46" s="12"/>
       <c r="K46" s="43"/>
-      <c r="L46" s="95"/>
+      <c r="L46" s="49"/>
       <c r="M46" s="42"/>
       <c r="N46" s="43"/>
       <c r="O46" s="43"/>
-      <c r="P46" s="95"/>
+      <c r="P46" s="49"/>
       <c r="Q46" s="11"/>
       <c r="R46" s="12"/>
       <c r="S46" s="12"/>
@@ -4032,10 +4054,10 @@
       <c r="AZ46" s="13"/>
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A47" s="53"/>
-      <c r="B47" s="49"/>
-      <c r="C47" s="50"/>
-      <c r="D47" s="59"/>
+      <c r="A47" s="79"/>
+      <c r="B47" s="66"/>
+      <c r="C47" s="95"/>
+      <c r="D47" s="64"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -4086,10 +4108,12 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="53"/>
-      <c r="B48" s="48"/>
-      <c r="C48" s="51"/>
-      <c r="D48" s="51"/>
+      <c r="A48" s="79"/>
+      <c r="B48" s="65" t="s">
+        <v>49</v>
+      </c>
+      <c r="C48" s="63"/>
+      <c r="D48" s="63"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4139,11 +4163,11 @@
       <c r="AY48" s="12"/>
       <c r="AZ48" s="13"/>
     </row>
-    <row r="49" spans="1:52" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="53"/>
-      <c r="B49" s="49"/>
-      <c r="C49" s="51"/>
-      <c r="D49" s="51"/>
+    <row r="49" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A49" s="79"/>
+      <c r="B49" s="66"/>
+      <c r="C49" s="63"/>
+      <c r="D49" s="63"/>
       <c r="E49" s="11"/>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
@@ -4194,10 +4218,10 @@
       <c r="AZ49" s="13"/>
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A50" s="53"/>
-      <c r="B50" s="48"/>
-      <c r="C50" s="51"/>
-      <c r="D50" s="51"/>
+      <c r="A50" s="79"/>
+      <c r="B50" s="65"/>
+      <c r="C50" s="63"/>
+      <c r="D50" s="63"/>
       <c r="E50" s="42"/>
       <c r="F50" s="43"/>
       <c r="G50" s="12"/>
@@ -4247,11 +4271,11 @@
       <c r="AY50" s="12"/>
       <c r="AZ50" s="13"/>
     </row>
-    <row r="51" spans="1:52" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="53"/>
-      <c r="B51" s="49"/>
-      <c r="C51" s="51"/>
-      <c r="D51" s="51"/>
+    <row r="51" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A51" s="79"/>
+      <c r="B51" s="66"/>
+      <c r="C51" s="63"/>
+      <c r="D51" s="63"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4302,14 +4326,14 @@
       <c r="AZ51" s="13"/>
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A52" s="53"/>
-      <c r="B52" s="48" t="s">
+      <c r="A52" s="79"/>
+      <c r="B52" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="51">
+      <c r="C52" s="63">
         <v>2</v>
       </c>
-      <c r="D52" s="51" t="s">
+      <c r="D52" s="63" t="s">
         <v>46</v>
       </c>
       <c r="E52" s="11"/>
@@ -4321,7 +4345,7 @@
       <c r="K52" s="12"/>
       <c r="L52" s="13"/>
       <c r="M52" s="11"/>
-      <c r="N52" s="101"/>
+      <c r="N52" s="55"/>
       <c r="O52" s="12"/>
       <c r="P52" s="13"/>
       <c r="Q52" s="11"/>
@@ -4361,11 +4385,11 @@
       <c r="AY52" s="12"/>
       <c r="AZ52" s="13"/>
     </row>
-    <row r="53" spans="1:52" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="53"/>
-      <c r="B53" s="49"/>
-      <c r="C53" s="51"/>
-      <c r="D53" s="51"/>
+    <row r="53" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A53" s="79"/>
+      <c r="B53" s="66"/>
+      <c r="C53" s="63"/>
+      <c r="D53" s="63"/>
       <c r="E53" s="11"/>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
@@ -4375,8 +4399,8 @@
       <c r="K53" s="12"/>
       <c r="L53" s="13"/>
       <c r="M53" s="11"/>
-      <c r="N53" s="106"/>
-      <c r="O53" s="106"/>
+      <c r="N53" s="60"/>
+      <c r="O53" s="60"/>
       <c r="P53" s="13"/>
       <c r="Q53" s="11"/>
       <c r="R53" s="12"/>
@@ -4416,12 +4440,12 @@
       <c r="AZ53" s="13"/>
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A54" s="53"/>
-      <c r="B54" s="48" t="s">
+      <c r="A54" s="79"/>
+      <c r="B54" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="C54" s="51"/>
-      <c r="D54" s="51"/>
+      <c r="C54" s="63"/>
+      <c r="D54" s="63"/>
       <c r="E54" s="11"/>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
@@ -4471,11 +4495,11 @@
       <c r="AY54" s="12"/>
       <c r="AZ54" s="13"/>
     </row>
-    <row r="55" spans="1:52" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A55" s="53"/>
-      <c r="B55" s="49"/>
-      <c r="C55" s="51"/>
-      <c r="D55" s="51"/>
+    <row r="55" spans="1:52" x14ac:dyDescent="0.25">
+      <c r="A55" s="79"/>
+      <c r="B55" s="66"/>
+      <c r="C55" s="63"/>
+      <c r="D55" s="63"/>
       <c r="E55" s="11"/>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
@@ -4526,12 +4550,12 @@
       <c r="AZ55" s="13"/>
     </row>
     <row r="56" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="53"/>
-      <c r="B56" s="48" t="s">
+      <c r="A56" s="79"/>
+      <c r="B56" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="C56" s="50"/>
-      <c r="D56" s="59"/>
+      <c r="C56" s="95"/>
+      <c r="D56" s="64"/>
       <c r="E56" s="11"/>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
@@ -4582,10 +4606,10 @@
       <c r="AZ56" s="13"/>
     </row>
     <row r="57" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="53"/>
-      <c r="B57" s="49"/>
-      <c r="C57" s="51"/>
-      <c r="D57" s="59"/>
+      <c r="A57" s="79"/>
+      <c r="B57" s="66"/>
+      <c r="C57" s="63"/>
+      <c r="D57" s="64"/>
       <c r="E57" s="11"/>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
@@ -4636,12 +4660,12 @@
       <c r="AZ57" s="13"/>
     </row>
     <row r="58" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A58" s="53"/>
-      <c r="B58" s="69" t="s">
+      <c r="A58" s="79"/>
+      <c r="B58" s="94" t="s">
         <v>26</v>
       </c>
-      <c r="C58" s="51"/>
-      <c r="D58" s="59"/>
+      <c r="C58" s="63"/>
+      <c r="D58" s="64"/>
       <c r="E58" s="11"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
@@ -4692,10 +4716,10 @@
       <c r="AZ58" s="13"/>
     </row>
     <row r="59" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A59" s="53"/>
-      <c r="B59" s="69"/>
-      <c r="C59" s="51"/>
-      <c r="D59" s="59"/>
+      <c r="A59" s="79"/>
+      <c r="B59" s="94"/>
+      <c r="C59" s="63"/>
+      <c r="D59" s="64"/>
       <c r="E59" s="11"/>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
@@ -4746,12 +4770,12 @@
       <c r="AZ59" s="13"/>
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A60" s="53"/>
-      <c r="B60" s="56" t="s">
+      <c r="A60" s="79"/>
+      <c r="B60" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="C60" s="51"/>
-      <c r="D60" s="59">
+      <c r="C60" s="63"/>
+      <c r="D60" s="64">
         <v>0</v>
       </c>
       <c r="E60" s="11"/>
@@ -4804,10 +4828,10 @@
       <c r="AZ60" s="13"/>
     </row>
     <row r="61" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="53"/>
-      <c r="B61" s="56"/>
-      <c r="C61" s="51"/>
-      <c r="D61" s="59"/>
+      <c r="A61" s="79"/>
+      <c r="B61" s="70"/>
+      <c r="C61" s="63"/>
+      <c r="D61" s="64"/>
       <c r="E61" s="11"/>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
@@ -4858,14 +4882,14 @@
       <c r="AZ61" s="13"/>
     </row>
     <row r="62" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A62" s="52" t="s">
+      <c r="A62" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="B62" s="55" t="s">
+      <c r="B62" s="96" t="s">
         <v>22</v>
       </c>
-      <c r="C62" s="57"/>
-      <c r="D62" s="58"/>
+      <c r="C62" s="98"/>
+      <c r="D62" s="99"/>
       <c r="E62" s="8"/>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -4916,10 +4940,10 @@
       <c r="AZ62" s="10"/>
     </row>
     <row r="63" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A63" s="53"/>
-      <c r="B63" s="56"/>
-      <c r="C63" s="51"/>
-      <c r="D63" s="59"/>
+      <c r="A63" s="79"/>
+      <c r="B63" s="70"/>
+      <c r="C63" s="63"/>
+      <c r="D63" s="64"/>
       <c r="E63" s="11"/>
       <c r="F63" s="12"/>
       <c r="G63" s="12"/>
@@ -4970,12 +4994,12 @@
       <c r="AZ63" s="13"/>
     </row>
     <row r="64" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="53"/>
-      <c r="B64" s="48" t="s">
+      <c r="A64" s="79"/>
+      <c r="B64" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="C64" s="50"/>
-      <c r="D64" s="50"/>
+      <c r="C64" s="95"/>
+      <c r="D64" s="95"/>
       <c r="E64" s="11"/>
       <c r="F64" s="12"/>
       <c r="G64" s="12"/>
@@ -5026,10 +5050,10 @@
       <c r="AZ64" s="13"/>
     </row>
     <row r="65" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="53"/>
-      <c r="B65" s="49"/>
-      <c r="C65" s="51"/>
-      <c r="D65" s="51"/>
+      <c r="A65" s="79"/>
+      <c r="B65" s="66"/>
+      <c r="C65" s="63"/>
+      <c r="D65" s="63"/>
       <c r="E65" s="11"/>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
@@ -5080,12 +5104,12 @@
       <c r="AZ65" s="13"/>
     </row>
     <row r="66" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A66" s="53"/>
-      <c r="B66" s="56" t="s">
+      <c r="A66" s="79"/>
+      <c r="B66" s="70" t="s">
         <v>24</v>
       </c>
-      <c r="C66" s="51"/>
-      <c r="D66" s="59"/>
+      <c r="C66" s="63"/>
+      <c r="D66" s="64"/>
       <c r="E66" s="11"/>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
@@ -5136,10 +5160,10 @@
       <c r="AZ66" s="13"/>
     </row>
     <row r="67" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="54"/>
-      <c r="B67" s="60"/>
-      <c r="C67" s="61"/>
-      <c r="D67" s="62"/>
+      <c r="A67" s="80"/>
+      <c r="B67" s="97"/>
+      <c r="C67" s="91"/>
+      <c r="D67" s="92"/>
       <c r="E67" s="17"/>
       <c r="F67" s="18"/>
       <c r="G67" s="18"/>
@@ -5190,14 +5214,14 @@
       <c r="AZ67" s="19"/>
     </row>
     <row r="68" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="52" t="s">
+      <c r="A68" s="78" t="s">
         <v>15</v>
       </c>
-      <c r="B68" s="48" t="s">
+      <c r="B68" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="C68" s="50"/>
-      <c r="D68" s="50"/>
+      <c r="C68" s="95"/>
+      <c r="D68" s="95"/>
       <c r="E68" s="11"/>
       <c r="F68" s="12"/>
       <c r="G68" s="12"/>
@@ -5248,10 +5272,10 @@
       <c r="AZ68" s="13"/>
     </row>
     <row r="69" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="53"/>
-      <c r="B69" s="49"/>
-      <c r="C69" s="51"/>
-      <c r="D69" s="51"/>
+      <c r="A69" s="79"/>
+      <c r="B69" s="66"/>
+      <c r="C69" s="63"/>
+      <c r="D69" s="63"/>
       <c r="E69" s="11"/>
       <c r="F69" s="12"/>
       <c r="G69" s="12"/>
@@ -5302,12 +5326,12 @@
       <c r="AZ69" s="13"/>
     </row>
     <row r="70" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="53"/>
-      <c r="B70" s="48" t="s">
+      <c r="A70" s="79"/>
+      <c r="B70" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="C70" s="50"/>
-      <c r="D70" s="50">
+      <c r="C70" s="95"/>
+      <c r="D70" s="95">
         <v>0</v>
       </c>
       <c r="E70" s="11"/>
@@ -5360,10 +5384,10 @@
       <c r="AZ70" s="13"/>
     </row>
     <row r="71" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="54"/>
-      <c r="B71" s="63"/>
-      <c r="C71" s="51"/>
-      <c r="D71" s="51"/>
+      <c r="A71" s="80"/>
+      <c r="B71" s="101"/>
+      <c r="C71" s="63"/>
+      <c r="D71" s="63"/>
       <c r="E71" s="17"/>
       <c r="F71" s="18"/>
       <c r="G71" s="18"/>
@@ -5423,7 +5447,7 @@
       </c>
       <c r="D72" s="5">
         <f>SUM(D4:D71)</f>
-        <v>18.7</v>
+        <v>20.7</v>
       </c>
       <c r="E72" s="6"/>
       <c r="F72" s="6"/>
@@ -5477,33 +5501,89 @@
     <row r="73" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="135">
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A61"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="C60:C61"/>
     <mergeCell ref="U1:X1"/>
     <mergeCell ref="D46:D47"/>
     <mergeCell ref="B10:B11"/>
@@ -5528,90 +5608,34 @@
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="U2:X2"/>
     <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A61"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C52:C53"/>
     <mergeCell ref="C46:C47"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AW1:AZ1"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="D70:D71"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Client side valid edit image + server side valid
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AF0E3EB-F880-4624-95AF-1A90555C9DF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49BB631-5C66-4D7E-9424-3754CAA9278D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -872,17 +872,88 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -893,11 +964,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -907,27 +975,6 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -950,68 +997,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -1346,162 +1346,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="108" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="82" t="s">
+      <c r="B1" s="99" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="85" t="s">
+      <c r="C1" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="86"/>
-      <c r="E1" s="67" t="s">
+      <c r="D1" s="103"/>
+      <c r="E1" s="92" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="67" t="s">
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="67" t="s">
+      <c r="J1" s="93"/>
+      <c r="K1" s="93"/>
+      <c r="L1" s="94"/>
+      <c r="M1" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="67" t="s">
+      <c r="N1" s="93"/>
+      <c r="O1" s="93"/>
+      <c r="P1" s="94"/>
+      <c r="Q1" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="69"/>
-      <c r="U1" s="67" t="s">
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="94"/>
+      <c r="U1" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="68"/>
-      <c r="W1" s="68"/>
-      <c r="X1" s="69"/>
-      <c r="Y1" s="67" t="s">
+      <c r="V1" s="93"/>
+      <c r="W1" s="93"/>
+      <c r="X1" s="94"/>
+      <c r="Y1" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="68"/>
-      <c r="AA1" s="68"/>
-      <c r="AB1" s="69"/>
-      <c r="AC1" s="67" t="s">
+      <c r="Z1" s="93"/>
+      <c r="AA1" s="93"/>
+      <c r="AB1" s="94"/>
+      <c r="AC1" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="AD1" s="68"/>
-      <c r="AE1" s="68"/>
-      <c r="AF1" s="69"/>
-      <c r="AG1" s="67" t="s">
+      <c r="AD1" s="93"/>
+      <c r="AE1" s="93"/>
+      <c r="AF1" s="94"/>
+      <c r="AG1" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="68"/>
-      <c r="AI1" s="68"/>
-      <c r="AJ1" s="69"/>
-      <c r="AK1" s="67" t="s">
+      <c r="AH1" s="93"/>
+      <c r="AI1" s="93"/>
+      <c r="AJ1" s="94"/>
+      <c r="AK1" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="AL1" s="68"/>
-      <c r="AM1" s="68"/>
-      <c r="AN1" s="69"/>
-      <c r="AO1" s="67" t="s">
+      <c r="AL1" s="93"/>
+      <c r="AM1" s="93"/>
+      <c r="AN1" s="94"/>
+      <c r="AO1" s="92" t="s">
         <v>27</v>
       </c>
-      <c r="AP1" s="68"/>
-      <c r="AQ1" s="68"/>
-      <c r="AR1" s="69"/>
-      <c r="AS1" s="67"/>
-      <c r="AT1" s="68"/>
-      <c r="AU1" s="68"/>
-      <c r="AV1" s="69"/>
-      <c r="AW1" s="67"/>
-      <c r="AX1" s="68"/>
-      <c r="AY1" s="68"/>
-      <c r="AZ1" s="69"/>
+      <c r="AP1" s="93"/>
+      <c r="AQ1" s="93"/>
+      <c r="AR1" s="94"/>
+      <c r="AS1" s="92"/>
+      <c r="AT1" s="93"/>
+      <c r="AU1" s="93"/>
+      <c r="AV1" s="94"/>
+      <c r="AW1" s="92"/>
+      <c r="AX1" s="93"/>
+      <c r="AY1" s="93"/>
+      <c r="AZ1" s="94"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="76"/>
-      <c r="B2" s="83"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="72">
+      <c r="A2" s="109"/>
+      <c r="B2" s="100"/>
+      <c r="C2" s="104"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="96">
         <v>44781</v>
       </c>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
-      <c r="H2" s="74"/>
-      <c r="I2" s="72">
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="96">
         <v>44782</v>
       </c>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="74"/>
-      <c r="M2" s="72">
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="96">
         <v>44783</v>
       </c>
-      <c r="N2" s="73"/>
-      <c r="O2" s="73"/>
-      <c r="P2" s="74"/>
-      <c r="Q2" s="72">
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
+      <c r="P2" s="98"/>
+      <c r="Q2" s="96">
         <v>44784</v>
       </c>
-      <c r="R2" s="73"/>
-      <c r="S2" s="73"/>
-      <c r="T2" s="74"/>
-      <c r="U2" s="72">
+      <c r="R2" s="97"/>
+      <c r="S2" s="97"/>
+      <c r="T2" s="98"/>
+      <c r="U2" s="96">
         <v>44785</v>
       </c>
-      <c r="V2" s="73"/>
-      <c r="W2" s="73"/>
-      <c r="X2" s="74"/>
-      <c r="Y2" s="72">
+      <c r="V2" s="97"/>
+      <c r="W2" s="97"/>
+      <c r="X2" s="98"/>
+      <c r="Y2" s="96">
         <v>44789</v>
       </c>
-      <c r="Z2" s="73"/>
-      <c r="AA2" s="73"/>
-      <c r="AB2" s="74"/>
-      <c r="AC2" s="72">
+      <c r="Z2" s="97"/>
+      <c r="AA2" s="97"/>
+      <c r="AB2" s="98"/>
+      <c r="AC2" s="96">
         <v>44790</v>
       </c>
-      <c r="AD2" s="73"/>
-      <c r="AE2" s="73"/>
-      <c r="AF2" s="74"/>
-      <c r="AG2" s="72">
+      <c r="AD2" s="97"/>
+      <c r="AE2" s="97"/>
+      <c r="AF2" s="98"/>
+      <c r="AG2" s="96">
         <v>44791</v>
       </c>
-      <c r="AH2" s="73"/>
-      <c r="AI2" s="73"/>
-      <c r="AJ2" s="74"/>
-      <c r="AK2" s="72">
+      <c r="AH2" s="97"/>
+      <c r="AI2" s="97"/>
+      <c r="AJ2" s="98"/>
+      <c r="AK2" s="96">
         <v>44792</v>
       </c>
-      <c r="AL2" s="73"/>
-      <c r="AM2" s="73"/>
-      <c r="AN2" s="74"/>
-      <c r="AO2" s="72">
+      <c r="AL2" s="97"/>
+      <c r="AM2" s="97"/>
+      <c r="AN2" s="98"/>
+      <c r="AO2" s="96">
         <v>44795</v>
       </c>
-      <c r="AP2" s="73"/>
-      <c r="AQ2" s="73"/>
-      <c r="AR2" s="74"/>
-      <c r="AS2" s="72"/>
-      <c r="AT2" s="73"/>
-      <c r="AU2" s="73"/>
-      <c r="AV2" s="74"/>
-      <c r="AW2" s="72"/>
-      <c r="AX2" s="73"/>
-      <c r="AY2" s="73"/>
-      <c r="AZ2" s="74"/>
+      <c r="AP2" s="97"/>
+      <c r="AQ2" s="97"/>
+      <c r="AR2" s="98"/>
+      <c r="AS2" s="96"/>
+      <c r="AT2" s="97"/>
+      <c r="AU2" s="97"/>
+      <c r="AV2" s="98"/>
+      <c r="AW2" s="96"/>
+      <c r="AX2" s="97"/>
+      <c r="AY2" s="97"/>
+      <c r="AZ2" s="98"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="77"/>
-      <c r="B3" s="84"/>
+      <c r="A3" s="110"/>
+      <c r="B3" s="101"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
@@ -1642,8 +1642,8 @@
       <c r="B4" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="71"/>
-      <c r="D4" s="103"/>
+      <c r="C4" s="82"/>
+      <c r="D4" s="84"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1699,9 +1699,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="89"/>
-      <c r="C5" s="81"/>
-      <c r="D5" s="102"/>
+      <c r="B5" s="81"/>
+      <c r="C5" s="83"/>
+      <c r="D5" s="85"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1757,9 +1757,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="94"/>
-      <c r="C6" s="63"/>
-      <c r="D6" s="64"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="76"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1805,8 +1805,8 @@
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
       <c r="B7" s="65"/>
-      <c r="C7" s="81"/>
-      <c r="D7" s="102"/>
+      <c r="C7" s="83"/>
+      <c r="D7" s="85"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1861,16 +1861,16 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="78" t="s">
+      <c r="A8" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="96" t="s">
+      <c r="B8" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="98">
+      <c r="C8" s="74">
         <v>0.1</v>
       </c>
-      <c r="D8" s="107">
+      <c r="D8" s="90">
         <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
@@ -1927,10 +1927,10 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="79"/>
-      <c r="B9" s="70"/>
-      <c r="C9" s="63"/>
-      <c r="D9" s="108"/>
+      <c r="A9" s="70"/>
+      <c r="B9" s="73"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="91"/>
       <c r="E9" s="42"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -1981,14 +1981,14 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="79"/>
-      <c r="B10" s="70" t="s">
+      <c r="A10" s="70"/>
+      <c r="B10" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="71">
+      <c r="C10" s="82">
         <v>1</v>
       </c>
-      <c r="D10" s="71">
+      <c r="D10" s="82">
         <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
@@ -2041,10 +2041,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="79"/>
-      <c r="B11" s="70"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="63"/>
+      <c r="A11" s="70"/>
+      <c r="B11" s="73"/>
+      <c r="C11" s="68"/>
+      <c r="D11" s="68"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2095,12 +2095,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="79"/>
-      <c r="B12" s="70" t="s">
+      <c r="A12" s="70"/>
+      <c r="B12" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="71"/>
-      <c r="D12" s="71"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2151,10 +2151,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="79"/>
-      <c r="B13" s="70"/>
-      <c r="C13" s="63"/>
-      <c r="D13" s="63"/>
+      <c r="A13" s="70"/>
+      <c r="B13" s="73"/>
+      <c r="C13" s="68"/>
+      <c r="D13" s="68"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2205,14 +2205,14 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="79"/>
-      <c r="B14" s="70" t="s">
+      <c r="A14" s="70"/>
+      <c r="B14" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="71" t="s">
+      <c r="C14" s="82" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="71" t="s">
+      <c r="D14" s="82" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="42"/>
@@ -2265,10 +2265,10 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="79"/>
-      <c r="B15" s="70"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
+      <c r="A15" s="70"/>
+      <c r="B15" s="73"/>
+      <c r="C15" s="68"/>
+      <c r="D15" s="68"/>
       <c r="E15" s="42"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -2319,14 +2319,14 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="79"/>
-      <c r="B16" s="89" t="s">
+      <c r="A16" s="70"/>
+      <c r="B16" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="63" t="s">
+      <c r="C16" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="64" t="s">
+      <c r="D16" s="76" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="20"/>
@@ -2379,10 +2379,10 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="80"/>
-      <c r="B17" s="90"/>
-      <c r="C17" s="91"/>
-      <c r="D17" s="92"/>
+      <c r="A17" s="71"/>
+      <c r="B17" s="106"/>
+      <c r="C17" s="78"/>
+      <c r="D17" s="79"/>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
@@ -2433,14 +2433,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="78" t="s">
+      <c r="A18" s="69" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="100" t="s">
+      <c r="B18" s="95" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="98"/>
-      <c r="D18" s="99"/>
+      <c r="C18" s="74"/>
+      <c r="D18" s="75"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2491,10 +2491,10 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="79"/>
-      <c r="B19" s="101"/>
-      <c r="C19" s="63"/>
-      <c r="D19" s="64"/>
+      <c r="A19" s="70"/>
+      <c r="B19" s="80"/>
+      <c r="C19" s="68"/>
+      <c r="D19" s="76"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2545,12 +2545,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="79"/>
-      <c r="B20" s="70" t="s">
+      <c r="A20" s="70"/>
+      <c r="B20" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="63"/>
-      <c r="D20" s="64"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="76"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2590,10 +2590,10 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="79"/>
-      <c r="B21" s="70"/>
-      <c r="C21" s="63"/>
-      <c r="D21" s="64"/>
+      <c r="A21" s="70"/>
+      <c r="B21" s="73"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="76"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2644,14 +2644,14 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="79"/>
-      <c r="B22" s="70" t="s">
+      <c r="A22" s="70"/>
+      <c r="B22" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="63">
+      <c r="C22" s="68">
         <v>0.1</v>
       </c>
-      <c r="D22" s="64">
+      <c r="D22" s="76">
         <v>0.1</v>
       </c>
       <c r="E22" s="11"/>
@@ -2704,10 +2704,10 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="79"/>
-      <c r="B23" s="70"/>
-      <c r="C23" s="63"/>
-      <c r="D23" s="64"/>
+      <c r="A23" s="70"/>
+      <c r="B23" s="73"/>
+      <c r="C23" s="68"/>
+      <c r="D23" s="76"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2758,10 +2758,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="79"/>
-      <c r="B24" s="89"/>
-      <c r="C24" s="81"/>
-      <c r="D24" s="104"/>
+      <c r="A24" s="70"/>
+      <c r="B24" s="81"/>
+      <c r="C24" s="83"/>
+      <c r="D24" s="87"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2812,10 +2812,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="79"/>
+      <c r="A25" s="70"/>
       <c r="B25" s="66"/>
-      <c r="C25" s="71"/>
-      <c r="D25" s="105"/>
+      <c r="C25" s="82"/>
+      <c r="D25" s="88"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2866,12 +2866,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="79"/>
-      <c r="B26" s="70" t="s">
+      <c r="A26" s="70"/>
+      <c r="B26" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="81"/>
-      <c r="D26" s="104">
+      <c r="C26" s="83"/>
+      <c r="D26" s="87">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2924,10 +2924,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="80"/>
-      <c r="B27" s="70"/>
-      <c r="C27" s="93"/>
-      <c r="D27" s="106"/>
+      <c r="A27" s="71"/>
+      <c r="B27" s="73"/>
+      <c r="C27" s="107"/>
+      <c r="D27" s="89"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2978,14 +2978,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="78" t="s">
+      <c r="A28" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="96" t="s">
+      <c r="B28" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="98"/>
-      <c r="D28" s="99"/>
+      <c r="C28" s="74"/>
+      <c r="D28" s="75"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -3036,10 +3036,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="79"/>
-      <c r="B29" s="97"/>
-      <c r="C29" s="91"/>
-      <c r="D29" s="92"/>
+      <c r="A29" s="70"/>
+      <c r="B29" s="77"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="79"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3090,16 +3090,16 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="78" t="s">
+      <c r="A30" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="96" t="s">
+      <c r="B30" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="98">
+      <c r="C30" s="74">
         <v>2</v>
       </c>
-      <c r="D30" s="99">
+      <c r="D30" s="75">
         <v>2</v>
       </c>
       <c r="E30" s="53"/>
@@ -3152,10 +3152,10 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="79"/>
-      <c r="B31" s="70"/>
-      <c r="C31" s="63"/>
-      <c r="D31" s="64"/>
+      <c r="A31" s="70"/>
+      <c r="B31" s="73"/>
+      <c r="C31" s="68"/>
+      <c r="D31" s="76"/>
       <c r="E31" s="59"/>
       <c r="F31" s="60"/>
       <c r="G31" s="43"/>
@@ -3206,14 +3206,14 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="79"/>
+      <c r="A32" s="70"/>
       <c r="B32" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="63">
+      <c r="C32" s="68">
         <v>4</v>
       </c>
-      <c r="D32" s="63">
+      <c r="D32" s="68">
         <v>7</v>
       </c>
       <c r="E32" s="11"/>
@@ -3266,10 +3266,10 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="79"/>
+      <c r="A33" s="70"/>
       <c r="B33" s="66"/>
-      <c r="C33" s="63"/>
-      <c r="D33" s="63"/>
+      <c r="C33" s="68"/>
+      <c r="D33" s="68"/>
       <c r="E33" s="11"/>
       <c r="F33" s="60"/>
       <c r="G33" s="60"/>
@@ -3320,14 +3320,14 @@
       <c r="AZ33" s="13"/>
     </row>
     <row r="34" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="79"/>
+      <c r="A34" s="70"/>
       <c r="B34" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="63" t="s">
+      <c r="C34" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="63" t="s">
+      <c r="D34" s="68" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="11"/>
@@ -3380,10 +3380,10 @@
       <c r="AZ34" s="13"/>
     </row>
     <row r="35" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="79"/>
+      <c r="A35" s="70"/>
       <c r="B35" s="66"/>
-      <c r="C35" s="63"/>
-      <c r="D35" s="63"/>
+      <c r="C35" s="68"/>
+      <c r="D35" s="68"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -3434,14 +3434,14 @@
       <c r="AZ35" s="13"/>
     </row>
     <row r="36" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="79"/>
+      <c r="A36" s="70"/>
       <c r="B36" s="65" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="63">
+      <c r="C36" s="68">
         <v>1.5</v>
       </c>
-      <c r="D36" s="63">
+      <c r="D36" s="68">
         <v>2</v>
       </c>
       <c r="E36" s="11"/>
@@ -3494,10 +3494,10 @@
       <c r="AZ36" s="13"/>
     </row>
     <row r="37" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="79"/>
+      <c r="A37" s="70"/>
       <c r="B37" s="66"/>
-      <c r="C37" s="63"/>
-      <c r="D37" s="63"/>
+      <c r="C37" s="68"/>
+      <c r="D37" s="68"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
@@ -3548,14 +3548,14 @@
       <c r="AZ37" s="13"/>
     </row>
     <row r="38" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="79"/>
+      <c r="A38" s="70"/>
       <c r="B38" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="63">
+      <c r="C38" s="68">
         <v>7</v>
       </c>
-      <c r="D38" s="64">
+      <c r="D38" s="76">
         <v>6</v>
       </c>
       <c r="E38" s="11"/>
@@ -3608,10 +3608,10 @@
       <c r="AZ38" s="13"/>
     </row>
     <row r="39" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="79"/>
+      <c r="A39" s="70"/>
       <c r="B39" s="66"/>
-      <c r="C39" s="63"/>
-      <c r="D39" s="64"/>
+      <c r="C39" s="68"/>
+      <c r="D39" s="76"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
@@ -3662,14 +3662,14 @@
       <c r="AZ39" s="13"/>
     </row>
     <row r="40" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="79"/>
+      <c r="A40" s="70"/>
       <c r="B40" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="63">
+      <c r="C40" s="68">
         <v>6</v>
       </c>
-      <c r="D40" s="64"/>
+      <c r="D40" s="76"/>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
@@ -3684,8 +3684,8 @@
       <c r="P40" s="13"/>
       <c r="Q40" s="11"/>
       <c r="R40" s="12"/>
-      <c r="S40" s="109"/>
-      <c r="T40" s="110"/>
+      <c r="S40" s="63"/>
+      <c r="T40" s="64"/>
       <c r="U40" s="11"/>
       <c r="V40" s="12"/>
       <c r="W40" s="12"/>
@@ -3720,10 +3720,10 @@
       <c r="AZ40" s="13"/>
     </row>
     <row r="41" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="79"/>
+      <c r="A41" s="70"/>
       <c r="B41" s="66"/>
-      <c r="C41" s="63"/>
-      <c r="D41" s="64"/>
+      <c r="C41" s="68"/>
+      <c r="D41" s="76"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
@@ -3740,7 +3740,7 @@
       <c r="R41" s="43"/>
       <c r="S41" s="43"/>
       <c r="T41" s="49"/>
-      <c r="U41" s="11"/>
+      <c r="U41" s="59"/>
       <c r="V41" s="12"/>
       <c r="W41" s="12"/>
       <c r="X41" s="13"/>
@@ -3774,14 +3774,14 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="79"/>
+      <c r="A42" s="70"/>
       <c r="B42" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="63">
+      <c r="C42" s="68">
         <v>4</v>
       </c>
-      <c r="D42" s="64">
+      <c r="D42" s="76">
         <v>2</v>
       </c>
       <c r="E42" s="11"/>
@@ -3834,10 +3834,10 @@
       <c r="AZ42" s="13"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A43" s="79"/>
+      <c r="A43" s="70"/>
       <c r="B43" s="66"/>
-      <c r="C43" s="63"/>
-      <c r="D43" s="64"/>
+      <c r="C43" s="68"/>
+      <c r="D43" s="76"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
@@ -3888,12 +3888,12 @@
       <c r="AZ43" s="13"/>
     </row>
     <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="79"/>
+      <c r="A44" s="70"/>
       <c r="B44" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="63"/>
-      <c r="D44" s="64"/>
+      <c r="C44" s="68"/>
+      <c r="D44" s="76"/>
       <c r="E44" s="11"/>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
@@ -3944,10 +3944,10 @@
       <c r="AZ44" s="13"/>
     </row>
     <row r="45" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="79"/>
+      <c r="A45" s="70"/>
       <c r="B45" s="66"/>
-      <c r="C45" s="63"/>
-      <c r="D45" s="64"/>
+      <c r="C45" s="68"/>
+      <c r="D45" s="76"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
@@ -3965,7 +3965,7 @@
       <c r="S45" s="12"/>
       <c r="T45" s="61"/>
       <c r="U45" s="11"/>
-      <c r="V45" s="12"/>
+      <c r="V45" s="60"/>
       <c r="W45" s="12"/>
       <c r="X45" s="13"/>
       <c r="Y45" s="11"/>
@@ -3998,12 +3998,12 @@
       <c r="AZ45" s="13"/>
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A46" s="79"/>
+      <c r="A46" s="70"/>
       <c r="B46" s="65" t="s">
         <v>48</v>
       </c>
-      <c r="C46" s="95"/>
-      <c r="D46" s="64"/>
+      <c r="C46" s="67"/>
+      <c r="D46" s="76"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -4054,10 +4054,10 @@
       <c r="AZ46" s="13"/>
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A47" s="79"/>
+      <c r="A47" s="70"/>
       <c r="B47" s="66"/>
-      <c r="C47" s="95"/>
-      <c r="D47" s="64"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="76"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -4108,12 +4108,12 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="79"/>
+      <c r="A48" s="70"/>
       <c r="B48" s="65" t="s">
         <v>49</v>
       </c>
-      <c r="C48" s="63"/>
-      <c r="D48" s="63"/>
+      <c r="C48" s="68"/>
+      <c r="D48" s="68"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4164,10 +4164,10 @@
       <c r="AZ48" s="13"/>
     </row>
     <row r="49" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A49" s="79"/>
+      <c r="A49" s="70"/>
       <c r="B49" s="66"/>
-      <c r="C49" s="63"/>
-      <c r="D49" s="63"/>
+      <c r="C49" s="68"/>
+      <c r="D49" s="68"/>
       <c r="E49" s="11"/>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
@@ -4218,10 +4218,10 @@
       <c r="AZ49" s="13"/>
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A50" s="79"/>
+      <c r="A50" s="70"/>
       <c r="B50" s="65"/>
-      <c r="C50" s="63"/>
-      <c r="D50" s="63"/>
+      <c r="C50" s="68"/>
+      <c r="D50" s="68"/>
       <c r="E50" s="42"/>
       <c r="F50" s="43"/>
       <c r="G50" s="12"/>
@@ -4272,10 +4272,10 @@
       <c r="AZ50" s="13"/>
     </row>
     <row r="51" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A51" s="79"/>
+      <c r="A51" s="70"/>
       <c r="B51" s="66"/>
-      <c r="C51" s="63"/>
-      <c r="D51" s="63"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="68"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4326,14 +4326,14 @@
       <c r="AZ51" s="13"/>
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A52" s="79"/>
+      <c r="A52" s="70"/>
       <c r="B52" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="63">
+      <c r="C52" s="68">
         <v>2</v>
       </c>
-      <c r="D52" s="63" t="s">
+      <c r="D52" s="68" t="s">
         <v>46</v>
       </c>
       <c r="E52" s="11"/>
@@ -4386,10 +4386,10 @@
       <c r="AZ52" s="13"/>
     </row>
     <row r="53" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A53" s="79"/>
+      <c r="A53" s="70"/>
       <c r="B53" s="66"/>
-      <c r="C53" s="63"/>
-      <c r="D53" s="63"/>
+      <c r="C53" s="68"/>
+      <c r="D53" s="68"/>
       <c r="E53" s="11"/>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
@@ -4440,12 +4440,12 @@
       <c r="AZ53" s="13"/>
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A54" s="79"/>
+      <c r="A54" s="70"/>
       <c r="B54" s="65" t="s">
         <v>44</v>
       </c>
-      <c r="C54" s="63"/>
-      <c r="D54" s="63"/>
+      <c r="C54" s="68"/>
+      <c r="D54" s="68"/>
       <c r="E54" s="11"/>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
@@ -4496,10 +4496,10 @@
       <c r="AZ54" s="13"/>
     </row>
     <row r="55" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A55" s="79"/>
+      <c r="A55" s="70"/>
       <c r="B55" s="66"/>
-      <c r="C55" s="63"/>
-      <c r="D55" s="63"/>
+      <c r="C55" s="68"/>
+      <c r="D55" s="68"/>
       <c r="E55" s="11"/>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
@@ -4550,12 +4550,12 @@
       <c r="AZ55" s="13"/>
     </row>
     <row r="56" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="79"/>
+      <c r="A56" s="70"/>
       <c r="B56" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="C56" s="95"/>
-      <c r="D56" s="64"/>
+      <c r="C56" s="67"/>
+      <c r="D56" s="76"/>
       <c r="E56" s="11"/>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
@@ -4606,10 +4606,10 @@
       <c r="AZ56" s="13"/>
     </row>
     <row r="57" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="79"/>
+      <c r="A57" s="70"/>
       <c r="B57" s="66"/>
-      <c r="C57" s="63"/>
-      <c r="D57" s="64"/>
+      <c r="C57" s="68"/>
+      <c r="D57" s="76"/>
       <c r="E57" s="11"/>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
@@ -4660,12 +4660,12 @@
       <c r="AZ57" s="13"/>
     </row>
     <row r="58" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A58" s="79"/>
-      <c r="B58" s="94" t="s">
+      <c r="A58" s="70"/>
+      <c r="B58" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="C58" s="63"/>
-      <c r="D58" s="64"/>
+      <c r="C58" s="68"/>
+      <c r="D58" s="76"/>
       <c r="E58" s="11"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
@@ -4716,10 +4716,10 @@
       <c r="AZ58" s="13"/>
     </row>
     <row r="59" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A59" s="79"/>
-      <c r="B59" s="94"/>
-      <c r="C59" s="63"/>
-      <c r="D59" s="64"/>
+      <c r="A59" s="70"/>
+      <c r="B59" s="86"/>
+      <c r="C59" s="68"/>
+      <c r="D59" s="76"/>
       <c r="E59" s="11"/>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
@@ -4770,12 +4770,12 @@
       <c r="AZ59" s="13"/>
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A60" s="79"/>
-      <c r="B60" s="70" t="s">
+      <c r="A60" s="70"/>
+      <c r="B60" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="C60" s="63"/>
-      <c r="D60" s="64">
+      <c r="C60" s="68"/>
+      <c r="D60" s="76">
         <v>0</v>
       </c>
       <c r="E60" s="11"/>
@@ -4828,10 +4828,10 @@
       <c r="AZ60" s="13"/>
     </row>
     <row r="61" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="79"/>
-      <c r="B61" s="70"/>
-      <c r="C61" s="63"/>
-      <c r="D61" s="64"/>
+      <c r="A61" s="70"/>
+      <c r="B61" s="73"/>
+      <c r="C61" s="68"/>
+      <c r="D61" s="76"/>
       <c r="E61" s="11"/>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
@@ -4882,14 +4882,14 @@
       <c r="AZ61" s="13"/>
     </row>
     <row r="62" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A62" s="78" t="s">
+      <c r="A62" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="B62" s="96" t="s">
+      <c r="B62" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="C62" s="98"/>
-      <c r="D62" s="99"/>
+      <c r="C62" s="74"/>
+      <c r="D62" s="75"/>
       <c r="E62" s="8"/>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -4940,10 +4940,10 @@
       <c r="AZ62" s="10"/>
     </row>
     <row r="63" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A63" s="79"/>
-      <c r="B63" s="70"/>
-      <c r="C63" s="63"/>
-      <c r="D63" s="64"/>
+      <c r="A63" s="70"/>
+      <c r="B63" s="73"/>
+      <c r="C63" s="68"/>
+      <c r="D63" s="76"/>
       <c r="E63" s="11"/>
       <c r="F63" s="12"/>
       <c r="G63" s="12"/>
@@ -4994,12 +4994,12 @@
       <c r="AZ63" s="13"/>
     </row>
     <row r="64" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="79"/>
+      <c r="A64" s="70"/>
       <c r="B64" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="C64" s="95"/>
-      <c r="D64" s="95"/>
+      <c r="C64" s="67"/>
+      <c r="D64" s="67"/>
       <c r="E64" s="11"/>
       <c r="F64" s="12"/>
       <c r="G64" s="12"/>
@@ -5050,10 +5050,10 @@
       <c r="AZ64" s="13"/>
     </row>
     <row r="65" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="79"/>
+      <c r="A65" s="70"/>
       <c r="B65" s="66"/>
-      <c r="C65" s="63"/>
-      <c r="D65" s="63"/>
+      <c r="C65" s="68"/>
+      <c r="D65" s="68"/>
       <c r="E65" s="11"/>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
@@ -5104,12 +5104,12 @@
       <c r="AZ65" s="13"/>
     </row>
     <row r="66" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A66" s="79"/>
-      <c r="B66" s="70" t="s">
+      <c r="A66" s="70"/>
+      <c r="B66" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="C66" s="63"/>
-      <c r="D66" s="64"/>
+      <c r="C66" s="68"/>
+      <c r="D66" s="76"/>
       <c r="E66" s="11"/>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
@@ -5160,10 +5160,10 @@
       <c r="AZ66" s="13"/>
     </row>
     <row r="67" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="80"/>
-      <c r="B67" s="97"/>
-      <c r="C67" s="91"/>
-      <c r="D67" s="92"/>
+      <c r="A67" s="71"/>
+      <c r="B67" s="77"/>
+      <c r="C67" s="78"/>
+      <c r="D67" s="79"/>
       <c r="E67" s="17"/>
       <c r="F67" s="18"/>
       <c r="G67" s="18"/>
@@ -5214,14 +5214,14 @@
       <c r="AZ67" s="19"/>
     </row>
     <row r="68" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="78" t="s">
+      <c r="A68" s="69" t="s">
         <v>15</v>
       </c>
       <c r="B68" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="C68" s="95"/>
-      <c r="D68" s="95"/>
+      <c r="C68" s="67"/>
+      <c r="D68" s="67"/>
       <c r="E68" s="11"/>
       <c r="F68" s="12"/>
       <c r="G68" s="12"/>
@@ -5272,10 +5272,10 @@
       <c r="AZ68" s="13"/>
     </row>
     <row r="69" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="79"/>
+      <c r="A69" s="70"/>
       <c r="B69" s="66"/>
-      <c r="C69" s="63"/>
-      <c r="D69" s="63"/>
+      <c r="C69" s="68"/>
+      <c r="D69" s="68"/>
       <c r="E69" s="11"/>
       <c r="F69" s="12"/>
       <c r="G69" s="12"/>
@@ -5326,12 +5326,12 @@
       <c r="AZ69" s="13"/>
     </row>
     <row r="70" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="79"/>
+      <c r="A70" s="70"/>
       <c r="B70" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="C70" s="95"/>
-      <c r="D70" s="95">
+      <c r="C70" s="67"/>
+      <c r="D70" s="67">
         <v>0</v>
       </c>
       <c r="E70" s="11"/>
@@ -5384,10 +5384,10 @@
       <c r="AZ70" s="13"/>
     </row>
     <row r="71" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="80"/>
-      <c r="B71" s="101"/>
-      <c r="C71" s="63"/>
-      <c r="D71" s="63"/>
+      <c r="A71" s="71"/>
+      <c r="B71" s="80"/>
+      <c r="C71" s="68"/>
+      <c r="D71" s="68"/>
       <c r="E71" s="17"/>
       <c r="F71" s="18"/>
       <c r="G71" s="18"/>
@@ -5501,41 +5501,77 @@
     <row r="73" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="135">
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="D70:D71"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="AS2:AV2"/>
+    <mergeCell ref="AW2:AZ2"/>
+    <mergeCell ref="AS1:AV1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="A8:A17"/>
+    <mergeCell ref="A18:A27"/>
+    <mergeCell ref="AK1:AN1"/>
+    <mergeCell ref="AO1:AR1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="Q1:T1"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="AK2:AN2"/>
+    <mergeCell ref="AO2:AR2"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="U2:X2"/>
+    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A61"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="C60:C61"/>
     <mergeCell ref="B56:B57"/>
     <mergeCell ref="C56:C57"/>
     <mergeCell ref="D56:D57"/>
@@ -5560,82 +5596,46 @@
     <mergeCell ref="D6:D7"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A61"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="AS2:AV2"/>
-    <mergeCell ref="AW2:AZ2"/>
-    <mergeCell ref="AS1:AV1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A8:A17"/>
-    <mergeCell ref="A18:A27"/>
-    <mergeCell ref="AK1:AN1"/>
-    <mergeCell ref="AO1:AR1"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="M1:P1"/>
-    <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="AG2:AJ2"/>
-    <mergeCell ref="AK2:AN2"/>
-    <mergeCell ref="AO2:AR2"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
     <mergeCell ref="B32:B33"/>
     <mergeCell ref="B34:B35"/>
     <mergeCell ref="C32:C33"/>
     <mergeCell ref="D32:D33"/>
     <mergeCell ref="C34:C35"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="D70:D71"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Responsive Navbar and security features
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8897C6B-360D-4A89-89FD-88DFF2735E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24405420-592F-4DCF-83B5-CDE038A613B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -166,9 +166,6 @@
     <t>ERM-Diagramm</t>
   </si>
   <si>
-    <t>Actifity Diagramm</t>
-  </si>
-  <si>
     <t>Klassendiagramm</t>
   </si>
   <si>
@@ -182,6 +179,9 @@
   </si>
   <si>
     <t>Projektstruktur verbessern</t>
+  </si>
+  <si>
+    <t>Responsive Design</t>
   </si>
 </sst>
 </file>
@@ -874,19 +874,85 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -898,11 +964,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -912,27 +975,6 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -955,62 +997,20 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1346,162 +1346,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="108" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="99" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="88" t="s">
+      <c r="C1" s="102" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="89"/>
-      <c r="E1" s="70" t="s">
+      <c r="D1" s="103"/>
+      <c r="E1" s="92" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="70" t="s">
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
+      <c r="H1" s="94"/>
+      <c r="I1" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="70" t="s">
+      <c r="J1" s="93"/>
+      <c r="K1" s="93"/>
+      <c r="L1" s="94"/>
+      <c r="M1" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="71"/>
-      <c r="O1" s="71"/>
-      <c r="P1" s="72"/>
-      <c r="Q1" s="70" t="s">
+      <c r="N1" s="93"/>
+      <c r="O1" s="93"/>
+      <c r="P1" s="94"/>
+      <c r="Q1" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="71"/>
-      <c r="S1" s="71"/>
-      <c r="T1" s="72"/>
-      <c r="U1" s="70" t="s">
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="94"/>
+      <c r="U1" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="71"/>
-      <c r="W1" s="71"/>
-      <c r="X1" s="72"/>
-      <c r="Y1" s="70" t="s">
+      <c r="V1" s="93"/>
+      <c r="W1" s="93"/>
+      <c r="X1" s="94"/>
+      <c r="Y1" s="92" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="71"/>
-      <c r="AA1" s="71"/>
-      <c r="AB1" s="72"/>
-      <c r="AC1" s="70" t="s">
+      <c r="Z1" s="93"/>
+      <c r="AA1" s="93"/>
+      <c r="AB1" s="94"/>
+      <c r="AC1" s="92" t="s">
         <v>29</v>
       </c>
-      <c r="AD1" s="71"/>
-      <c r="AE1" s="71"/>
-      <c r="AF1" s="72"/>
-      <c r="AG1" s="70" t="s">
+      <c r="AD1" s="93"/>
+      <c r="AE1" s="93"/>
+      <c r="AF1" s="94"/>
+      <c r="AG1" s="92" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="71"/>
-      <c r="AI1" s="71"/>
-      <c r="AJ1" s="72"/>
-      <c r="AK1" s="70" t="s">
+      <c r="AH1" s="93"/>
+      <c r="AI1" s="93"/>
+      <c r="AJ1" s="94"/>
+      <c r="AK1" s="92" t="s">
         <v>31</v>
       </c>
-      <c r="AL1" s="71"/>
-      <c r="AM1" s="71"/>
-      <c r="AN1" s="72"/>
-      <c r="AO1" s="70" t="s">
+      <c r="AL1" s="93"/>
+      <c r="AM1" s="93"/>
+      <c r="AN1" s="94"/>
+      <c r="AO1" s="92" t="s">
         <v>27</v>
       </c>
-      <c r="AP1" s="71"/>
-      <c r="AQ1" s="71"/>
-      <c r="AR1" s="72"/>
-      <c r="AS1" s="70"/>
-      <c r="AT1" s="71"/>
-      <c r="AU1" s="71"/>
-      <c r="AV1" s="72"/>
-      <c r="AW1" s="70"/>
-      <c r="AX1" s="71"/>
-      <c r="AY1" s="71"/>
-      <c r="AZ1" s="72"/>
+      <c r="AP1" s="93"/>
+      <c r="AQ1" s="93"/>
+      <c r="AR1" s="94"/>
+      <c r="AS1" s="92"/>
+      <c r="AT1" s="93"/>
+      <c r="AU1" s="93"/>
+      <c r="AV1" s="94"/>
+      <c r="AW1" s="92"/>
+      <c r="AX1" s="93"/>
+      <c r="AY1" s="93"/>
+      <c r="AZ1" s="94"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="79"/>
-      <c r="B2" s="86"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="75">
+      <c r="A2" s="109"/>
+      <c r="B2" s="100"/>
+      <c r="C2" s="104"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="96">
         <v>44781</v>
       </c>
-      <c r="F2" s="76"/>
-      <c r="G2" s="76"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="75">
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="96">
         <v>44782</v>
       </c>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="77"/>
-      <c r="M2" s="75">
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="96">
         <v>44783</v>
       </c>
-      <c r="N2" s="76"/>
-      <c r="O2" s="76"/>
-      <c r="P2" s="77"/>
-      <c r="Q2" s="75">
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
+      <c r="P2" s="98"/>
+      <c r="Q2" s="96">
         <v>44784</v>
       </c>
-      <c r="R2" s="76"/>
-      <c r="S2" s="76"/>
-      <c r="T2" s="77"/>
-      <c r="U2" s="75">
+      <c r="R2" s="97"/>
+      <c r="S2" s="97"/>
+      <c r="T2" s="98"/>
+      <c r="U2" s="96">
         <v>44785</v>
       </c>
-      <c r="V2" s="76"/>
-      <c r="W2" s="76"/>
-      <c r="X2" s="77"/>
-      <c r="Y2" s="75">
+      <c r="V2" s="97"/>
+      <c r="W2" s="97"/>
+      <c r="X2" s="98"/>
+      <c r="Y2" s="96">
         <v>44789</v>
       </c>
-      <c r="Z2" s="76"/>
-      <c r="AA2" s="76"/>
-      <c r="AB2" s="77"/>
-      <c r="AC2" s="75">
+      <c r="Z2" s="97"/>
+      <c r="AA2" s="97"/>
+      <c r="AB2" s="98"/>
+      <c r="AC2" s="96">
         <v>44790</v>
       </c>
-      <c r="AD2" s="76"/>
-      <c r="AE2" s="76"/>
-      <c r="AF2" s="77"/>
-      <c r="AG2" s="75">
+      <c r="AD2" s="97"/>
+      <c r="AE2" s="97"/>
+      <c r="AF2" s="98"/>
+      <c r="AG2" s="96">
         <v>44791</v>
       </c>
-      <c r="AH2" s="76"/>
-      <c r="AI2" s="76"/>
-      <c r="AJ2" s="77"/>
-      <c r="AK2" s="75">
+      <c r="AH2" s="97"/>
+      <c r="AI2" s="97"/>
+      <c r="AJ2" s="98"/>
+      <c r="AK2" s="96">
         <v>44792</v>
       </c>
-      <c r="AL2" s="76"/>
-      <c r="AM2" s="76"/>
-      <c r="AN2" s="77"/>
-      <c r="AO2" s="75">
+      <c r="AL2" s="97"/>
+      <c r="AM2" s="97"/>
+      <c r="AN2" s="98"/>
+      <c r="AO2" s="96">
         <v>44795</v>
       </c>
-      <c r="AP2" s="76"/>
-      <c r="AQ2" s="76"/>
-      <c r="AR2" s="77"/>
-      <c r="AS2" s="75"/>
-      <c r="AT2" s="76"/>
-      <c r="AU2" s="76"/>
-      <c r="AV2" s="77"/>
-      <c r="AW2" s="75"/>
-      <c r="AX2" s="76"/>
-      <c r="AY2" s="76"/>
-      <c r="AZ2" s="77"/>
+      <c r="AP2" s="97"/>
+      <c r="AQ2" s="97"/>
+      <c r="AR2" s="98"/>
+      <c r="AS2" s="96"/>
+      <c r="AT2" s="97"/>
+      <c r="AU2" s="97"/>
+      <c r="AV2" s="98"/>
+      <c r="AW2" s="96"/>
+      <c r="AX2" s="97"/>
+      <c r="AY2" s="97"/>
+      <c r="AZ2" s="98"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="80"/>
-      <c r="B3" s="87"/>
+      <c r="A3" s="110"/>
+      <c r="B3" s="101"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
@@ -1639,11 +1639,11 @@
     </row>
     <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="67" t="s">
+      <c r="B4" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="74"/>
-      <c r="D4" s="105"/>
+      <c r="C4" s="82"/>
+      <c r="D4" s="84"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1699,9 +1699,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="92"/>
-      <c r="C5" s="84"/>
-      <c r="D5" s="104"/>
+      <c r="B5" s="81"/>
+      <c r="C5" s="83"/>
+      <c r="D5" s="85"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1757,9 +1757,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="97"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="68"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="76"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1804,9 +1804,9 @@
     </row>
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="66"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="104"/>
+      <c r="B7" s="65"/>
+      <c r="C7" s="83"/>
+      <c r="D7" s="85"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1861,16 +1861,16 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="81" t="s">
+      <c r="A8" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="98" t="s">
+      <c r="B8" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="100">
+      <c r="C8" s="74">
         <v>0.1</v>
       </c>
-      <c r="D8" s="109">
+      <c r="D8" s="90">
         <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
@@ -1927,10 +1927,10 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="82"/>
+      <c r="A9" s="70"/>
       <c r="B9" s="73"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="110"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="91"/>
       <c r="E9" s="42"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -1981,14 +1981,14 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="82"/>
+      <c r="A10" s="70"/>
       <c r="B10" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="74">
+      <c r="C10" s="82">
         <v>1</v>
       </c>
-      <c r="D10" s="74">
+      <c r="D10" s="82">
         <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
@@ -2041,10 +2041,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="82"/>
+      <c r="A11" s="70"/>
       <c r="B11" s="73"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
+      <c r="C11" s="68"/>
+      <c r="D11" s="68"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2095,12 +2095,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="82"/>
+      <c r="A12" s="70"/>
       <c r="B12" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="74"/>
-      <c r="D12" s="74"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="82"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2151,10 +2151,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="82"/>
+      <c r="A13" s="70"/>
       <c r="B13" s="73"/>
-      <c r="C13" s="65"/>
-      <c r="D13" s="65"/>
+      <c r="C13" s="68"/>
+      <c r="D13" s="68"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2205,14 +2205,14 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="82"/>
+      <c r="A14" s="70"/>
       <c r="B14" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="74" t="s">
+      <c r="C14" s="82" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="74" t="s">
+      <c r="D14" s="82" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="42"/>
@@ -2265,10 +2265,10 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="82"/>
+      <c r="A15" s="70"/>
       <c r="B15" s="73"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="65"/>
+      <c r="C15" s="68"/>
+      <c r="D15" s="68"/>
       <c r="E15" s="42"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -2319,14 +2319,14 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="82"/>
-      <c r="B16" s="92" t="s">
+      <c r="A16" s="70"/>
+      <c r="B16" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="65" t="s">
+      <c r="C16" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="68" t="s">
+      <c r="D16" s="76" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="20"/>
@@ -2379,10 +2379,10 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="83"/>
-      <c r="B17" s="93"/>
-      <c r="C17" s="94"/>
-      <c r="D17" s="95"/>
+      <c r="A17" s="71"/>
+      <c r="B17" s="106"/>
+      <c r="C17" s="78"/>
+      <c r="D17" s="79"/>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
@@ -2433,14 +2433,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="81" t="s">
+      <c r="A18" s="69" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="102" t="s">
+      <c r="B18" s="95" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="100"/>
-      <c r="D18" s="101"/>
+      <c r="C18" s="74"/>
+      <c r="D18" s="75"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2491,10 +2491,10 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="82"/>
-      <c r="B19" s="103"/>
-      <c r="C19" s="65"/>
-      <c r="D19" s="68"/>
+      <c r="A19" s="70"/>
+      <c r="B19" s="80"/>
+      <c r="C19" s="68"/>
+      <c r="D19" s="76"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2545,12 +2545,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="82"/>
+      <c r="A20" s="70"/>
       <c r="B20" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="65"/>
-      <c r="D20" s="68"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="76"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2590,10 +2590,10 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="82"/>
+      <c r="A21" s="70"/>
       <c r="B21" s="73"/>
-      <c r="C21" s="65"/>
-      <c r="D21" s="68"/>
+      <c r="C21" s="68"/>
+      <c r="D21" s="76"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2644,14 +2644,14 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="82"/>
+      <c r="A22" s="70"/>
       <c r="B22" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="65">
+      <c r="C22" s="68">
         <v>0.1</v>
       </c>
-      <c r="D22" s="68">
+      <c r="D22" s="76">
         <v>0.1</v>
       </c>
       <c r="E22" s="11"/>
@@ -2704,10 +2704,10 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="82"/>
+      <c r="A23" s="70"/>
       <c r="B23" s="73"/>
-      <c r="C23" s="65"/>
-      <c r="D23" s="68"/>
+      <c r="C23" s="68"/>
+      <c r="D23" s="76"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2758,10 +2758,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="82"/>
-      <c r="B24" s="92"/>
-      <c r="C24" s="84"/>
-      <c r="D24" s="106"/>
+      <c r="A24" s="70"/>
+      <c r="B24" s="81"/>
+      <c r="C24" s="83"/>
+      <c r="D24" s="87"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2812,10 +2812,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="82"/>
-      <c r="B25" s="67"/>
-      <c r="C25" s="74"/>
-      <c r="D25" s="107"/>
+      <c r="A25" s="70"/>
+      <c r="B25" s="66"/>
+      <c r="C25" s="82"/>
+      <c r="D25" s="88"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2866,12 +2866,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="82"/>
+      <c r="A26" s="70"/>
       <c r="B26" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="84"/>
-      <c r="D26" s="106">
+      <c r="C26" s="83"/>
+      <c r="D26" s="87">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2924,10 +2924,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="83"/>
+      <c r="A27" s="71"/>
       <c r="B27" s="73"/>
-      <c r="C27" s="96"/>
-      <c r="D27" s="108"/>
+      <c r="C27" s="107"/>
+      <c r="D27" s="89"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2978,14 +2978,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="81" t="s">
+      <c r="A28" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="98" t="s">
+      <c r="B28" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="100"/>
-      <c r="D28" s="101"/>
+      <c r="C28" s="74"/>
+      <c r="D28" s="75"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -3036,10 +3036,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="82"/>
-      <c r="B29" s="99"/>
-      <c r="C29" s="94"/>
-      <c r="D29" s="95"/>
+      <c r="A29" s="70"/>
+      <c r="B29" s="77"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="79"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3090,16 +3090,16 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="81" t="s">
+      <c r="A30" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="98" t="s">
+      <c r="B30" s="72" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="100">
+      <c r="C30" s="74">
         <v>2</v>
       </c>
-      <c r="D30" s="101">
+      <c r="D30" s="75">
         <v>2</v>
       </c>
       <c r="E30" s="53"/>
@@ -3152,10 +3152,10 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="82"/>
+      <c r="A31" s="70"/>
       <c r="B31" s="73"/>
-      <c r="C31" s="65"/>
-      <c r="D31" s="68"/>
+      <c r="C31" s="68"/>
+      <c r="D31" s="76"/>
       <c r="E31" s="59"/>
       <c r="F31" s="60"/>
       <c r="G31" s="43"/>
@@ -3206,14 +3206,14 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="82"/>
-      <c r="B32" s="66" t="s">
+      <c r="A32" s="70"/>
+      <c r="B32" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="65">
+      <c r="C32" s="68">
         <v>4</v>
       </c>
-      <c r="D32" s="65">
+      <c r="D32" s="68">
         <v>7</v>
       </c>
       <c r="E32" s="11"/>
@@ -3266,10 +3266,10 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="82"/>
-      <c r="B33" s="67"/>
-      <c r="C33" s="65"/>
-      <c r="D33" s="65"/>
+      <c r="A33" s="70"/>
+      <c r="B33" s="66"/>
+      <c r="C33" s="68"/>
+      <c r="D33" s="68"/>
       <c r="E33" s="11"/>
       <c r="F33" s="60"/>
       <c r="G33" s="60"/>
@@ -3320,14 +3320,14 @@
       <c r="AZ33" s="13"/>
     </row>
     <row r="34" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="82"/>
-      <c r="B34" s="66" t="s">
+      <c r="A34" s="70"/>
+      <c r="B34" s="65" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="65" t="s">
+      <c r="C34" s="68" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="65" t="s">
+      <c r="D34" s="68" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="11"/>
@@ -3380,10 +3380,10 @@
       <c r="AZ34" s="13"/>
     </row>
     <row r="35" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="82"/>
-      <c r="B35" s="67"/>
-      <c r="C35" s="65"/>
-      <c r="D35" s="65"/>
+      <c r="A35" s="70"/>
+      <c r="B35" s="66"/>
+      <c r="C35" s="68"/>
+      <c r="D35" s="68"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -3434,14 +3434,14 @@
       <c r="AZ35" s="13"/>
     </row>
     <row r="36" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="82"/>
-      <c r="B36" s="66" t="s">
+      <c r="A36" s="70"/>
+      <c r="B36" s="65" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="65">
+      <c r="C36" s="68">
         <v>1.5</v>
       </c>
-      <c r="D36" s="65">
+      <c r="D36" s="68">
         <v>2</v>
       </c>
       <c r="E36" s="11"/>
@@ -3494,10 +3494,10 @@
       <c r="AZ36" s="13"/>
     </row>
     <row r="37" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="82"/>
-      <c r="B37" s="67"/>
-      <c r="C37" s="65"/>
-      <c r="D37" s="65"/>
+      <c r="A37" s="70"/>
+      <c r="B37" s="66"/>
+      <c r="C37" s="68"/>
+      <c r="D37" s="68"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
@@ -3548,14 +3548,14 @@
       <c r="AZ37" s="13"/>
     </row>
     <row r="38" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="82"/>
-      <c r="B38" s="66" t="s">
+      <c r="A38" s="70"/>
+      <c r="B38" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="65">
+      <c r="C38" s="68">
         <v>7</v>
       </c>
-      <c r="D38" s="68">
+      <c r="D38" s="76">
         <v>6</v>
       </c>
       <c r="E38" s="11"/>
@@ -3608,10 +3608,10 @@
       <c r="AZ38" s="13"/>
     </row>
     <row r="39" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="82"/>
-      <c r="B39" s="67"/>
-      <c r="C39" s="65"/>
-      <c r="D39" s="68"/>
+      <c r="A39" s="70"/>
+      <c r="B39" s="66"/>
+      <c r="C39" s="68"/>
+      <c r="D39" s="76"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
@@ -3662,14 +3662,14 @@
       <c r="AZ39" s="13"/>
     </row>
     <row r="40" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="82"/>
-      <c r="B40" s="66" t="s">
+      <c r="A40" s="70"/>
+      <c r="B40" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="65">
+      <c r="C40" s="68">
         <v>6</v>
       </c>
-      <c r="D40" s="68"/>
+      <c r="D40" s="76"/>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
@@ -3720,10 +3720,10 @@
       <c r="AZ40" s="13"/>
     </row>
     <row r="41" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="82"/>
-      <c r="B41" s="67"/>
-      <c r="C41" s="65"/>
-      <c r="D41" s="68"/>
+      <c r="A41" s="70"/>
+      <c r="B41" s="66"/>
+      <c r="C41" s="68"/>
+      <c r="D41" s="76"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
@@ -3774,14 +3774,14 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="82"/>
-      <c r="B42" s="66" t="s">
+      <c r="A42" s="70"/>
+      <c r="B42" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="65">
+      <c r="C42" s="68">
         <v>4</v>
       </c>
-      <c r="D42" s="68">
+      <c r="D42" s="76">
         <v>2</v>
       </c>
       <c r="E42" s="11"/>
@@ -3834,10 +3834,10 @@
       <c r="AZ42" s="13"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A43" s="82"/>
-      <c r="B43" s="67"/>
-      <c r="C43" s="65"/>
-      <c r="D43" s="68"/>
+      <c r="A43" s="70"/>
+      <c r="B43" s="66"/>
+      <c r="C43" s="68"/>
+      <c r="D43" s="76"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
@@ -3859,7 +3859,7 @@
       <c r="W43" s="12"/>
       <c r="X43" s="13"/>
       <c r="Y43" s="11"/>
-      <c r="Z43" s="12"/>
+      <c r="Z43" s="60"/>
       <c r="AA43" s="12"/>
       <c r="AB43" s="13"/>
       <c r="AC43" s="11"/>
@@ -3888,12 +3888,12 @@
       <c r="AZ43" s="13"/>
     </row>
     <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="82"/>
-      <c r="B44" s="66" t="s">
-        <v>47</v>
-      </c>
-      <c r="C44" s="65"/>
-      <c r="D44" s="68"/>
+      <c r="A44" s="70"/>
+      <c r="B44" s="65" t="s">
+        <v>46</v>
+      </c>
+      <c r="C44" s="68"/>
+      <c r="D44" s="76"/>
       <c r="E44" s="11"/>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
@@ -3944,10 +3944,10 @@
       <c r="AZ44" s="13"/>
     </row>
     <row r="45" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="82"/>
-      <c r="B45" s="67"/>
-      <c r="C45" s="65"/>
-      <c r="D45" s="68"/>
+      <c r="A45" s="70"/>
+      <c r="B45" s="66"/>
+      <c r="C45" s="68"/>
+      <c r="D45" s="76"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
@@ -3998,12 +3998,12 @@
       <c r="AZ45" s="13"/>
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A46" s="82"/>
-      <c r="B46" s="66" t="s">
-        <v>48</v>
-      </c>
-      <c r="C46" s="69"/>
-      <c r="D46" s="68"/>
+      <c r="A46" s="70"/>
+      <c r="B46" s="65" t="s">
+        <v>47</v>
+      </c>
+      <c r="C46" s="67"/>
+      <c r="D46" s="76"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -4054,10 +4054,10 @@
       <c r="AZ46" s="13"/>
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A47" s="82"/>
-      <c r="B47" s="67"/>
-      <c r="C47" s="69"/>
-      <c r="D47" s="68"/>
+      <c r="A47" s="70"/>
+      <c r="B47" s="66"/>
+      <c r="C47" s="67"/>
+      <c r="D47" s="76"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -4108,12 +4108,12 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="82"/>
-      <c r="B48" s="66" t="s">
-        <v>49</v>
-      </c>
-      <c r="C48" s="65"/>
-      <c r="D48" s="65"/>
+      <c r="A48" s="70"/>
+      <c r="B48" s="65" t="s">
+        <v>48</v>
+      </c>
+      <c r="C48" s="68"/>
+      <c r="D48" s="68"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4164,10 +4164,10 @@
       <c r="AZ48" s="13"/>
     </row>
     <row r="49" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A49" s="82"/>
-      <c r="B49" s="67"/>
-      <c r="C49" s="65"/>
-      <c r="D49" s="65"/>
+      <c r="A49" s="70"/>
+      <c r="B49" s="66"/>
+      <c r="C49" s="68"/>
+      <c r="D49" s="68"/>
       <c r="E49" s="11"/>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
@@ -4218,10 +4218,12 @@
       <c r="AZ49" s="13"/>
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A50" s="82"/>
-      <c r="B50" s="66"/>
-      <c r="C50" s="65"/>
-      <c r="D50" s="65"/>
+      <c r="A50" s="70"/>
+      <c r="B50" s="65" t="s">
+        <v>49</v>
+      </c>
+      <c r="C50" s="68"/>
+      <c r="D50" s="68"/>
       <c r="E50" s="42"/>
       <c r="F50" s="43"/>
       <c r="G50" s="12"/>
@@ -4272,10 +4274,10 @@
       <c r="AZ50" s="13"/>
     </row>
     <row r="51" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A51" s="82"/>
-      <c r="B51" s="67"/>
-      <c r="C51" s="65"/>
-      <c r="D51" s="65"/>
+      <c r="A51" s="70"/>
+      <c r="B51" s="66"/>
+      <c r="C51" s="68"/>
+      <c r="D51" s="68"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4296,8 +4298,8 @@
       <c r="V51" s="12"/>
       <c r="W51" s="12"/>
       <c r="X51" s="13"/>
-      <c r="Y51" s="11"/>
-      <c r="Z51" s="12"/>
+      <c r="Y51" s="59"/>
+      <c r="Z51" s="60"/>
       <c r="AA51" s="12"/>
       <c r="AB51" s="13"/>
       <c r="AC51" s="11"/>
@@ -4326,15 +4328,15 @@
       <c r="AZ51" s="13"/>
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A52" s="82"/>
-      <c r="B52" s="66" t="s">
+      <c r="A52" s="70"/>
+      <c r="B52" s="65" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="65">
+      <c r="C52" s="68">
         <v>2</v>
       </c>
-      <c r="D52" s="65" t="s">
-        <v>46</v>
+      <c r="D52" s="68" t="s">
+        <v>45</v>
       </c>
       <c r="E52" s="11"/>
       <c r="F52" s="12"/>
@@ -4386,10 +4388,10 @@
       <c r="AZ52" s="13"/>
     </row>
     <row r="53" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A53" s="82"/>
-      <c r="B53" s="67"/>
-      <c r="C53" s="65"/>
-      <c r="D53" s="65"/>
+      <c r="A53" s="70"/>
+      <c r="B53" s="66"/>
+      <c r="C53" s="68"/>
+      <c r="D53" s="68"/>
       <c r="E53" s="11"/>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
@@ -4440,12 +4442,10 @@
       <c r="AZ53" s="13"/>
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A54" s="82"/>
-      <c r="B54" s="66" t="s">
-        <v>44</v>
-      </c>
-      <c r="C54" s="65"/>
-      <c r="D54" s="65"/>
+      <c r="A54" s="70"/>
+      <c r="B54" s="65"/>
+      <c r="C54" s="68"/>
+      <c r="D54" s="68"/>
       <c r="E54" s="11"/>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
@@ -4496,10 +4496,10 @@
       <c r="AZ54" s="13"/>
     </row>
     <row r="55" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A55" s="82"/>
-      <c r="B55" s="67"/>
-      <c r="C55" s="65"/>
-      <c r="D55" s="65"/>
+      <c r="A55" s="70"/>
+      <c r="B55" s="66"/>
+      <c r="C55" s="68"/>
+      <c r="D55" s="68"/>
       <c r="E55" s="11"/>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
@@ -4550,12 +4550,12 @@
       <c r="AZ55" s="13"/>
     </row>
     <row r="56" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="82"/>
-      <c r="B56" s="66" t="s">
-        <v>45</v>
-      </c>
-      <c r="C56" s="69"/>
-      <c r="D56" s="68"/>
+      <c r="A56" s="70"/>
+      <c r="B56" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="C56" s="67"/>
+      <c r="D56" s="76"/>
       <c r="E56" s="11"/>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
@@ -4606,10 +4606,10 @@
       <c r="AZ56" s="13"/>
     </row>
     <row r="57" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="82"/>
-      <c r="B57" s="67"/>
-      <c r="C57" s="65"/>
-      <c r="D57" s="68"/>
+      <c r="A57" s="70"/>
+      <c r="B57" s="66"/>
+      <c r="C57" s="68"/>
+      <c r="D57" s="76"/>
       <c r="E57" s="11"/>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
@@ -4660,12 +4660,12 @@
       <c r="AZ57" s="13"/>
     </row>
     <row r="58" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A58" s="82"/>
-      <c r="B58" s="97" t="s">
+      <c r="A58" s="70"/>
+      <c r="B58" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="C58" s="65"/>
-      <c r="D58" s="68"/>
+      <c r="C58" s="68"/>
+      <c r="D58" s="76"/>
       <c r="E58" s="11"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
@@ -4716,10 +4716,10 @@
       <c r="AZ58" s="13"/>
     </row>
     <row r="59" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A59" s="82"/>
-      <c r="B59" s="97"/>
-      <c r="C59" s="65"/>
-      <c r="D59" s="68"/>
+      <c r="A59" s="70"/>
+      <c r="B59" s="86"/>
+      <c r="C59" s="68"/>
+      <c r="D59" s="76"/>
       <c r="E59" s="11"/>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
@@ -4770,12 +4770,12 @@
       <c r="AZ59" s="13"/>
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A60" s="82"/>
+      <c r="A60" s="70"/>
       <c r="B60" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="C60" s="65"/>
-      <c r="D60" s="68">
+      <c r="C60" s="68"/>
+      <c r="D60" s="76">
         <v>0</v>
       </c>
       <c r="E60" s="11"/>
@@ -4828,10 +4828,10 @@
       <c r="AZ60" s="13"/>
     </row>
     <row r="61" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="82"/>
+      <c r="A61" s="70"/>
       <c r="B61" s="73"/>
-      <c r="C61" s="65"/>
-      <c r="D61" s="68"/>
+      <c r="C61" s="68"/>
+      <c r="D61" s="76"/>
       <c r="E61" s="11"/>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
@@ -4882,14 +4882,14 @@
       <c r="AZ61" s="13"/>
     </row>
     <row r="62" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A62" s="81" t="s">
+      <c r="A62" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="B62" s="98" t="s">
+      <c r="B62" s="72" t="s">
         <v>22</v>
       </c>
-      <c r="C62" s="100"/>
-      <c r="D62" s="101"/>
+      <c r="C62" s="74"/>
+      <c r="D62" s="75"/>
       <c r="E62" s="8"/>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -4940,10 +4940,10 @@
       <c r="AZ62" s="10"/>
     </row>
     <row r="63" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A63" s="82"/>
+      <c r="A63" s="70"/>
       <c r="B63" s="73"/>
-      <c r="C63" s="65"/>
-      <c r="D63" s="68"/>
+      <c r="C63" s="68"/>
+      <c r="D63" s="76"/>
       <c r="E63" s="11"/>
       <c r="F63" s="12"/>
       <c r="G63" s="12"/>
@@ -4994,12 +4994,12 @@
       <c r="AZ63" s="13"/>
     </row>
     <row r="64" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="82"/>
-      <c r="B64" s="66" t="s">
+      <c r="A64" s="70"/>
+      <c r="B64" s="65" t="s">
         <v>23</v>
       </c>
-      <c r="C64" s="69"/>
-      <c r="D64" s="69"/>
+      <c r="C64" s="67"/>
+      <c r="D64" s="67"/>
       <c r="E64" s="11"/>
       <c r="F64" s="12"/>
       <c r="G64" s="12"/>
@@ -5050,10 +5050,10 @@
       <c r="AZ64" s="13"/>
     </row>
     <row r="65" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="82"/>
-      <c r="B65" s="67"/>
-      <c r="C65" s="65"/>
-      <c r="D65" s="65"/>
+      <c r="A65" s="70"/>
+      <c r="B65" s="66"/>
+      <c r="C65" s="68"/>
+      <c r="D65" s="68"/>
       <c r="E65" s="11"/>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
@@ -5104,12 +5104,12 @@
       <c r="AZ65" s="13"/>
     </row>
     <row r="66" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A66" s="82"/>
+      <c r="A66" s="70"/>
       <c r="B66" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="C66" s="65"/>
-      <c r="D66" s="68"/>
+      <c r="C66" s="68"/>
+      <c r="D66" s="76"/>
       <c r="E66" s="11"/>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
@@ -5160,10 +5160,10 @@
       <c r="AZ66" s="13"/>
     </row>
     <row r="67" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="83"/>
-      <c r="B67" s="99"/>
-      <c r="C67" s="94"/>
-      <c r="D67" s="95"/>
+      <c r="A67" s="71"/>
+      <c r="B67" s="77"/>
+      <c r="C67" s="78"/>
+      <c r="D67" s="79"/>
       <c r="E67" s="17"/>
       <c r="F67" s="18"/>
       <c r="G67" s="18"/>
@@ -5214,14 +5214,14 @@
       <c r="AZ67" s="19"/>
     </row>
     <row r="68" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="81" t="s">
+      <c r="A68" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="B68" s="66" t="s">
+      <c r="B68" s="65" t="s">
         <v>25</v>
       </c>
-      <c r="C68" s="69"/>
-      <c r="D68" s="69"/>
+      <c r="C68" s="67"/>
+      <c r="D68" s="67"/>
       <c r="E68" s="11"/>
       <c r="F68" s="12"/>
       <c r="G68" s="12"/>
@@ -5272,10 +5272,10 @@
       <c r="AZ68" s="13"/>
     </row>
     <row r="69" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="82"/>
-      <c r="B69" s="67"/>
-      <c r="C69" s="65"/>
-      <c r="D69" s="65"/>
+      <c r="A69" s="70"/>
+      <c r="B69" s="66"/>
+      <c r="C69" s="68"/>
+      <c r="D69" s="68"/>
       <c r="E69" s="11"/>
       <c r="F69" s="12"/>
       <c r="G69" s="12"/>
@@ -5326,12 +5326,12 @@
       <c r="AZ69" s="13"/>
     </row>
     <row r="70" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="82"/>
-      <c r="B70" s="66" t="s">
+      <c r="A70" s="70"/>
+      <c r="B70" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="C70" s="69"/>
-      <c r="D70" s="69">
+      <c r="C70" s="67"/>
+      <c r="D70" s="67">
         <v>0</v>
       </c>
       <c r="E70" s="11"/>
@@ -5384,10 +5384,10 @@
       <c r="AZ70" s="13"/>
     </row>
     <row r="71" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="83"/>
-      <c r="B71" s="103"/>
-      <c r="C71" s="65"/>
-      <c r="D71" s="65"/>
+      <c r="A71" s="71"/>
+      <c r="B71" s="80"/>
+      <c r="C71" s="68"/>
+      <c r="D71" s="68"/>
       <c r="E71" s="17"/>
       <c r="F71" s="18"/>
       <c r="G71" s="18"/>
@@ -5501,22 +5501,101 @@
     <row r="73" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="135">
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="AS2:AV2"/>
+    <mergeCell ref="AW2:AZ2"/>
+    <mergeCell ref="AS1:AV1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="A8:A17"/>
+    <mergeCell ref="A18:A27"/>
+    <mergeCell ref="AK1:AN1"/>
+    <mergeCell ref="AO1:AR1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="Q1:T1"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="AK2:AN2"/>
+    <mergeCell ref="AO2:AR2"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="U2:X2"/>
+    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A61"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
@@ -5541,101 +5620,22 @@
     <mergeCell ref="C32:C33"/>
     <mergeCell ref="D32:D33"/>
     <mergeCell ref="C34:C35"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AW1:AZ1"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A61"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="AS2:AV2"/>
-    <mergeCell ref="AW2:AZ2"/>
-    <mergeCell ref="AS1:AV1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A8:A17"/>
-    <mergeCell ref="A18:A27"/>
-    <mergeCell ref="AK1:AN1"/>
-    <mergeCell ref="AO1:AR1"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="M1:P1"/>
-    <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="AG2:AJ2"/>
-    <mergeCell ref="AK2:AN2"/>
-    <mergeCell ref="AO2:AR2"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="D70:D71"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Fixing bugs + Security features
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24405420-592F-4DCF-83B5-CDE038A613B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8897C6B-360D-4A89-89FD-88DFF2735E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -166,6 +166,9 @@
     <t>ERM-Diagramm</t>
   </si>
   <si>
+    <t>Actifity Diagramm</t>
+  </si>
+  <si>
     <t>Klassendiagramm</t>
   </si>
   <si>
@@ -179,9 +182,6 @@
   </si>
   <si>
     <t>Projektstruktur verbessern</t>
-  </si>
-  <si>
-    <t>Responsive Design</t>
   </si>
 </sst>
 </file>
@@ -874,85 +874,19 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -964,8 +898,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -975,6 +912,27 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -997,20 +955,62 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -1346,162 +1346,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="B1" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="102" t="s">
+      <c r="C1" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="103"/>
-      <c r="E1" s="92" t="s">
+      <c r="D1" s="89"/>
+      <c r="E1" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="94"/>
-      <c r="I1" s="92" t="s">
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="93"/>
-      <c r="K1" s="93"/>
-      <c r="L1" s="94"/>
-      <c r="M1" s="92" t="s">
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="94"/>
-      <c r="Q1" s="92" t="s">
+      <c r="N1" s="71"/>
+      <c r="O1" s="71"/>
+      <c r="P1" s="72"/>
+      <c r="Q1" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="93"/>
-      <c r="S1" s="93"/>
-      <c r="T1" s="94"/>
-      <c r="U1" s="92" t="s">
+      <c r="R1" s="71"/>
+      <c r="S1" s="71"/>
+      <c r="T1" s="72"/>
+      <c r="U1" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="93"/>
-      <c r="W1" s="93"/>
-      <c r="X1" s="94"/>
-      <c r="Y1" s="92" t="s">
+      <c r="V1" s="71"/>
+      <c r="W1" s="71"/>
+      <c r="X1" s="72"/>
+      <c r="Y1" s="70" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="93"/>
-      <c r="AA1" s="93"/>
-      <c r="AB1" s="94"/>
-      <c r="AC1" s="92" t="s">
+      <c r="Z1" s="71"/>
+      <c r="AA1" s="71"/>
+      <c r="AB1" s="72"/>
+      <c r="AC1" s="70" t="s">
         <v>29</v>
       </c>
-      <c r="AD1" s="93"/>
-      <c r="AE1" s="93"/>
-      <c r="AF1" s="94"/>
-      <c r="AG1" s="92" t="s">
+      <c r="AD1" s="71"/>
+      <c r="AE1" s="71"/>
+      <c r="AF1" s="72"/>
+      <c r="AG1" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="93"/>
-      <c r="AI1" s="93"/>
-      <c r="AJ1" s="94"/>
-      <c r="AK1" s="92" t="s">
+      <c r="AH1" s="71"/>
+      <c r="AI1" s="71"/>
+      <c r="AJ1" s="72"/>
+      <c r="AK1" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="AL1" s="93"/>
-      <c r="AM1" s="93"/>
-      <c r="AN1" s="94"/>
-      <c r="AO1" s="92" t="s">
+      <c r="AL1" s="71"/>
+      <c r="AM1" s="71"/>
+      <c r="AN1" s="72"/>
+      <c r="AO1" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="AP1" s="93"/>
-      <c r="AQ1" s="93"/>
-      <c r="AR1" s="94"/>
-      <c r="AS1" s="92"/>
-      <c r="AT1" s="93"/>
-      <c r="AU1" s="93"/>
-      <c r="AV1" s="94"/>
-      <c r="AW1" s="92"/>
-      <c r="AX1" s="93"/>
-      <c r="AY1" s="93"/>
-      <c r="AZ1" s="94"/>
+      <c r="AP1" s="71"/>
+      <c r="AQ1" s="71"/>
+      <c r="AR1" s="72"/>
+      <c r="AS1" s="70"/>
+      <c r="AT1" s="71"/>
+      <c r="AU1" s="71"/>
+      <c r="AV1" s="72"/>
+      <c r="AW1" s="70"/>
+      <c r="AX1" s="71"/>
+      <c r="AY1" s="71"/>
+      <c r="AZ1" s="72"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="109"/>
-      <c r="B2" s="100"/>
-      <c r="C2" s="104"/>
-      <c r="D2" s="105"/>
-      <c r="E2" s="96">
+      <c r="A2" s="79"/>
+      <c r="B2" s="86"/>
+      <c r="C2" s="90"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="75">
         <v>44781</v>
       </c>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="98"/>
-      <c r="I2" s="96">
+      <c r="F2" s="76"/>
+      <c r="G2" s="76"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="75">
         <v>44782</v>
       </c>
-      <c r="J2" s="97"/>
-      <c r="K2" s="97"/>
-      <c r="L2" s="98"/>
-      <c r="M2" s="96">
+      <c r="J2" s="76"/>
+      <c r="K2" s="76"/>
+      <c r="L2" s="77"/>
+      <c r="M2" s="75">
         <v>44783</v>
       </c>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
-      <c r="P2" s="98"/>
-      <c r="Q2" s="96">
+      <c r="N2" s="76"/>
+      <c r="O2" s="76"/>
+      <c r="P2" s="77"/>
+      <c r="Q2" s="75">
         <v>44784</v>
       </c>
-      <c r="R2" s="97"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="98"/>
-      <c r="U2" s="96">
+      <c r="R2" s="76"/>
+      <c r="S2" s="76"/>
+      <c r="T2" s="77"/>
+      <c r="U2" s="75">
         <v>44785</v>
       </c>
-      <c r="V2" s="97"/>
-      <c r="W2" s="97"/>
-      <c r="X2" s="98"/>
-      <c r="Y2" s="96">
+      <c r="V2" s="76"/>
+      <c r="W2" s="76"/>
+      <c r="X2" s="77"/>
+      <c r="Y2" s="75">
         <v>44789</v>
       </c>
-      <c r="Z2" s="97"/>
-      <c r="AA2" s="97"/>
-      <c r="AB2" s="98"/>
-      <c r="AC2" s="96">
+      <c r="Z2" s="76"/>
+      <c r="AA2" s="76"/>
+      <c r="AB2" s="77"/>
+      <c r="AC2" s="75">
         <v>44790</v>
       </c>
-      <c r="AD2" s="97"/>
-      <c r="AE2" s="97"/>
-      <c r="AF2" s="98"/>
-      <c r="AG2" s="96">
+      <c r="AD2" s="76"/>
+      <c r="AE2" s="76"/>
+      <c r="AF2" s="77"/>
+      <c r="AG2" s="75">
         <v>44791</v>
       </c>
-      <c r="AH2" s="97"/>
-      <c r="AI2" s="97"/>
-      <c r="AJ2" s="98"/>
-      <c r="AK2" s="96">
+      <c r="AH2" s="76"/>
+      <c r="AI2" s="76"/>
+      <c r="AJ2" s="77"/>
+      <c r="AK2" s="75">
         <v>44792</v>
       </c>
-      <c r="AL2" s="97"/>
-      <c r="AM2" s="97"/>
-      <c r="AN2" s="98"/>
-      <c r="AO2" s="96">
+      <c r="AL2" s="76"/>
+      <c r="AM2" s="76"/>
+      <c r="AN2" s="77"/>
+      <c r="AO2" s="75">
         <v>44795</v>
       </c>
-      <c r="AP2" s="97"/>
-      <c r="AQ2" s="97"/>
-      <c r="AR2" s="98"/>
-      <c r="AS2" s="96"/>
-      <c r="AT2" s="97"/>
-      <c r="AU2" s="97"/>
-      <c r="AV2" s="98"/>
-      <c r="AW2" s="96"/>
-      <c r="AX2" s="97"/>
-      <c r="AY2" s="97"/>
-      <c r="AZ2" s="98"/>
+      <c r="AP2" s="76"/>
+      <c r="AQ2" s="76"/>
+      <c r="AR2" s="77"/>
+      <c r="AS2" s="75"/>
+      <c r="AT2" s="76"/>
+      <c r="AU2" s="76"/>
+      <c r="AV2" s="77"/>
+      <c r="AW2" s="75"/>
+      <c r="AX2" s="76"/>
+      <c r="AY2" s="76"/>
+      <c r="AZ2" s="77"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="110"/>
-      <c r="B3" s="101"/>
+      <c r="A3" s="80"/>
+      <c r="B3" s="87"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
@@ -1639,11 +1639,11 @@
     </row>
     <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="66" t="s">
+      <c r="B4" s="67" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="82"/>
-      <c r="D4" s="84"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="105"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1699,9 +1699,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="81"/>
-      <c r="C5" s="83"/>
-      <c r="D5" s="85"/>
+      <c r="B5" s="92"/>
+      <c r="C5" s="84"/>
+      <c r="D5" s="104"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1757,9 +1757,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="86"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="76"/>
+      <c r="B6" s="97"/>
+      <c r="C6" s="65"/>
+      <c r="D6" s="68"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1804,9 +1804,9 @@
     </row>
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="65"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="85"/>
+      <c r="B7" s="66"/>
+      <c r="C7" s="84"/>
+      <c r="D7" s="104"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1861,16 +1861,16 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="69" t="s">
+      <c r="A8" s="81" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="72" t="s">
+      <c r="B8" s="98" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="74">
+      <c r="C8" s="100">
         <v>0.1</v>
       </c>
-      <c r="D8" s="90">
+      <c r="D8" s="109">
         <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
@@ -1927,10 +1927,10 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="70"/>
+      <c r="A9" s="82"/>
       <c r="B9" s="73"/>
-      <c r="C9" s="68"/>
-      <c r="D9" s="91"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="110"/>
       <c r="E9" s="42"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -1981,14 +1981,14 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="70"/>
+      <c r="A10" s="82"/>
       <c r="B10" s="73" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="82">
+      <c r="C10" s="74">
         <v>1</v>
       </c>
-      <c r="D10" s="82">
+      <c r="D10" s="74">
         <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
@@ -2041,10 +2041,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="70"/>
+      <c r="A11" s="82"/>
       <c r="B11" s="73"/>
-      <c r="C11" s="68"/>
-      <c r="D11" s="68"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2095,12 +2095,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="70"/>
+      <c r="A12" s="82"/>
       <c r="B12" s="73" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="82"/>
-      <c r="D12" s="82"/>
+      <c r="C12" s="74"/>
+      <c r="D12" s="74"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2151,10 +2151,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="70"/>
+      <c r="A13" s="82"/>
       <c r="B13" s="73"/>
-      <c r="C13" s="68"/>
-      <c r="D13" s="68"/>
+      <c r="C13" s="65"/>
+      <c r="D13" s="65"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2205,14 +2205,14 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="70"/>
+      <c r="A14" s="82"/>
       <c r="B14" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="82" t="s">
+      <c r="C14" s="74" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="82" t="s">
+      <c r="D14" s="74" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="42"/>
@@ -2265,10 +2265,10 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="70"/>
+      <c r="A15" s="82"/>
       <c r="B15" s="73"/>
-      <c r="C15" s="68"/>
-      <c r="D15" s="68"/>
+      <c r="C15" s="65"/>
+      <c r="D15" s="65"/>
       <c r="E15" s="42"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -2319,14 +2319,14 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="70"/>
-      <c r="B16" s="81" t="s">
+      <c r="A16" s="82"/>
+      <c r="B16" s="92" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="68" t="s">
+      <c r="C16" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="76" t="s">
+      <c r="D16" s="68" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="20"/>
@@ -2379,10 +2379,10 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="71"/>
-      <c r="B17" s="106"/>
-      <c r="C17" s="78"/>
-      <c r="D17" s="79"/>
+      <c r="A17" s="83"/>
+      <c r="B17" s="93"/>
+      <c r="C17" s="94"/>
+      <c r="D17" s="95"/>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
@@ -2433,14 +2433,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="69" t="s">
+      <c r="A18" s="81" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="95" t="s">
+      <c r="B18" s="102" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="74"/>
-      <c r="D18" s="75"/>
+      <c r="C18" s="100"/>
+      <c r="D18" s="101"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2491,10 +2491,10 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="70"/>
-      <c r="B19" s="80"/>
-      <c r="C19" s="68"/>
-      <c r="D19" s="76"/>
+      <c r="A19" s="82"/>
+      <c r="B19" s="103"/>
+      <c r="C19" s="65"/>
+      <c r="D19" s="68"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2545,12 +2545,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="70"/>
+      <c r="A20" s="82"/>
       <c r="B20" s="73" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="68"/>
-      <c r="D20" s="76"/>
+      <c r="C20" s="65"/>
+      <c r="D20" s="68"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2590,10 +2590,10 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="70"/>
+      <c r="A21" s="82"/>
       <c r="B21" s="73"/>
-      <c r="C21" s="68"/>
-      <c r="D21" s="76"/>
+      <c r="C21" s="65"/>
+      <c r="D21" s="68"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2644,14 +2644,14 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="70"/>
+      <c r="A22" s="82"/>
       <c r="B22" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="68">
+      <c r="C22" s="65">
         <v>0.1</v>
       </c>
-      <c r="D22" s="76">
+      <c r="D22" s="68">
         <v>0.1</v>
       </c>
       <c r="E22" s="11"/>
@@ -2704,10 +2704,10 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="70"/>
+      <c r="A23" s="82"/>
       <c r="B23" s="73"/>
-      <c r="C23" s="68"/>
-      <c r="D23" s="76"/>
+      <c r="C23" s="65"/>
+      <c r="D23" s="68"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2758,10 +2758,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="70"/>
-      <c r="B24" s="81"/>
-      <c r="C24" s="83"/>
-      <c r="D24" s="87"/>
+      <c r="A24" s="82"/>
+      <c r="B24" s="92"/>
+      <c r="C24" s="84"/>
+      <c r="D24" s="106"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2812,10 +2812,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="70"/>
-      <c r="B25" s="66"/>
-      <c r="C25" s="82"/>
-      <c r="D25" s="88"/>
+      <c r="A25" s="82"/>
+      <c r="B25" s="67"/>
+      <c r="C25" s="74"/>
+      <c r="D25" s="107"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2866,12 +2866,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="70"/>
+      <c r="A26" s="82"/>
       <c r="B26" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="83"/>
-      <c r="D26" s="87">
+      <c r="C26" s="84"/>
+      <c r="D26" s="106">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2924,10 +2924,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="71"/>
+      <c r="A27" s="83"/>
       <c r="B27" s="73"/>
-      <c r="C27" s="107"/>
-      <c r="D27" s="89"/>
+      <c r="C27" s="96"/>
+      <c r="D27" s="108"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2978,14 +2978,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="69" t="s">
+      <c r="A28" s="81" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="72" t="s">
+      <c r="B28" s="98" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="74"/>
-      <c r="D28" s="75"/>
+      <c r="C28" s="100"/>
+      <c r="D28" s="101"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -3036,10 +3036,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="70"/>
-      <c r="B29" s="77"/>
-      <c r="C29" s="78"/>
-      <c r="D29" s="79"/>
+      <c r="A29" s="82"/>
+      <c r="B29" s="99"/>
+      <c r="C29" s="94"/>
+      <c r="D29" s="95"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3090,16 +3090,16 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="69" t="s">
+      <c r="A30" s="81" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="72" t="s">
+      <c r="B30" s="98" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="74">
+      <c r="C30" s="100">
         <v>2</v>
       </c>
-      <c r="D30" s="75">
+      <c r="D30" s="101">
         <v>2</v>
       </c>
       <c r="E30" s="53"/>
@@ -3152,10 +3152,10 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="70"/>
+      <c r="A31" s="82"/>
       <c r="B31" s="73"/>
-      <c r="C31" s="68"/>
-      <c r="D31" s="76"/>
+      <c r="C31" s="65"/>
+      <c r="D31" s="68"/>
       <c r="E31" s="59"/>
       <c r="F31" s="60"/>
       <c r="G31" s="43"/>
@@ -3206,14 +3206,14 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="70"/>
-      <c r="B32" s="65" t="s">
+      <c r="A32" s="82"/>
+      <c r="B32" s="66" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="68">
+      <c r="C32" s="65">
         <v>4</v>
       </c>
-      <c r="D32" s="68">
+      <c r="D32" s="65">
         <v>7</v>
       </c>
       <c r="E32" s="11"/>
@@ -3266,10 +3266,10 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="70"/>
-      <c r="B33" s="66"/>
-      <c r="C33" s="68"/>
-      <c r="D33" s="68"/>
+      <c r="A33" s="82"/>
+      <c r="B33" s="67"/>
+      <c r="C33" s="65"/>
+      <c r="D33" s="65"/>
       <c r="E33" s="11"/>
       <c r="F33" s="60"/>
       <c r="G33" s="60"/>
@@ -3320,14 +3320,14 @@
       <c r="AZ33" s="13"/>
     </row>
     <row r="34" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="70"/>
-      <c r="B34" s="65" t="s">
+      <c r="A34" s="82"/>
+      <c r="B34" s="66" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="68" t="s">
+      <c r="C34" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="68" t="s">
+      <c r="D34" s="65" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="11"/>
@@ -3380,10 +3380,10 @@
       <c r="AZ34" s="13"/>
     </row>
     <row r="35" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="70"/>
-      <c r="B35" s="66"/>
-      <c r="C35" s="68"/>
-      <c r="D35" s="68"/>
+      <c r="A35" s="82"/>
+      <c r="B35" s="67"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -3434,14 +3434,14 @@
       <c r="AZ35" s="13"/>
     </row>
     <row r="36" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="70"/>
-      <c r="B36" s="65" t="s">
+      <c r="A36" s="82"/>
+      <c r="B36" s="66" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="68">
+      <c r="C36" s="65">
         <v>1.5</v>
       </c>
-      <c r="D36" s="68">
+      <c r="D36" s="65">
         <v>2</v>
       </c>
       <c r="E36" s="11"/>
@@ -3494,10 +3494,10 @@
       <c r="AZ36" s="13"/>
     </row>
     <row r="37" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="70"/>
-      <c r="B37" s="66"/>
-      <c r="C37" s="68"/>
-      <c r="D37" s="68"/>
+      <c r="A37" s="82"/>
+      <c r="B37" s="67"/>
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
@@ -3548,14 +3548,14 @@
       <c r="AZ37" s="13"/>
     </row>
     <row r="38" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="70"/>
-      <c r="B38" s="65" t="s">
+      <c r="A38" s="82"/>
+      <c r="B38" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="68">
+      <c r="C38" s="65">
         <v>7</v>
       </c>
-      <c r="D38" s="76">
+      <c r="D38" s="68">
         <v>6</v>
       </c>
       <c r="E38" s="11"/>
@@ -3608,10 +3608,10 @@
       <c r="AZ38" s="13"/>
     </row>
     <row r="39" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="70"/>
-      <c r="B39" s="66"/>
-      <c r="C39" s="68"/>
-      <c r="D39" s="76"/>
+      <c r="A39" s="82"/>
+      <c r="B39" s="67"/>
+      <c r="C39" s="65"/>
+      <c r="D39" s="68"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
@@ -3662,14 +3662,14 @@
       <c r="AZ39" s="13"/>
     </row>
     <row r="40" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="70"/>
-      <c r="B40" s="65" t="s">
+      <c r="A40" s="82"/>
+      <c r="B40" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="68">
+      <c r="C40" s="65">
         <v>6</v>
       </c>
-      <c r="D40" s="76"/>
+      <c r="D40" s="68"/>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
@@ -3720,10 +3720,10 @@
       <c r="AZ40" s="13"/>
     </row>
     <row r="41" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="70"/>
-      <c r="B41" s="66"/>
-      <c r="C41" s="68"/>
-      <c r="D41" s="76"/>
+      <c r="A41" s="82"/>
+      <c r="B41" s="67"/>
+      <c r="C41" s="65"/>
+      <c r="D41" s="68"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
@@ -3774,14 +3774,14 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="70"/>
-      <c r="B42" s="65" t="s">
+      <c r="A42" s="82"/>
+      <c r="B42" s="66" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="68">
+      <c r="C42" s="65">
         <v>4</v>
       </c>
-      <c r="D42" s="76">
+      <c r="D42" s="68">
         <v>2</v>
       </c>
       <c r="E42" s="11"/>
@@ -3834,10 +3834,10 @@
       <c r="AZ42" s="13"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A43" s="70"/>
-      <c r="B43" s="66"/>
-      <c r="C43" s="68"/>
-      <c r="D43" s="76"/>
+      <c r="A43" s="82"/>
+      <c r="B43" s="67"/>
+      <c r="C43" s="65"/>
+      <c r="D43" s="68"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
@@ -3859,7 +3859,7 @@
       <c r="W43" s="12"/>
       <c r="X43" s="13"/>
       <c r="Y43" s="11"/>
-      <c r="Z43" s="60"/>
+      <c r="Z43" s="12"/>
       <c r="AA43" s="12"/>
       <c r="AB43" s="13"/>
       <c r="AC43" s="11"/>
@@ -3888,12 +3888,12 @@
       <c r="AZ43" s="13"/>
     </row>
     <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="70"/>
-      <c r="B44" s="65" t="s">
-        <v>46</v>
-      </c>
-      <c r="C44" s="68"/>
-      <c r="D44" s="76"/>
+      <c r="A44" s="82"/>
+      <c r="B44" s="66" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="65"/>
+      <c r="D44" s="68"/>
       <c r="E44" s="11"/>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
@@ -3944,10 +3944,10 @@
       <c r="AZ44" s="13"/>
     </row>
     <row r="45" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="70"/>
-      <c r="B45" s="66"/>
-      <c r="C45" s="68"/>
-      <c r="D45" s="76"/>
+      <c r="A45" s="82"/>
+      <c r="B45" s="67"/>
+      <c r="C45" s="65"/>
+      <c r="D45" s="68"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
@@ -3998,12 +3998,12 @@
       <c r="AZ45" s="13"/>
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A46" s="70"/>
-      <c r="B46" s="65" t="s">
-        <v>47</v>
-      </c>
-      <c r="C46" s="67"/>
-      <c r="D46" s="76"/>
+      <c r="A46" s="82"/>
+      <c r="B46" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="C46" s="69"/>
+      <c r="D46" s="68"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -4054,10 +4054,10 @@
       <c r="AZ46" s="13"/>
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A47" s="70"/>
-      <c r="B47" s="66"/>
-      <c r="C47" s="67"/>
-      <c r="D47" s="76"/>
+      <c r="A47" s="82"/>
+      <c r="B47" s="67"/>
+      <c r="C47" s="69"/>
+      <c r="D47" s="68"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -4108,12 +4108,12 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="70"/>
-      <c r="B48" s="65" t="s">
-        <v>48</v>
-      </c>
-      <c r="C48" s="68"/>
-      <c r="D48" s="68"/>
+      <c r="A48" s="82"/>
+      <c r="B48" s="66" t="s">
+        <v>49</v>
+      </c>
+      <c r="C48" s="65"/>
+      <c r="D48" s="65"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4164,10 +4164,10 @@
       <c r="AZ48" s="13"/>
     </row>
     <row r="49" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A49" s="70"/>
-      <c r="B49" s="66"/>
-      <c r="C49" s="68"/>
-      <c r="D49" s="68"/>
+      <c r="A49" s="82"/>
+      <c r="B49" s="67"/>
+      <c r="C49" s="65"/>
+      <c r="D49" s="65"/>
       <c r="E49" s="11"/>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
@@ -4218,12 +4218,10 @@
       <c r="AZ49" s="13"/>
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A50" s="70"/>
-      <c r="B50" s="65" t="s">
-        <v>49</v>
-      </c>
-      <c r="C50" s="68"/>
-      <c r="D50" s="68"/>
+      <c r="A50" s="82"/>
+      <c r="B50" s="66"/>
+      <c r="C50" s="65"/>
+      <c r="D50" s="65"/>
       <c r="E50" s="42"/>
       <c r="F50" s="43"/>
       <c r="G50" s="12"/>
@@ -4274,10 +4272,10 @@
       <c r="AZ50" s="13"/>
     </row>
     <row r="51" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A51" s="70"/>
-      <c r="B51" s="66"/>
-      <c r="C51" s="68"/>
-      <c r="D51" s="68"/>
+      <c r="A51" s="82"/>
+      <c r="B51" s="67"/>
+      <c r="C51" s="65"/>
+      <c r="D51" s="65"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4298,8 +4296,8 @@
       <c r="V51" s="12"/>
       <c r="W51" s="12"/>
       <c r="X51" s="13"/>
-      <c r="Y51" s="59"/>
-      <c r="Z51" s="60"/>
+      <c r="Y51" s="11"/>
+      <c r="Z51" s="12"/>
       <c r="AA51" s="12"/>
       <c r="AB51" s="13"/>
       <c r="AC51" s="11"/>
@@ -4328,15 +4326,15 @@
       <c r="AZ51" s="13"/>
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A52" s="70"/>
-      <c r="B52" s="65" t="s">
+      <c r="A52" s="82"/>
+      <c r="B52" s="66" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="68">
+      <c r="C52" s="65">
         <v>2</v>
       </c>
-      <c r="D52" s="68" t="s">
-        <v>45</v>
+      <c r="D52" s="65" t="s">
+        <v>46</v>
       </c>
       <c r="E52" s="11"/>
       <c r="F52" s="12"/>
@@ -4388,10 +4386,10 @@
       <c r="AZ52" s="13"/>
     </row>
     <row r="53" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A53" s="70"/>
-      <c r="B53" s="66"/>
-      <c r="C53" s="68"/>
-      <c r="D53" s="68"/>
+      <c r="A53" s="82"/>
+      <c r="B53" s="67"/>
+      <c r="C53" s="65"/>
+      <c r="D53" s="65"/>
       <c r="E53" s="11"/>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
@@ -4442,10 +4440,12 @@
       <c r="AZ53" s="13"/>
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A54" s="70"/>
-      <c r="B54" s="65"/>
-      <c r="C54" s="68"/>
-      <c r="D54" s="68"/>
+      <c r="A54" s="82"/>
+      <c r="B54" s="66" t="s">
+        <v>44</v>
+      </c>
+      <c r="C54" s="65"/>
+      <c r="D54" s="65"/>
       <c r="E54" s="11"/>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
@@ -4496,10 +4496,10 @@
       <c r="AZ54" s="13"/>
     </row>
     <row r="55" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A55" s="70"/>
-      <c r="B55" s="66"/>
-      <c r="C55" s="68"/>
-      <c r="D55" s="68"/>
+      <c r="A55" s="82"/>
+      <c r="B55" s="67"/>
+      <c r="C55" s="65"/>
+      <c r="D55" s="65"/>
       <c r="E55" s="11"/>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
@@ -4550,12 +4550,12 @@
       <c r="AZ55" s="13"/>
     </row>
     <row r="56" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="70"/>
-      <c r="B56" s="65" t="s">
-        <v>44</v>
-      </c>
-      <c r="C56" s="67"/>
-      <c r="D56" s="76"/>
+      <c r="A56" s="82"/>
+      <c r="B56" s="66" t="s">
+        <v>45</v>
+      </c>
+      <c r="C56" s="69"/>
+      <c r="D56" s="68"/>
       <c r="E56" s="11"/>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
@@ -4606,10 +4606,10 @@
       <c r="AZ56" s="13"/>
     </row>
     <row r="57" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="70"/>
-      <c r="B57" s="66"/>
-      <c r="C57" s="68"/>
-      <c r="D57" s="76"/>
+      <c r="A57" s="82"/>
+      <c r="B57" s="67"/>
+      <c r="C57" s="65"/>
+      <c r="D57" s="68"/>
       <c r="E57" s="11"/>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
@@ -4660,12 +4660,12 @@
       <c r="AZ57" s="13"/>
     </row>
     <row r="58" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A58" s="70"/>
-      <c r="B58" s="86" t="s">
+      <c r="A58" s="82"/>
+      <c r="B58" s="97" t="s">
         <v>26</v>
       </c>
-      <c r="C58" s="68"/>
-      <c r="D58" s="76"/>
+      <c r="C58" s="65"/>
+      <c r="D58" s="68"/>
       <c r="E58" s="11"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
@@ -4716,10 +4716,10 @@
       <c r="AZ58" s="13"/>
     </row>
     <row r="59" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A59" s="70"/>
-      <c r="B59" s="86"/>
-      <c r="C59" s="68"/>
-      <c r="D59" s="76"/>
+      <c r="A59" s="82"/>
+      <c r="B59" s="97"/>
+      <c r="C59" s="65"/>
+      <c r="D59" s="68"/>
       <c r="E59" s="11"/>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
@@ -4770,12 +4770,12 @@
       <c r="AZ59" s="13"/>
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A60" s="70"/>
+      <c r="A60" s="82"/>
       <c r="B60" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="C60" s="68"/>
-      <c r="D60" s="76">
+      <c r="C60" s="65"/>
+      <c r="D60" s="68">
         <v>0</v>
       </c>
       <c r="E60" s="11"/>
@@ -4828,10 +4828,10 @@
       <c r="AZ60" s="13"/>
     </row>
     <row r="61" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="70"/>
+      <c r="A61" s="82"/>
       <c r="B61" s="73"/>
-      <c r="C61" s="68"/>
-      <c r="D61" s="76"/>
+      <c r="C61" s="65"/>
+      <c r="D61" s="68"/>
       <c r="E61" s="11"/>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
@@ -4882,14 +4882,14 @@
       <c r="AZ61" s="13"/>
     </row>
     <row r="62" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A62" s="69" t="s">
+      <c r="A62" s="81" t="s">
         <v>14</v>
       </c>
-      <c r="B62" s="72" t="s">
+      <c r="B62" s="98" t="s">
         <v>22</v>
       </c>
-      <c r="C62" s="74"/>
-      <c r="D62" s="75"/>
+      <c r="C62" s="100"/>
+      <c r="D62" s="101"/>
       <c r="E62" s="8"/>
       <c r="F62" s="9"/>
       <c r="G62" s="9"/>
@@ -4940,10 +4940,10 @@
       <c r="AZ62" s="10"/>
     </row>
     <row r="63" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A63" s="70"/>
+      <c r="A63" s="82"/>
       <c r="B63" s="73"/>
-      <c r="C63" s="68"/>
-      <c r="D63" s="76"/>
+      <c r="C63" s="65"/>
+      <c r="D63" s="68"/>
       <c r="E63" s="11"/>
       <c r="F63" s="12"/>
       <c r="G63" s="12"/>
@@ -4994,12 +4994,12 @@
       <c r="AZ63" s="13"/>
     </row>
     <row r="64" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="70"/>
-      <c r="B64" s="65" t="s">
+      <c r="A64" s="82"/>
+      <c r="B64" s="66" t="s">
         <v>23</v>
       </c>
-      <c r="C64" s="67"/>
-      <c r="D64" s="67"/>
+      <c r="C64" s="69"/>
+      <c r="D64" s="69"/>
       <c r="E64" s="11"/>
       <c r="F64" s="12"/>
       <c r="G64" s="12"/>
@@ -5050,10 +5050,10 @@
       <c r="AZ64" s="13"/>
     </row>
     <row r="65" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="70"/>
-      <c r="B65" s="66"/>
-      <c r="C65" s="68"/>
-      <c r="D65" s="68"/>
+      <c r="A65" s="82"/>
+      <c r="B65" s="67"/>
+      <c r="C65" s="65"/>
+      <c r="D65" s="65"/>
       <c r="E65" s="11"/>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
@@ -5104,12 +5104,12 @@
       <c r="AZ65" s="13"/>
     </row>
     <row r="66" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A66" s="70"/>
+      <c r="A66" s="82"/>
       <c r="B66" s="73" t="s">
         <v>24</v>
       </c>
-      <c r="C66" s="68"/>
-      <c r="D66" s="76"/>
+      <c r="C66" s="65"/>
+      <c r="D66" s="68"/>
       <c r="E66" s="11"/>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
@@ -5160,10 +5160,10 @@
       <c r="AZ66" s="13"/>
     </row>
     <row r="67" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="71"/>
-      <c r="B67" s="77"/>
-      <c r="C67" s="78"/>
-      <c r="D67" s="79"/>
+      <c r="A67" s="83"/>
+      <c r="B67" s="99"/>
+      <c r="C67" s="94"/>
+      <c r="D67" s="95"/>
       <c r="E67" s="17"/>
       <c r="F67" s="18"/>
       <c r="G67" s="18"/>
@@ -5214,14 +5214,14 @@
       <c r="AZ67" s="19"/>
     </row>
     <row r="68" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="69" t="s">
+      <c r="A68" s="81" t="s">
         <v>15</v>
       </c>
-      <c r="B68" s="65" t="s">
+      <c r="B68" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="C68" s="67"/>
-      <c r="D68" s="67"/>
+      <c r="C68" s="69"/>
+      <c r="D68" s="69"/>
       <c r="E68" s="11"/>
       <c r="F68" s="12"/>
       <c r="G68" s="12"/>
@@ -5272,10 +5272,10 @@
       <c r="AZ68" s="13"/>
     </row>
     <row r="69" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="70"/>
-      <c r="B69" s="66"/>
-      <c r="C69" s="68"/>
-      <c r="D69" s="68"/>
+      <c r="A69" s="82"/>
+      <c r="B69" s="67"/>
+      <c r="C69" s="65"/>
+      <c r="D69" s="65"/>
       <c r="E69" s="11"/>
       <c r="F69" s="12"/>
       <c r="G69" s="12"/>
@@ -5326,12 +5326,12 @@
       <c r="AZ69" s="13"/>
     </row>
     <row r="70" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="70"/>
-      <c r="B70" s="65" t="s">
+      <c r="A70" s="82"/>
+      <c r="B70" s="66" t="s">
         <v>7</v>
       </c>
-      <c r="C70" s="67"/>
-      <c r="D70" s="67">
+      <c r="C70" s="69"/>
+      <c r="D70" s="69">
         <v>0</v>
       </c>
       <c r="E70" s="11"/>
@@ -5384,10 +5384,10 @@
       <c r="AZ70" s="13"/>
     </row>
     <row r="71" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="71"/>
-      <c r="B71" s="80"/>
-      <c r="C71" s="68"/>
-      <c r="D71" s="68"/>
+      <c r="A71" s="83"/>
+      <c r="B71" s="103"/>
+      <c r="C71" s="65"/>
+      <c r="D71" s="65"/>
       <c r="E71" s="17"/>
       <c r="F71" s="18"/>
       <c r="G71" s="18"/>
@@ -5501,29 +5501,94 @@
     <row r="73" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="135">
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A61"/>
+    <mergeCell ref="A62:A67"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="C60:C61"/>
     <mergeCell ref="U1:X1"/>
     <mergeCell ref="D46:D47"/>
     <mergeCell ref="B10:B11"/>
@@ -5548,94 +5613,29 @@
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="U2:X2"/>
     <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A61"/>
-    <mergeCell ref="A62:A67"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AW1:AZ1"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C46:C47"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Code Refactoring + Kommentare
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8897C6B-360D-4A89-89FD-88DFF2735E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22313717-F9EA-4B9B-834D-A7FD9B2102C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -166,9 +166,6 @@
     <t>ERM-Diagramm</t>
   </si>
   <si>
-    <t>Actifity Diagramm</t>
-  </si>
-  <si>
     <t>Klassendiagramm</t>
   </si>
   <si>
@@ -182,6 +179,9 @@
   </si>
   <si>
     <t>Projektstruktur verbessern</t>
+  </si>
+  <si>
+    <t>Responsive Design</t>
   </si>
 </sst>
 </file>
@@ -794,7 +794,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1012,6 +1012,7 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -3858,11 +3859,11 @@
       <c r="V43" s="12"/>
       <c r="W43" s="12"/>
       <c r="X43" s="13"/>
-      <c r="Y43" s="11"/>
+      <c r="Y43" s="59"/>
       <c r="Z43" s="12"/>
       <c r="AA43" s="12"/>
       <c r="AB43" s="13"/>
-      <c r="AC43" s="11"/>
+      <c r="AC43" s="111"/>
       <c r="AD43" s="12"/>
       <c r="AE43" s="12"/>
       <c r="AF43" s="13"/>
@@ -3890,7 +3891,7 @@
     <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="82"/>
       <c r="B44" s="66" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C44" s="65"/>
       <c r="D44" s="68"/>
@@ -3969,11 +3970,11 @@
       <c r="W45" s="12"/>
       <c r="X45" s="13"/>
       <c r="Y45" s="11"/>
-      <c r="Z45" s="12"/>
-      <c r="AA45" s="12"/>
-      <c r="AB45" s="13"/>
-      <c r="AC45" s="11"/>
-      <c r="AD45" s="12"/>
+      <c r="Z45" s="60"/>
+      <c r="AA45" s="60"/>
+      <c r="AB45" s="61"/>
+      <c r="AC45" s="59"/>
+      <c r="AD45" s="60"/>
       <c r="AE45" s="12"/>
       <c r="AF45" s="13"/>
       <c r="AG45" s="11"/>
@@ -4000,7 +4001,7 @@
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A46" s="82"/>
       <c r="B46" s="66" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C46" s="69"/>
       <c r="D46" s="68"/>
@@ -4110,7 +4111,7 @@
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A48" s="82"/>
       <c r="B48" s="66" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C48" s="65"/>
       <c r="D48" s="65"/>
@@ -4219,7 +4220,9 @@
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A50" s="82"/>
-      <c r="B50" s="66"/>
+      <c r="B50" s="66" t="s">
+        <v>49</v>
+      </c>
       <c r="C50" s="65"/>
       <c r="D50" s="65"/>
       <c r="E50" s="42"/>
@@ -4296,11 +4299,11 @@
       <c r="V51" s="12"/>
       <c r="W51" s="12"/>
       <c r="X51" s="13"/>
-      <c r="Y51" s="11"/>
-      <c r="Z51" s="12"/>
+      <c r="Y51" s="59"/>
+      <c r="Z51" s="60"/>
       <c r="AA51" s="12"/>
       <c r="AB51" s="13"/>
-      <c r="AC51" s="11"/>
+      <c r="AC51" s="111"/>
       <c r="AD51" s="12"/>
       <c r="AE51" s="12"/>
       <c r="AF51" s="13"/>
@@ -4334,7 +4337,7 @@
         <v>2</v>
       </c>
       <c r="D52" s="65" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E52" s="11"/>
       <c r="F52" s="12"/>
@@ -4441,9 +4444,7 @@
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A54" s="82"/>
-      <c r="B54" s="66" t="s">
-        <v>44</v>
-      </c>
+      <c r="B54" s="66"/>
       <c r="C54" s="65"/>
       <c r="D54" s="65"/>
       <c r="E54" s="11"/>
@@ -4552,7 +4553,7 @@
     <row r="56" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="82"/>
       <c r="B56" s="66" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C56" s="69"/>
       <c r="D56" s="68"/>

</xml_diff>

<commit_message>
Quellen hinzugefügt + Abbildungsverzeichnis
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007C2338-24BF-47C4-AFBC-9164A7B22DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BDB46E-8EC3-4DA2-A809-2746C3D569DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -881,71 +881,13 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -953,13 +895,19 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -971,8 +919,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -982,6 +930,24 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1004,23 +970,57 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -1355,162 +1355,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="100" t="s">
+      <c r="B1" s="90" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="103" t="s">
+      <c r="C1" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="104"/>
-      <c r="E1" s="93" t="s">
+      <c r="D1" s="94"/>
+      <c r="E1" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="94"/>
-      <c r="G1" s="94"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="93" t="s">
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="79"/>
+      <c r="I1" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="94"/>
-      <c r="K1" s="94"/>
-      <c r="L1" s="95"/>
-      <c r="M1" s="93" t="s">
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="79"/>
+      <c r="M1" s="77" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="94"/>
-      <c r="O1" s="94"/>
-      <c r="P1" s="95"/>
-      <c r="Q1" s="93" t="s">
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="79"/>
+      <c r="Q1" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="94"/>
-      <c r="S1" s="94"/>
-      <c r="T1" s="95"/>
-      <c r="U1" s="93" t="s">
+      <c r="R1" s="78"/>
+      <c r="S1" s="78"/>
+      <c r="T1" s="79"/>
+      <c r="U1" s="77" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="94"/>
-      <c r="W1" s="94"/>
-      <c r="X1" s="95"/>
-      <c r="Y1" s="93" t="s">
+      <c r="V1" s="78"/>
+      <c r="W1" s="78"/>
+      <c r="X1" s="79"/>
+      <c r="Y1" s="77" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="94"/>
-      <c r="AA1" s="94"/>
-      <c r="AB1" s="95"/>
-      <c r="AC1" s="93" t="s">
+      <c r="Z1" s="78"/>
+      <c r="AA1" s="78"/>
+      <c r="AB1" s="79"/>
+      <c r="AC1" s="77" t="s">
         <v>29</v>
       </c>
-      <c r="AD1" s="94"/>
-      <c r="AE1" s="94"/>
-      <c r="AF1" s="95"/>
-      <c r="AG1" s="93" t="s">
+      <c r="AD1" s="78"/>
+      <c r="AE1" s="78"/>
+      <c r="AF1" s="79"/>
+      <c r="AG1" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="94"/>
-      <c r="AI1" s="94"/>
-      <c r="AJ1" s="95"/>
-      <c r="AK1" s="93" t="s">
+      <c r="AH1" s="78"/>
+      <c r="AI1" s="78"/>
+      <c r="AJ1" s="79"/>
+      <c r="AK1" s="77" t="s">
         <v>31</v>
       </c>
-      <c r="AL1" s="94"/>
-      <c r="AM1" s="94"/>
-      <c r="AN1" s="95"/>
-      <c r="AO1" s="93" t="s">
+      <c r="AL1" s="78"/>
+      <c r="AM1" s="78"/>
+      <c r="AN1" s="79"/>
+      <c r="AO1" s="77" t="s">
         <v>27</v>
       </c>
-      <c r="AP1" s="94"/>
-      <c r="AQ1" s="94"/>
-      <c r="AR1" s="95"/>
-      <c r="AS1" s="93"/>
-      <c r="AT1" s="94"/>
-      <c r="AU1" s="94"/>
-      <c r="AV1" s="95"/>
-      <c r="AW1" s="93"/>
-      <c r="AX1" s="94"/>
-      <c r="AY1" s="94"/>
-      <c r="AZ1" s="95"/>
+      <c r="AP1" s="78"/>
+      <c r="AQ1" s="78"/>
+      <c r="AR1" s="79"/>
+      <c r="AS1" s="77"/>
+      <c r="AT1" s="78"/>
+      <c r="AU1" s="78"/>
+      <c r="AV1" s="79"/>
+      <c r="AW1" s="77"/>
+      <c r="AX1" s="78"/>
+      <c r="AY1" s="78"/>
+      <c r="AZ1" s="79"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="110"/>
-      <c r="B2" s="101"/>
-      <c r="C2" s="105"/>
-      <c r="D2" s="106"/>
-      <c r="E2" s="97">
+      <c r="A2" s="85"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="95"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="81">
         <v>44781</v>
       </c>
-      <c r="F2" s="98"/>
-      <c r="G2" s="98"/>
-      <c r="H2" s="99"/>
-      <c r="I2" s="97">
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="83"/>
+      <c r="I2" s="81">
         <v>44782</v>
       </c>
-      <c r="J2" s="98"/>
-      <c r="K2" s="98"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="97">
+      <c r="J2" s="82"/>
+      <c r="K2" s="82"/>
+      <c r="L2" s="83"/>
+      <c r="M2" s="81">
         <v>44783</v>
       </c>
-      <c r="N2" s="98"/>
-      <c r="O2" s="98"/>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="97">
+      <c r="N2" s="82"/>
+      <c r="O2" s="82"/>
+      <c r="P2" s="83"/>
+      <c r="Q2" s="81">
         <v>44784</v>
       </c>
-      <c r="R2" s="98"/>
-      <c r="S2" s="98"/>
-      <c r="T2" s="99"/>
-      <c r="U2" s="97">
+      <c r="R2" s="82"/>
+      <c r="S2" s="82"/>
+      <c r="T2" s="83"/>
+      <c r="U2" s="81">
         <v>44785</v>
       </c>
-      <c r="V2" s="98"/>
-      <c r="W2" s="98"/>
-      <c r="X2" s="99"/>
-      <c r="Y2" s="97">
+      <c r="V2" s="82"/>
+      <c r="W2" s="82"/>
+      <c r="X2" s="83"/>
+      <c r="Y2" s="81">
         <v>44789</v>
       </c>
-      <c r="Z2" s="98"/>
-      <c r="AA2" s="98"/>
-      <c r="AB2" s="99"/>
-      <c r="AC2" s="97">
+      <c r="Z2" s="82"/>
+      <c r="AA2" s="82"/>
+      <c r="AB2" s="83"/>
+      <c r="AC2" s="81">
         <v>44790</v>
       </c>
-      <c r="AD2" s="98"/>
-      <c r="AE2" s="98"/>
-      <c r="AF2" s="99"/>
-      <c r="AG2" s="97">
+      <c r="AD2" s="82"/>
+      <c r="AE2" s="82"/>
+      <c r="AF2" s="83"/>
+      <c r="AG2" s="81">
         <v>44791</v>
       </c>
-      <c r="AH2" s="98"/>
-      <c r="AI2" s="98"/>
-      <c r="AJ2" s="99"/>
-      <c r="AK2" s="97">
+      <c r="AH2" s="82"/>
+      <c r="AI2" s="82"/>
+      <c r="AJ2" s="83"/>
+      <c r="AK2" s="81">
         <v>44792</v>
       </c>
-      <c r="AL2" s="98"/>
-      <c r="AM2" s="98"/>
-      <c r="AN2" s="99"/>
-      <c r="AO2" s="97">
+      <c r="AL2" s="82"/>
+      <c r="AM2" s="82"/>
+      <c r="AN2" s="83"/>
+      <c r="AO2" s="81">
         <v>44795</v>
       </c>
-      <c r="AP2" s="98"/>
-      <c r="AQ2" s="98"/>
-      <c r="AR2" s="99"/>
-      <c r="AS2" s="97"/>
-      <c r="AT2" s="98"/>
-      <c r="AU2" s="98"/>
-      <c r="AV2" s="99"/>
-      <c r="AW2" s="97"/>
-      <c r="AX2" s="98"/>
-      <c r="AY2" s="98"/>
-      <c r="AZ2" s="99"/>
+      <c r="AP2" s="82"/>
+      <c r="AQ2" s="82"/>
+      <c r="AR2" s="83"/>
+      <c r="AS2" s="81"/>
+      <c r="AT2" s="82"/>
+      <c r="AU2" s="82"/>
+      <c r="AV2" s="83"/>
+      <c r="AW2" s="81"/>
+      <c r="AX2" s="82"/>
+      <c r="AY2" s="82"/>
+      <c r="AZ2" s="83"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="111"/>
-      <c r="B3" s="102"/>
+      <c r="A3" s="86"/>
+      <c r="B3" s="92"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
@@ -1648,11 +1648,11 @@
     </row>
     <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="67" t="s">
+      <c r="B4" s="74" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="83"/>
-      <c r="D4" s="85"/>
+      <c r="C4" s="69"/>
+      <c r="D4" s="110"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1708,9 +1708,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="82"/>
-      <c r="C5" s="84"/>
-      <c r="D5" s="86"/>
+      <c r="B5" s="97"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="109"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1766,9 +1766,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="87"/>
-      <c r="C6" s="69"/>
-      <c r="D6" s="77"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="72"/>
+      <c r="D6" s="75"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1813,9 +1813,9 @@
     </row>
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="66"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="86"/>
+      <c r="B7" s="73"/>
+      <c r="C7" s="68"/>
+      <c r="D7" s="109"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1870,16 +1870,16 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="70" t="s">
+      <c r="A8" s="87" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="73" t="s">
+      <c r="B8" s="103" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="75">
+      <c r="C8" s="105">
         <v>0.1</v>
       </c>
-      <c r="D8" s="91">
+      <c r="D8" s="112">
         <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
@@ -1936,10 +1936,10 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="71"/>
-      <c r="B9" s="74"/>
-      <c r="C9" s="69"/>
-      <c r="D9" s="92"/>
+      <c r="A9" s="88"/>
+      <c r="B9" s="80"/>
+      <c r="C9" s="72"/>
+      <c r="D9" s="113"/>
       <c r="E9" s="42"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -1990,14 +1990,14 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="71"/>
-      <c r="B10" s="74" t="s">
+      <c r="A10" s="88"/>
+      <c r="B10" s="80" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="83">
+      <c r="C10" s="69">
         <v>1</v>
       </c>
-      <c r="D10" s="83">
+      <c r="D10" s="69">
         <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
@@ -2050,10 +2050,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="71"/>
-      <c r="B11" s="74"/>
-      <c r="C11" s="69"/>
-      <c r="D11" s="69"/>
+      <c r="A11" s="88"/>
+      <c r="B11" s="80"/>
+      <c r="C11" s="72"/>
+      <c r="D11" s="72"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2104,12 +2104,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="71"/>
-      <c r="B12" s="74" t="s">
+      <c r="A12" s="88"/>
+      <c r="B12" s="80" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="83"/>
-      <c r="D12" s="83"/>
+      <c r="C12" s="69"/>
+      <c r="D12" s="69"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2160,10 +2160,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="71"/>
-      <c r="B13" s="74"/>
-      <c r="C13" s="69"/>
-      <c r="D13" s="69"/>
+      <c r="A13" s="88"/>
+      <c r="B13" s="80"/>
+      <c r="C13" s="72"/>
+      <c r="D13" s="72"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2214,14 +2214,14 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="71"/>
-      <c r="B14" s="74" t="s">
+      <c r="A14" s="88"/>
+      <c r="B14" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="83" t="s">
+      <c r="C14" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="83" t="s">
+      <c r="D14" s="69" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="42"/>
@@ -2274,10 +2274,10 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="71"/>
-      <c r="B15" s="74"/>
-      <c r="C15" s="69"/>
-      <c r="D15" s="69"/>
+      <c r="A15" s="88"/>
+      <c r="B15" s="80"/>
+      <c r="C15" s="72"/>
+      <c r="D15" s="72"/>
       <c r="E15" s="42"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -2328,14 +2328,14 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="71"/>
-      <c r="B16" s="82" t="s">
+      <c r="A16" s="88"/>
+      <c r="B16" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="69" t="s">
+      <c r="C16" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="77" t="s">
+      <c r="D16" s="75" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="20"/>
@@ -2388,10 +2388,10 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="72"/>
-      <c r="B17" s="107"/>
-      <c r="C17" s="79"/>
-      <c r="D17" s="80"/>
+      <c r="A17" s="89"/>
+      <c r="B17" s="98"/>
+      <c r="C17" s="99"/>
+      <c r="D17" s="100"/>
       <c r="E17" s="17"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
@@ -2442,14 +2442,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="70" t="s">
+      <c r="A18" s="87" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="96" t="s">
+      <c r="B18" s="107" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="75"/>
-      <c r="D18" s="76"/>
+      <c r="C18" s="105"/>
+      <c r="D18" s="106"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2500,10 +2500,10 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="71"/>
-      <c r="B19" s="81"/>
-      <c r="C19" s="69"/>
-      <c r="D19" s="77"/>
+      <c r="A19" s="88"/>
+      <c r="B19" s="108"/>
+      <c r="C19" s="72"/>
+      <c r="D19" s="75"/>
       <c r="E19" s="11"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2554,12 +2554,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="71"/>
-      <c r="B20" s="74" t="s">
+      <c r="A20" s="88"/>
+      <c r="B20" s="80" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="69"/>
-      <c r="D20" s="77"/>
+      <c r="C20" s="72"/>
+      <c r="D20" s="75"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2599,10 +2599,10 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="71"/>
-      <c r="B21" s="74"/>
-      <c r="C21" s="69"/>
-      <c r="D21" s="77"/>
+      <c r="A21" s="88"/>
+      <c r="B21" s="80"/>
+      <c r="C21" s="72"/>
+      <c r="D21" s="75"/>
       <c r="E21" s="11"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2653,14 +2653,14 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="71"/>
-      <c r="B22" s="74" t="s">
+      <c r="A22" s="88"/>
+      <c r="B22" s="80" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="69">
+      <c r="C22" s="72">
         <v>0.1</v>
       </c>
-      <c r="D22" s="77">
+      <c r="D22" s="75">
         <v>0.1</v>
       </c>
       <c r="E22" s="11"/>
@@ -2713,10 +2713,10 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="71"/>
-      <c r="B23" s="74"/>
-      <c r="C23" s="69"/>
-      <c r="D23" s="77"/>
+      <c r="A23" s="88"/>
+      <c r="B23" s="80"/>
+      <c r="C23" s="72"/>
+      <c r="D23" s="75"/>
       <c r="E23" s="11"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2767,10 +2767,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="71"/>
-      <c r="B24" s="82"/>
-      <c r="C24" s="84"/>
-      <c r="D24" s="88"/>
+      <c r="A24" s="88"/>
+      <c r="B24" s="97"/>
+      <c r="C24" s="68"/>
+      <c r="D24" s="70"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2821,10 +2821,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="71"/>
-      <c r="B25" s="67"/>
-      <c r="C25" s="83"/>
-      <c r="D25" s="89"/>
+      <c r="A25" s="88"/>
+      <c r="B25" s="74"/>
+      <c r="C25" s="69"/>
+      <c r="D25" s="71"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2875,12 +2875,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="71"/>
-      <c r="B26" s="74" t="s">
+      <c r="A26" s="88"/>
+      <c r="B26" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="84"/>
-      <c r="D26" s="88">
+      <c r="C26" s="68"/>
+      <c r="D26" s="70">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2933,10 +2933,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="72"/>
-      <c r="B27" s="74"/>
-      <c r="C27" s="108"/>
-      <c r="D27" s="90"/>
+      <c r="A27" s="89"/>
+      <c r="B27" s="80"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="111"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2987,14 +2987,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="70" t="s">
+      <c r="A28" s="87" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="73" t="s">
+      <c r="B28" s="103" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="75"/>
-      <c r="D28" s="76"/>
+      <c r="C28" s="105"/>
+      <c r="D28" s="106"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -3045,10 +3045,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="71"/>
-      <c r="B29" s="78"/>
-      <c r="C29" s="79"/>
-      <c r="D29" s="80"/>
+      <c r="A29" s="88"/>
+      <c r="B29" s="104"/>
+      <c r="C29" s="99"/>
+      <c r="D29" s="100"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3099,16 +3099,16 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="70" t="s">
+      <c r="A30" s="87" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="73" t="s">
+      <c r="B30" s="103" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="75">
+      <c r="C30" s="105">
         <v>2</v>
       </c>
-      <c r="D30" s="76">
+      <c r="D30" s="106">
         <v>2</v>
       </c>
       <c r="E30" s="53"/>
@@ -3161,10 +3161,10 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="71"/>
-      <c r="B31" s="74"/>
-      <c r="C31" s="69"/>
-      <c r="D31" s="77"/>
+      <c r="A31" s="88"/>
+      <c r="B31" s="80"/>
+      <c r="C31" s="72"/>
+      <c r="D31" s="75"/>
       <c r="E31" s="59"/>
       <c r="F31" s="60"/>
       <c r="G31" s="43"/>
@@ -3215,14 +3215,14 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="71"/>
-      <c r="B32" s="66" t="s">
+      <c r="A32" s="88"/>
+      <c r="B32" s="73" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="69">
+      <c r="C32" s="72">
         <v>4</v>
       </c>
-      <c r="D32" s="69">
+      <c r="D32" s="72">
         <v>7</v>
       </c>
       <c r="E32" s="11"/>
@@ -3275,10 +3275,10 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="71"/>
-      <c r="B33" s="67"/>
-      <c r="C33" s="69"/>
-      <c r="D33" s="69"/>
+      <c r="A33" s="88"/>
+      <c r="B33" s="74"/>
+      <c r="C33" s="72"/>
+      <c r="D33" s="72"/>
       <c r="E33" s="11"/>
       <c r="F33" s="60"/>
       <c r="G33" s="60"/>
@@ -3329,14 +3329,14 @@
       <c r="AZ33" s="13"/>
     </row>
     <row r="34" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="71"/>
-      <c r="B34" s="66" t="s">
+      <c r="A34" s="88"/>
+      <c r="B34" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="69" t="s">
+      <c r="C34" s="72" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="69" t="s">
+      <c r="D34" s="72" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="11"/>
@@ -3389,10 +3389,10 @@
       <c r="AZ34" s="13"/>
     </row>
     <row r="35" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="71"/>
-      <c r="B35" s="67"/>
-      <c r="C35" s="69"/>
-      <c r="D35" s="69"/>
+      <c r="A35" s="88"/>
+      <c r="B35" s="74"/>
+      <c r="C35" s="72"/>
+      <c r="D35" s="72"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -3443,14 +3443,14 @@
       <c r="AZ35" s="13"/>
     </row>
     <row r="36" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="71"/>
-      <c r="B36" s="66" t="s">
+      <c r="A36" s="88"/>
+      <c r="B36" s="73" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="69">
+      <c r="C36" s="72">
         <v>1.5</v>
       </c>
-      <c r="D36" s="69">
+      <c r="D36" s="72">
         <v>2</v>
       </c>
       <c r="E36" s="11"/>
@@ -3503,10 +3503,10 @@
       <c r="AZ36" s="13"/>
     </row>
     <row r="37" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="71"/>
-      <c r="B37" s="67"/>
-      <c r="C37" s="69"/>
-      <c r="D37" s="69"/>
+      <c r="A37" s="88"/>
+      <c r="B37" s="74"/>
+      <c r="C37" s="72"/>
+      <c r="D37" s="72"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
@@ -3557,14 +3557,14 @@
       <c r="AZ37" s="13"/>
     </row>
     <row r="38" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="71"/>
-      <c r="B38" s="66" t="s">
+      <c r="A38" s="88"/>
+      <c r="B38" s="73" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="69">
+      <c r="C38" s="72">
         <v>7</v>
       </c>
-      <c r="D38" s="77">
+      <c r="D38" s="75">
         <v>6</v>
       </c>
       <c r="E38" s="11"/>
@@ -3617,10 +3617,10 @@
       <c r="AZ38" s="13"/>
     </row>
     <row r="39" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="71"/>
-      <c r="B39" s="67"/>
-      <c r="C39" s="69"/>
-      <c r="D39" s="77"/>
+      <c r="A39" s="88"/>
+      <c r="B39" s="74"/>
+      <c r="C39" s="72"/>
+      <c r="D39" s="75"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
@@ -3671,14 +3671,14 @@
       <c r="AZ39" s="13"/>
     </row>
     <row r="40" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="71"/>
-      <c r="B40" s="66" t="s">
+      <c r="A40" s="88"/>
+      <c r="B40" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="69">
+      <c r="C40" s="72">
         <v>6</v>
       </c>
-      <c r="D40" s="77"/>
+      <c r="D40" s="75"/>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
@@ -3729,10 +3729,10 @@
       <c r="AZ40" s="13"/>
     </row>
     <row r="41" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="71"/>
-      <c r="B41" s="67"/>
-      <c r="C41" s="69"/>
-      <c r="D41" s="77"/>
+      <c r="A41" s="88"/>
+      <c r="B41" s="74"/>
+      <c r="C41" s="72"/>
+      <c r="D41" s="75"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
@@ -3783,14 +3783,14 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="71"/>
-      <c r="B42" s="66" t="s">
+      <c r="A42" s="88"/>
+      <c r="B42" s="73" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="69">
+      <c r="C42" s="72">
         <v>4</v>
       </c>
-      <c r="D42" s="77">
+      <c r="D42" s="75">
         <v>2</v>
       </c>
       <c r="E42" s="11"/>
@@ -3843,10 +3843,10 @@
       <c r="AZ42" s="13"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A43" s="71"/>
-      <c r="B43" s="67"/>
-      <c r="C43" s="69"/>
-      <c r="D43" s="77"/>
+      <c r="A43" s="88"/>
+      <c r="B43" s="74"/>
+      <c r="C43" s="72"/>
+      <c r="D43" s="75"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
@@ -3897,12 +3897,12 @@
       <c r="AZ43" s="13"/>
     </row>
     <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="71"/>
-      <c r="B44" s="66" t="s">
+      <c r="A44" s="88"/>
+      <c r="B44" s="73" t="s">
         <v>46</v>
       </c>
-      <c r="C44" s="69"/>
-      <c r="D44" s="77"/>
+      <c r="C44" s="72"/>
+      <c r="D44" s="75"/>
       <c r="E44" s="11"/>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
@@ -3953,10 +3953,10 @@
       <c r="AZ44" s="13"/>
     </row>
     <row r="45" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="71"/>
-      <c r="B45" s="67"/>
-      <c r="C45" s="69"/>
-      <c r="D45" s="77"/>
+      <c r="A45" s="88"/>
+      <c r="B45" s="74"/>
+      <c r="C45" s="72"/>
+      <c r="D45" s="75"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
@@ -4007,12 +4007,12 @@
       <c r="AZ45" s="13"/>
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A46" s="71"/>
-      <c r="B46" s="66" t="s">
+      <c r="A46" s="88"/>
+      <c r="B46" s="73" t="s">
         <v>47</v>
       </c>
-      <c r="C46" s="68"/>
-      <c r="D46" s="77"/>
+      <c r="C46" s="76"/>
+      <c r="D46" s="75"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -4063,10 +4063,10 @@
       <c r="AZ46" s="13"/>
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A47" s="71"/>
-      <c r="B47" s="67"/>
-      <c r="C47" s="68"/>
-      <c r="D47" s="77"/>
+      <c r="A47" s="88"/>
+      <c r="B47" s="74"/>
+      <c r="C47" s="76"/>
+      <c r="D47" s="75"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -4117,12 +4117,12 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="71"/>
-      <c r="B48" s="66" t="s">
+      <c r="A48" s="88"/>
+      <c r="B48" s="73" t="s">
         <v>48</v>
       </c>
-      <c r="C48" s="69"/>
-      <c r="D48" s="69"/>
+      <c r="C48" s="72"/>
+      <c r="D48" s="72"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4173,10 +4173,10 @@
       <c r="AZ48" s="13"/>
     </row>
     <row r="49" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A49" s="71"/>
-      <c r="B49" s="67"/>
-      <c r="C49" s="69"/>
-      <c r="D49" s="69"/>
+      <c r="A49" s="88"/>
+      <c r="B49" s="74"/>
+      <c r="C49" s="72"/>
+      <c r="D49" s="72"/>
       <c r="E49" s="11"/>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
@@ -4227,12 +4227,12 @@
       <c r="AZ49" s="13"/>
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A50" s="71"/>
-      <c r="B50" s="66" t="s">
+      <c r="A50" s="88"/>
+      <c r="B50" s="73" t="s">
         <v>49</v>
       </c>
-      <c r="C50" s="69"/>
-      <c r="D50" s="69"/>
+      <c r="C50" s="72"/>
+      <c r="D50" s="72"/>
       <c r="E50" s="42"/>
       <c r="F50" s="43"/>
       <c r="G50" s="12"/>
@@ -4283,10 +4283,10 @@
       <c r="AZ50" s="13"/>
     </row>
     <row r="51" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A51" s="71"/>
-      <c r="B51" s="67"/>
-      <c r="C51" s="69"/>
-      <c r="D51" s="69"/>
+      <c r="A51" s="88"/>
+      <c r="B51" s="74"/>
+      <c r="C51" s="72"/>
+      <c r="D51" s="72"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4337,14 +4337,14 @@
       <c r="AZ51" s="13"/>
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A52" s="71"/>
-      <c r="B52" s="66" t="s">
+      <c r="A52" s="88"/>
+      <c r="B52" s="73" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="69">
+      <c r="C52" s="72">
         <v>2</v>
       </c>
-      <c r="D52" s="69" t="s">
+      <c r="D52" s="72" t="s">
         <v>45</v>
       </c>
       <c r="E52" s="11"/>
@@ -4397,10 +4397,10 @@
       <c r="AZ52" s="13"/>
     </row>
     <row r="53" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A53" s="71"/>
-      <c r="B53" s="67"/>
-      <c r="C53" s="69"/>
-      <c r="D53" s="69"/>
+      <c r="A53" s="88"/>
+      <c r="B53" s="74"/>
+      <c r="C53" s="72"/>
+      <c r="D53" s="72"/>
       <c r="E53" s="11"/>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
@@ -4451,12 +4451,12 @@
       <c r="AZ53" s="13"/>
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A54" s="71"/>
-      <c r="B54" s="66" t="s">
+      <c r="A54" s="88"/>
+      <c r="B54" s="73" t="s">
         <v>50</v>
       </c>
-      <c r="C54" s="84"/>
-      <c r="D54" s="88"/>
+      <c r="C54" s="68"/>
+      <c r="D54" s="70"/>
       <c r="E54" s="11"/>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
@@ -4507,10 +4507,10 @@
       <c r="AZ54" s="13"/>
     </row>
     <row r="55" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A55" s="71"/>
-      <c r="B55" s="67"/>
-      <c r="C55" s="83"/>
-      <c r="D55" s="89"/>
+      <c r="A55" s="88"/>
+      <c r="B55" s="74"/>
+      <c r="C55" s="69"/>
+      <c r="D55" s="71"/>
       <c r="E55" s="11"/>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
@@ -4541,8 +4541,8 @@
       <c r="AF55" s="13"/>
       <c r="AG55" s="59"/>
       <c r="AH55" s="60"/>
-      <c r="AI55" s="12"/>
-      <c r="AJ55" s="13"/>
+      <c r="AI55" s="60"/>
+      <c r="AJ55" s="61"/>
       <c r="AK55" s="11"/>
       <c r="AL55" s="12"/>
       <c r="AM55" s="12"/>
@@ -4561,12 +4561,12 @@
       <c r="AZ55" s="13"/>
     </row>
     <row r="56" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A56" s="71"/>
-      <c r="B56" s="66" t="s">
+      <c r="A56" s="88"/>
+      <c r="B56" s="73" t="s">
         <v>51</v>
       </c>
-      <c r="C56" s="69"/>
-      <c r="D56" s="69"/>
+      <c r="C56" s="72"/>
+      <c r="D56" s="72"/>
       <c r="E56" s="11"/>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
@@ -4617,10 +4617,10 @@
       <c r="AZ56" s="13"/>
     </row>
     <row r="57" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A57" s="71"/>
-      <c r="B57" s="67"/>
-      <c r="C57" s="69"/>
-      <c r="D57" s="69"/>
+      <c r="A57" s="88"/>
+      <c r="B57" s="74"/>
+      <c r="C57" s="72"/>
+      <c r="D57" s="72"/>
       <c r="E57" s="11"/>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
@@ -4671,12 +4671,12 @@
       <c r="AZ57" s="13"/>
     </row>
     <row r="58" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="71"/>
-      <c r="B58" s="66" t="s">
+      <c r="A58" s="88"/>
+      <c r="B58" s="73" t="s">
         <v>44</v>
       </c>
-      <c r="C58" s="68"/>
-      <c r="D58" s="77"/>
+      <c r="C58" s="76"/>
+      <c r="D58" s="75"/>
       <c r="E58" s="11"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
@@ -4727,10 +4727,10 @@
       <c r="AZ58" s="13"/>
     </row>
     <row r="59" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="71"/>
-      <c r="B59" s="67"/>
-      <c r="C59" s="69"/>
-      <c r="D59" s="77"/>
+      <c r="A59" s="88"/>
+      <c r="B59" s="74"/>
+      <c r="C59" s="72"/>
+      <c r="D59" s="75"/>
       <c r="E59" s="11"/>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
@@ -4781,12 +4781,12 @@
       <c r="AZ59" s="13"/>
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A60" s="71"/>
-      <c r="B60" s="87" t="s">
+      <c r="A60" s="88"/>
+      <c r="B60" s="102" t="s">
         <v>26</v>
       </c>
-      <c r="C60" s="69"/>
-      <c r="D60" s="77"/>
+      <c r="C60" s="72"/>
+      <c r="D60" s="75"/>
       <c r="E60" s="11"/>
       <c r="F60" s="12"/>
       <c r="G60" s="12"/>
@@ -4837,10 +4837,10 @@
       <c r="AZ60" s="13"/>
     </row>
     <row r="61" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A61" s="71"/>
-      <c r="B61" s="87"/>
-      <c r="C61" s="69"/>
-      <c r="D61" s="77"/>
+      <c r="A61" s="88"/>
+      <c r="B61" s="102"/>
+      <c r="C61" s="72"/>
+      <c r="D61" s="75"/>
       <c r="E61" s="11"/>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
@@ -4891,12 +4891,12 @@
       <c r="AZ61" s="13"/>
     </row>
     <row r="62" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A62" s="71"/>
-      <c r="B62" s="74" t="s">
+      <c r="A62" s="88"/>
+      <c r="B62" s="80" t="s">
         <v>7</v>
       </c>
-      <c r="C62" s="69"/>
-      <c r="D62" s="77">
+      <c r="C62" s="72"/>
+      <c r="D62" s="75">
         <v>0</v>
       </c>
       <c r="E62" s="11"/>
@@ -4949,10 +4949,10 @@
       <c r="AZ62" s="13"/>
     </row>
     <row r="63" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="71"/>
-      <c r="B63" s="74"/>
-      <c r="C63" s="69"/>
-      <c r="D63" s="77"/>
+      <c r="A63" s="88"/>
+      <c r="B63" s="80"/>
+      <c r="C63" s="72"/>
+      <c r="D63" s="75"/>
       <c r="E63" s="11"/>
       <c r="F63" s="12"/>
       <c r="G63" s="12"/>
@@ -5003,14 +5003,14 @@
       <c r="AZ63" s="13"/>
     </row>
     <row r="64" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A64" s="70" t="s">
+      <c r="A64" s="87" t="s">
         <v>14</v>
       </c>
-      <c r="B64" s="73" t="s">
+      <c r="B64" s="103" t="s">
         <v>22</v>
       </c>
-      <c r="C64" s="75"/>
-      <c r="D64" s="76"/>
+      <c r="C64" s="105"/>
+      <c r="D64" s="106"/>
       <c r="E64" s="8"/>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -5061,10 +5061,10 @@
       <c r="AZ64" s="10"/>
     </row>
     <row r="65" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A65" s="71"/>
-      <c r="B65" s="74"/>
-      <c r="C65" s="69"/>
-      <c r="D65" s="77"/>
+      <c r="A65" s="88"/>
+      <c r="B65" s="80"/>
+      <c r="C65" s="72"/>
+      <c r="D65" s="75"/>
       <c r="E65" s="11"/>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
@@ -5115,12 +5115,12 @@
       <c r="AZ65" s="13"/>
     </row>
     <row r="66" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="71"/>
-      <c r="B66" s="66" t="s">
+      <c r="A66" s="88"/>
+      <c r="B66" s="73" t="s">
         <v>23</v>
       </c>
-      <c r="C66" s="68"/>
-      <c r="D66" s="68"/>
+      <c r="C66" s="76"/>
+      <c r="D66" s="76"/>
       <c r="E66" s="11"/>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
@@ -5171,10 +5171,10 @@
       <c r="AZ66" s="13"/>
     </row>
     <row r="67" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="71"/>
-      <c r="B67" s="67"/>
-      <c r="C67" s="69"/>
-      <c r="D67" s="69"/>
+      <c r="A67" s="88"/>
+      <c r="B67" s="74"/>
+      <c r="C67" s="72"/>
+      <c r="D67" s="72"/>
       <c r="E67" s="11"/>
       <c r="F67" s="12"/>
       <c r="G67" s="12"/>
@@ -5225,12 +5225,12 @@
       <c r="AZ67" s="13"/>
     </row>
     <row r="68" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A68" s="71"/>
-      <c r="B68" s="74" t="s">
+      <c r="A68" s="88"/>
+      <c r="B68" s="80" t="s">
         <v>24</v>
       </c>
-      <c r="C68" s="69"/>
-      <c r="D68" s="77"/>
+      <c r="C68" s="72"/>
+      <c r="D68" s="75"/>
       <c r="E68" s="11"/>
       <c r="F68" s="12"/>
       <c r="G68" s="12"/>
@@ -5281,10 +5281,10 @@
       <c r="AZ68" s="13"/>
     </row>
     <row r="69" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="72"/>
-      <c r="B69" s="78"/>
-      <c r="C69" s="79"/>
-      <c r="D69" s="80"/>
+      <c r="A69" s="89"/>
+      <c r="B69" s="104"/>
+      <c r="C69" s="99"/>
+      <c r="D69" s="100"/>
       <c r="E69" s="17"/>
       <c r="F69" s="18"/>
       <c r="G69" s="18"/>
@@ -5319,8 +5319,8 @@
       <c r="AJ69" s="19"/>
       <c r="AK69" s="17"/>
       <c r="AL69" s="18"/>
-      <c r="AM69" s="112"/>
-      <c r="AN69" s="113"/>
+      <c r="AM69" s="66"/>
+      <c r="AN69" s="67"/>
       <c r="AO69" s="17"/>
       <c r="AP69" s="18"/>
       <c r="AQ69" s="18"/>
@@ -5335,14 +5335,14 @@
       <c r="AZ69" s="19"/>
     </row>
     <row r="70" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="70" t="s">
+      <c r="A70" s="87" t="s">
         <v>15</v>
       </c>
-      <c r="B70" s="66" t="s">
+      <c r="B70" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="C70" s="68"/>
-      <c r="D70" s="68"/>
+      <c r="C70" s="76"/>
+      <c r="D70" s="76"/>
       <c r="E70" s="11"/>
       <c r="F70" s="12"/>
       <c r="G70" s="12"/>
@@ -5393,10 +5393,10 @@
       <c r="AZ70" s="13"/>
     </row>
     <row r="71" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="71"/>
-      <c r="B71" s="67"/>
-      <c r="C71" s="69"/>
-      <c r="D71" s="69"/>
+      <c r="A71" s="88"/>
+      <c r="B71" s="74"/>
+      <c r="C71" s="72"/>
+      <c r="D71" s="72"/>
       <c r="E71" s="11"/>
       <c r="F71" s="12"/>
       <c r="G71" s="12"/>
@@ -5447,12 +5447,12 @@
       <c r="AZ71" s="13"/>
     </row>
     <row r="72" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="71"/>
-      <c r="B72" s="66" t="s">
+      <c r="A72" s="88"/>
+      <c r="B72" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="C72" s="68"/>
-      <c r="D72" s="68">
+      <c r="C72" s="76"/>
+      <c r="D72" s="76">
         <v>0</v>
       </c>
       <c r="E72" s="11"/>
@@ -5505,10 +5505,10 @@
       <c r="AZ72" s="13"/>
     </row>
     <row r="73" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="72"/>
-      <c r="B73" s="81"/>
-      <c r="C73" s="69"/>
-      <c r="D73" s="69"/>
+      <c r="A73" s="89"/>
+      <c r="B73" s="108"/>
+      <c r="C73" s="72"/>
+      <c r="D73" s="72"/>
       <c r="E73" s="17"/>
       <c r="F73" s="18"/>
       <c r="G73" s="18"/>
@@ -5622,32 +5622,94 @@
     <row r="75" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="138">
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="D52:D53"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="C72:C73"/>
+    <mergeCell ref="D72:D73"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A63"/>
+    <mergeCell ref="A64:A69"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="C62:C63"/>
     <mergeCell ref="U1:X1"/>
     <mergeCell ref="D46:D47"/>
     <mergeCell ref="B10:B11"/>
@@ -5672,94 +5734,32 @@
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="U2:X2"/>
     <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A63"/>
-    <mergeCell ref="A64:A69"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AW1:AZ1"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="D70:D71"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="C72:C73"/>
-    <mergeCell ref="D72:D73"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="D52:D53"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
VIPs können eigene Bilder löschen und bearbeiten
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BDB46E-8EC3-4DA2-A809-2746C3D569DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E37E85-F071-4310-ADDF-65BC44DA3350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -800,7 +800,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -868,7 +868,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -883,11 +882,71 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -895,19 +954,13 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -919,8 +972,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -930,24 +983,6 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -970,57 +1005,23 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -1355,162 +1356,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="110" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="90" t="s">
+      <c r="B1" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="93" t="s">
+      <c r="C1" s="104" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="94"/>
-      <c r="E1" s="77" t="s">
+      <c r="D1" s="105"/>
+      <c r="E1" s="94" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="77" t="s">
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="96"/>
+      <c r="I1" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="79"/>
-      <c r="M1" s="77" t="s">
+      <c r="J1" s="95"/>
+      <c r="K1" s="95"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="94" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="78"/>
-      <c r="O1" s="78"/>
-      <c r="P1" s="79"/>
-      <c r="Q1" s="77" t="s">
+      <c r="N1" s="95"/>
+      <c r="O1" s="95"/>
+      <c r="P1" s="96"/>
+      <c r="Q1" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="78"/>
-      <c r="S1" s="78"/>
-      <c r="T1" s="79"/>
-      <c r="U1" s="77" t="s">
+      <c r="R1" s="95"/>
+      <c r="S1" s="95"/>
+      <c r="T1" s="96"/>
+      <c r="U1" s="94" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="78"/>
-      <c r="W1" s="78"/>
-      <c r="X1" s="79"/>
-      <c r="Y1" s="77" t="s">
+      <c r="V1" s="95"/>
+      <c r="W1" s="95"/>
+      <c r="X1" s="96"/>
+      <c r="Y1" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="78"/>
-      <c r="AA1" s="78"/>
-      <c r="AB1" s="79"/>
-      <c r="AC1" s="77" t="s">
+      <c r="Z1" s="95"/>
+      <c r="AA1" s="95"/>
+      <c r="AB1" s="96"/>
+      <c r="AC1" s="94" t="s">
         <v>29</v>
       </c>
-      <c r="AD1" s="78"/>
-      <c r="AE1" s="78"/>
-      <c r="AF1" s="79"/>
-      <c r="AG1" s="77" t="s">
+      <c r="AD1" s="95"/>
+      <c r="AE1" s="95"/>
+      <c r="AF1" s="96"/>
+      <c r="AG1" s="94" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="78"/>
-      <c r="AI1" s="78"/>
-      <c r="AJ1" s="79"/>
-      <c r="AK1" s="77" t="s">
+      <c r="AH1" s="95"/>
+      <c r="AI1" s="95"/>
+      <c r="AJ1" s="96"/>
+      <c r="AK1" s="94" t="s">
         <v>31</v>
       </c>
-      <c r="AL1" s="78"/>
-      <c r="AM1" s="78"/>
-      <c r="AN1" s="79"/>
-      <c r="AO1" s="77" t="s">
+      <c r="AL1" s="95"/>
+      <c r="AM1" s="95"/>
+      <c r="AN1" s="96"/>
+      <c r="AO1" s="94" t="s">
         <v>27</v>
       </c>
-      <c r="AP1" s="78"/>
-      <c r="AQ1" s="78"/>
-      <c r="AR1" s="79"/>
-      <c r="AS1" s="77"/>
-      <c r="AT1" s="78"/>
-      <c r="AU1" s="78"/>
-      <c r="AV1" s="79"/>
-      <c r="AW1" s="77"/>
-      <c r="AX1" s="78"/>
-      <c r="AY1" s="78"/>
-      <c r="AZ1" s="79"/>
+      <c r="AP1" s="95"/>
+      <c r="AQ1" s="95"/>
+      <c r="AR1" s="96"/>
+      <c r="AS1" s="94"/>
+      <c r="AT1" s="95"/>
+      <c r="AU1" s="95"/>
+      <c r="AV1" s="96"/>
+      <c r="AW1" s="94"/>
+      <c r="AX1" s="95"/>
+      <c r="AY1" s="95"/>
+      <c r="AZ1" s="96"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="85"/>
-      <c r="B2" s="91"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="81">
+      <c r="A2" s="111"/>
+      <c r="B2" s="102"/>
+      <c r="C2" s="106"/>
+      <c r="D2" s="107"/>
+      <c r="E2" s="98">
         <v>44781</v>
       </c>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="83"/>
-      <c r="I2" s="81">
+      <c r="F2" s="99"/>
+      <c r="G2" s="99"/>
+      <c r="H2" s="100"/>
+      <c r="I2" s="98">
         <v>44782</v>
       </c>
-      <c r="J2" s="82"/>
-      <c r="K2" s="82"/>
-      <c r="L2" s="83"/>
-      <c r="M2" s="81">
+      <c r="J2" s="99"/>
+      <c r="K2" s="99"/>
+      <c r="L2" s="100"/>
+      <c r="M2" s="98">
         <v>44783</v>
       </c>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
-      <c r="P2" s="83"/>
-      <c r="Q2" s="81">
+      <c r="N2" s="99"/>
+      <c r="O2" s="99"/>
+      <c r="P2" s="100"/>
+      <c r="Q2" s="98">
         <v>44784</v>
       </c>
-      <c r="R2" s="82"/>
-      <c r="S2" s="82"/>
-      <c r="T2" s="83"/>
-      <c r="U2" s="81">
+      <c r="R2" s="99"/>
+      <c r="S2" s="99"/>
+      <c r="T2" s="100"/>
+      <c r="U2" s="98">
         <v>44785</v>
       </c>
-      <c r="V2" s="82"/>
-      <c r="W2" s="82"/>
-      <c r="X2" s="83"/>
-      <c r="Y2" s="81">
+      <c r="V2" s="99"/>
+      <c r="W2" s="99"/>
+      <c r="X2" s="100"/>
+      <c r="Y2" s="98">
         <v>44789</v>
       </c>
-      <c r="Z2" s="82"/>
-      <c r="AA2" s="82"/>
-      <c r="AB2" s="83"/>
-      <c r="AC2" s="81">
+      <c r="Z2" s="99"/>
+      <c r="AA2" s="99"/>
+      <c r="AB2" s="100"/>
+      <c r="AC2" s="98">
         <v>44790</v>
       </c>
-      <c r="AD2" s="82"/>
-      <c r="AE2" s="82"/>
-      <c r="AF2" s="83"/>
-      <c r="AG2" s="81">
+      <c r="AD2" s="99"/>
+      <c r="AE2" s="99"/>
+      <c r="AF2" s="100"/>
+      <c r="AG2" s="98">
         <v>44791</v>
       </c>
-      <c r="AH2" s="82"/>
-      <c r="AI2" s="82"/>
-      <c r="AJ2" s="83"/>
-      <c r="AK2" s="81">
+      <c r="AH2" s="99"/>
+      <c r="AI2" s="99"/>
+      <c r="AJ2" s="100"/>
+      <c r="AK2" s="98">
         <v>44792</v>
       </c>
-      <c r="AL2" s="82"/>
-      <c r="AM2" s="82"/>
-      <c r="AN2" s="83"/>
-      <c r="AO2" s="81">
+      <c r="AL2" s="99"/>
+      <c r="AM2" s="99"/>
+      <c r="AN2" s="100"/>
+      <c r="AO2" s="98">
         <v>44795</v>
       </c>
-      <c r="AP2" s="82"/>
-      <c r="AQ2" s="82"/>
-      <c r="AR2" s="83"/>
-      <c r="AS2" s="81"/>
-      <c r="AT2" s="82"/>
-      <c r="AU2" s="82"/>
-      <c r="AV2" s="83"/>
-      <c r="AW2" s="81"/>
-      <c r="AX2" s="82"/>
-      <c r="AY2" s="82"/>
-      <c r="AZ2" s="83"/>
+      <c r="AP2" s="99"/>
+      <c r="AQ2" s="99"/>
+      <c r="AR2" s="100"/>
+      <c r="AS2" s="98"/>
+      <c r="AT2" s="99"/>
+      <c r="AU2" s="99"/>
+      <c r="AV2" s="100"/>
+      <c r="AW2" s="98"/>
+      <c r="AX2" s="99"/>
+      <c r="AY2" s="99"/>
+      <c r="AZ2" s="100"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="86"/>
-      <c r="B3" s="92"/>
+      <c r="A3" s="112"/>
+      <c r="B3" s="103"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
@@ -1648,11 +1649,11 @@
     </row>
     <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="74" t="s">
+      <c r="B4" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="69"/>
-      <c r="D4" s="110"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="86"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1708,9 +1709,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="97"/>
-      <c r="C5" s="68"/>
-      <c r="D5" s="109"/>
+      <c r="B5" s="83"/>
+      <c r="C5" s="85"/>
+      <c r="D5" s="87"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1766,9 +1767,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="102"/>
-      <c r="C6" s="72"/>
-      <c r="D6" s="75"/>
+      <c r="B6" s="88"/>
+      <c r="C6" s="70"/>
+      <c r="D6" s="78"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1813,9 +1814,9 @@
     </row>
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="73"/>
-      <c r="C7" s="68"/>
-      <c r="D7" s="109"/>
+      <c r="B7" s="67"/>
+      <c r="C7" s="85"/>
+      <c r="D7" s="87"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1870,16 +1871,16 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="87" t="s">
+      <c r="A8" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="103" t="s">
+      <c r="B8" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="105">
+      <c r="C8" s="76">
         <v>0.1</v>
       </c>
-      <c r="D8" s="112">
+      <c r="D8" s="92">
         <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
@@ -1936,11 +1937,11 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="88"/>
-      <c r="B9" s="80"/>
-      <c r="C9" s="72"/>
-      <c r="D9" s="113"/>
-      <c r="E9" s="42"/>
+      <c r="A9" s="72"/>
+      <c r="B9" s="75"/>
+      <c r="C9" s="70"/>
+      <c r="D9" s="93"/>
+      <c r="E9" s="58"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
       <c r="H9" s="13"/>
@@ -1990,14 +1991,14 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="88"/>
-      <c r="B10" s="80" t="s">
+      <c r="A10" s="72"/>
+      <c r="B10" s="75" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="69">
+      <c r="C10" s="84">
         <v>1</v>
       </c>
-      <c r="D10" s="69">
+      <c r="D10" s="84">
         <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
@@ -2050,10 +2051,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="88"/>
-      <c r="B11" s="80"/>
-      <c r="C11" s="72"/>
-      <c r="D11" s="72"/>
+      <c r="A11" s="72"/>
+      <c r="B11" s="75"/>
+      <c r="C11" s="70"/>
+      <c r="D11" s="70"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2090,8 +2091,8 @@
       <c r="AL11" s="12"/>
       <c r="AM11" s="12"/>
       <c r="AN11" s="13"/>
-      <c r="AO11" s="11"/>
-      <c r="AP11" s="12"/>
+      <c r="AO11" s="58"/>
+      <c r="AP11" s="59"/>
       <c r="AQ11" s="12"/>
       <c r="AR11" s="13"/>
       <c r="AS11" s="11"/>
@@ -2104,12 +2105,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="88"/>
-      <c r="B12" s="80" t="s">
+      <c r="A12" s="72"/>
+      <c r="B12" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="69"/>
-      <c r="D12" s="69"/>
+      <c r="C12" s="84"/>
+      <c r="D12" s="84"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2160,10 +2161,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="88"/>
-      <c r="B13" s="80"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
+      <c r="A13" s="72"/>
+      <c r="B13" s="75"/>
+      <c r="C13" s="70"/>
+      <c r="D13" s="70"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2214,14 +2215,14 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="88"/>
-      <c r="B14" s="80" t="s">
+      <c r="A14" s="72"/>
+      <c r="B14" s="75" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="69" t="s">
+      <c r="C14" s="84" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="69" t="s">
+      <c r="D14" s="84" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="42"/>
@@ -2274,11 +2275,11 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="88"/>
-      <c r="B15" s="80"/>
-      <c r="C15" s="72"/>
-      <c r="D15" s="72"/>
-      <c r="E15" s="42"/>
+      <c r="A15" s="72"/>
+      <c r="B15" s="75"/>
+      <c r="C15" s="70"/>
+      <c r="D15" s="70"/>
+      <c r="E15" s="58"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
       <c r="H15" s="13"/>
@@ -2328,14 +2329,14 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="88"/>
-      <c r="B16" s="97" t="s">
+      <c r="A16" s="72"/>
+      <c r="B16" s="83" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="72" t="s">
+      <c r="C16" s="70" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="75" t="s">
+      <c r="D16" s="78" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="20"/>
@@ -2388,11 +2389,11 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="89"/>
-      <c r="B17" s="98"/>
-      <c r="C17" s="99"/>
-      <c r="D17" s="100"/>
-      <c r="E17" s="17"/>
+      <c r="A17" s="73"/>
+      <c r="B17" s="108"/>
+      <c r="C17" s="80"/>
+      <c r="D17" s="81"/>
+      <c r="E17" s="114"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
       <c r="H17" s="19"/>
@@ -2442,14 +2443,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="87" t="s">
+      <c r="A18" s="71" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="107" t="s">
+      <c r="B18" s="97" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="105"/>
-      <c r="D18" s="106"/>
+      <c r="C18" s="76"/>
+      <c r="D18" s="77"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2500,11 +2501,11 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="88"/>
-      <c r="B19" s="108"/>
-      <c r="C19" s="72"/>
-      <c r="D19" s="75"/>
-      <c r="E19" s="11"/>
+      <c r="A19" s="72"/>
+      <c r="B19" s="82"/>
+      <c r="C19" s="70"/>
+      <c r="D19" s="78"/>
+      <c r="E19" s="58"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
       <c r="H19" s="13"/>
@@ -2554,12 +2555,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="88"/>
-      <c r="B20" s="80" t="s">
+      <c r="A20" s="72"/>
+      <c r="B20" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="72"/>
-      <c r="D20" s="75"/>
+      <c r="C20" s="70"/>
+      <c r="D20" s="78"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2599,11 +2600,11 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="88"/>
-      <c r="B21" s="80"/>
-      <c r="C21" s="72"/>
-      <c r="D21" s="75"/>
-      <c r="E21" s="11"/>
+      <c r="A21" s="72"/>
+      <c r="B21" s="75"/>
+      <c r="C21" s="70"/>
+      <c r="D21" s="78"/>
+      <c r="E21" s="58"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
       <c r="H21" s="13"/>
@@ -2653,14 +2654,14 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="88"/>
-      <c r="B22" s="80" t="s">
+      <c r="A22" s="72"/>
+      <c r="B22" s="75" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="72">
+      <c r="C22" s="70">
         <v>0.1</v>
       </c>
-      <c r="D22" s="75">
+      <c r="D22" s="78">
         <v>0.1</v>
       </c>
       <c r="E22" s="11"/>
@@ -2713,11 +2714,11 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="88"/>
-      <c r="B23" s="80"/>
-      <c r="C23" s="72"/>
-      <c r="D23" s="75"/>
-      <c r="E23" s="11"/>
+      <c r="A23" s="72"/>
+      <c r="B23" s="75"/>
+      <c r="C23" s="70"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="58"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
       <c r="H23" s="13"/>
@@ -2767,10 +2768,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="88"/>
-      <c r="B24" s="97"/>
-      <c r="C24" s="68"/>
-      <c r="D24" s="70"/>
+      <c r="A24" s="72"/>
+      <c r="B24" s="83"/>
+      <c r="C24" s="85"/>
+      <c r="D24" s="89"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2821,10 +2822,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="88"/>
-      <c r="B25" s="74"/>
-      <c r="C25" s="69"/>
-      <c r="D25" s="71"/>
+      <c r="A25" s="72"/>
+      <c r="B25" s="68"/>
+      <c r="C25" s="84"/>
+      <c r="D25" s="90"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2875,12 +2876,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="88"/>
-      <c r="B26" s="80" t="s">
+      <c r="A26" s="72"/>
+      <c r="B26" s="75" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="68"/>
-      <c r="D26" s="70">
+      <c r="C26" s="85"/>
+      <c r="D26" s="89">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2933,10 +2934,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="89"/>
-      <c r="B27" s="80"/>
-      <c r="C27" s="101"/>
-      <c r="D27" s="111"/>
+      <c r="A27" s="73"/>
+      <c r="B27" s="75"/>
+      <c r="C27" s="109"/>
+      <c r="D27" s="91"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2987,14 +2988,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="87" t="s">
+      <c r="A28" s="71" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="103" t="s">
+      <c r="B28" s="74" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="105"/>
-      <c r="D28" s="106"/>
+      <c r="C28" s="76"/>
+      <c r="D28" s="77"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -3045,10 +3046,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="88"/>
-      <c r="B29" s="104"/>
-      <c r="C29" s="99"/>
-      <c r="D29" s="100"/>
+      <c r="A29" s="72"/>
+      <c r="B29" s="79"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="81"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3099,20 +3100,20 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="87" t="s">
+      <c r="A30" s="71" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="103" t="s">
+      <c r="B30" s="74" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="105">
+      <c r="C30" s="76">
         <v>2</v>
       </c>
-      <c r="D30" s="106">
+      <c r="D30" s="77">
         <v>2</v>
       </c>
-      <c r="E30" s="53"/>
-      <c r="F30" s="54"/>
+      <c r="E30" s="113"/>
+      <c r="F30" s="53"/>
       <c r="G30" s="47"/>
       <c r="H30" s="48"/>
       <c r="I30" s="8"/>
@@ -3161,12 +3162,12 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="88"/>
-      <c r="B31" s="80"/>
-      <c r="C31" s="72"/>
-      <c r="D31" s="75"/>
-      <c r="E31" s="59"/>
-      <c r="F31" s="60"/>
+      <c r="A31" s="72"/>
+      <c r="B31" s="75"/>
+      <c r="C31" s="70"/>
+      <c r="D31" s="78"/>
+      <c r="E31" s="42"/>
+      <c r="F31" s="59"/>
       <c r="G31" s="43"/>
       <c r="H31" s="49"/>
       <c r="I31" s="11"/>
@@ -3181,9 +3182,9 @@
       <c r="R31" s="12"/>
       <c r="S31" s="12"/>
       <c r="T31" s="13"/>
-      <c r="U31" s="59"/>
-      <c r="V31" s="60"/>
-      <c r="W31" s="60"/>
+      <c r="U31" s="58"/>
+      <c r="V31" s="59"/>
+      <c r="W31" s="59"/>
       <c r="X31" s="13"/>
       <c r="Y31" s="11"/>
       <c r="Z31" s="12"/>
@@ -3215,21 +3216,21 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="88"/>
-      <c r="B32" s="73" t="s">
+      <c r="A32" s="72"/>
+      <c r="B32" s="67" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="72">
+      <c r="C32" s="70">
         <v>4</v>
       </c>
-      <c r="D32" s="72">
+      <c r="D32" s="70">
         <v>7</v>
       </c>
       <c r="E32" s="11"/>
       <c r="F32" s="12"/>
-      <c r="G32" s="55"/>
-      <c r="H32" s="56"/>
-      <c r="I32" s="57"/>
+      <c r="G32" s="54"/>
+      <c r="H32" s="55"/>
+      <c r="I32" s="56"/>
       <c r="J32" s="12"/>
       <c r="K32" s="12"/>
       <c r="L32" s="13"/>
@@ -3275,16 +3276,16 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="88"/>
-      <c r="B33" s="74"/>
-      <c r="C33" s="72"/>
-      <c r="D33" s="72"/>
+      <c r="A33" s="72"/>
+      <c r="B33" s="68"/>
+      <c r="C33" s="70"/>
+      <c r="D33" s="70"/>
       <c r="E33" s="11"/>
-      <c r="F33" s="60"/>
-      <c r="G33" s="60"/>
-      <c r="H33" s="61"/>
-      <c r="I33" s="59"/>
-      <c r="J33" s="60"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="59"/>
+      <c r="H33" s="60"/>
+      <c r="I33" s="58"/>
+      <c r="J33" s="59"/>
       <c r="K33" s="12"/>
       <c r="L33" s="13"/>
       <c r="M33" s="11"/>
@@ -3329,21 +3330,21 @@
       <c r="AZ33" s="13"/>
     </row>
     <row r="34" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="88"/>
-      <c r="B34" s="73" t="s">
+      <c r="A34" s="72"/>
+      <c r="B34" s="67" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="72" t="s">
+      <c r="C34" s="70" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="72" t="s">
+      <c r="D34" s="70" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="11"/>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
       <c r="H34" s="13"/>
-      <c r="I34" s="57"/>
+      <c r="I34" s="56"/>
       <c r="J34" s="43"/>
       <c r="K34" s="12"/>
       <c r="L34" s="13"/>
@@ -3389,15 +3390,15 @@
       <c r="AZ34" s="13"/>
     </row>
     <row r="35" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="88"/>
-      <c r="B35" s="74"/>
-      <c r="C35" s="72"/>
-      <c r="D35" s="72"/>
+      <c r="A35" s="72"/>
+      <c r="B35" s="68"/>
+      <c r="C35" s="70"/>
+      <c r="D35" s="70"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
       <c r="H35" s="13"/>
-      <c r="I35" s="62"/>
+      <c r="I35" s="61"/>
       <c r="J35" s="12"/>
       <c r="K35" s="12"/>
       <c r="L35" s="13"/>
@@ -3443,22 +3444,22 @@
       <c r="AZ35" s="13"/>
     </row>
     <row r="36" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="88"/>
-      <c r="B36" s="73" t="s">
+      <c r="A36" s="72"/>
+      <c r="B36" s="67" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="72">
+      <c r="C36" s="70">
         <v>1.5</v>
       </c>
-      <c r="D36" s="72">
+      <c r="D36" s="70">
         <v>2</v>
       </c>
       <c r="E36" s="11"/>
       <c r="F36" s="12"/>
       <c r="G36" s="12"/>
       <c r="H36" s="13"/>
-      <c r="I36" s="58"/>
-      <c r="J36" s="55"/>
+      <c r="I36" s="57"/>
+      <c r="J36" s="54"/>
       <c r="K36" s="12"/>
       <c r="L36" s="13"/>
       <c r="M36" s="11"/>
@@ -3503,16 +3504,16 @@
       <c r="AZ36" s="13"/>
     </row>
     <row r="37" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="88"/>
-      <c r="B37" s="74"/>
-      <c r="C37" s="72"/>
-      <c r="D37" s="72"/>
+      <c r="A37" s="72"/>
+      <c r="B37" s="68"/>
+      <c r="C37" s="70"/>
+      <c r="D37" s="70"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
       <c r="H37" s="13"/>
       <c r="I37" s="50"/>
-      <c r="J37" s="60"/>
+      <c r="J37" s="59"/>
       <c r="K37" s="51"/>
       <c r="L37" s="13"/>
       <c r="M37" s="11"/>
@@ -3557,14 +3558,14 @@
       <c r="AZ37" s="13"/>
     </row>
     <row r="38" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="88"/>
-      <c r="B38" s="73" t="s">
+      <c r="A38" s="72"/>
+      <c r="B38" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="72">
+      <c r="C38" s="70">
         <v>7</v>
       </c>
-      <c r="D38" s="75">
+      <c r="D38" s="78">
         <v>6</v>
       </c>
       <c r="E38" s="11"/>
@@ -3573,10 +3574,10 @@
       <c r="H38" s="13"/>
       <c r="I38" s="11"/>
       <c r="J38" s="12"/>
-      <c r="K38" s="55"/>
-      <c r="L38" s="56"/>
-      <c r="M38" s="57"/>
-      <c r="N38" s="55"/>
+      <c r="K38" s="54"/>
+      <c r="L38" s="55"/>
+      <c r="M38" s="56"/>
+      <c r="N38" s="54"/>
       <c r="O38" s="12"/>
       <c r="P38" s="13"/>
       <c r="Q38" s="11"/>
@@ -3617,24 +3618,24 @@
       <c r="AZ38" s="13"/>
     </row>
     <row r="39" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="88"/>
-      <c r="B39" s="74"/>
-      <c r="C39" s="72"/>
-      <c r="D39" s="75"/>
+      <c r="A39" s="72"/>
+      <c r="B39" s="68"/>
+      <c r="C39" s="70"/>
+      <c r="D39" s="78"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
       <c r="H39" s="13"/>
       <c r="I39" s="11"/>
-      <c r="J39" s="60"/>
+      <c r="J39" s="59"/>
       <c r="K39" s="43"/>
       <c r="L39" s="13"/>
       <c r="M39" s="11"/>
       <c r="N39" s="12"/>
       <c r="O39" s="12"/>
       <c r="P39" s="13"/>
-      <c r="Q39" s="59"/>
-      <c r="R39" s="60"/>
+      <c r="Q39" s="58"/>
+      <c r="R39" s="59"/>
       <c r="S39" s="51"/>
       <c r="T39" s="13"/>
       <c r="U39" s="11"/>
@@ -3671,30 +3672,30 @@
       <c r="AZ39" s="13"/>
     </row>
     <row r="40" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="88"/>
-      <c r="B40" s="73" t="s">
+      <c r="A40" s="72"/>
+      <c r="B40" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="72">
+      <c r="C40" s="70">
         <v>6</v>
       </c>
-      <c r="D40" s="75"/>
+      <c r="D40" s="78"/>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
       <c r="H40" s="13"/>
       <c r="I40" s="11"/>
       <c r="J40" s="12"/>
-      <c r="K40" s="55"/>
-      <c r="L40" s="56"/>
-      <c r="M40" s="57"/>
-      <c r="N40" s="55"/>
+      <c r="K40" s="54"/>
+      <c r="L40" s="55"/>
+      <c r="M40" s="56"/>
+      <c r="N40" s="54"/>
       <c r="O40" s="12"/>
       <c r="P40" s="13"/>
       <c r="Q40" s="11"/>
       <c r="R40" s="12"/>
-      <c r="S40" s="63"/>
-      <c r="T40" s="64"/>
+      <c r="S40" s="62"/>
+      <c r="T40" s="63"/>
       <c r="U40" s="11"/>
       <c r="V40" s="12"/>
       <c r="W40" s="12"/>
@@ -3729,27 +3730,27 @@
       <c r="AZ40" s="13"/>
     </row>
     <row r="41" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="88"/>
-      <c r="B41" s="74"/>
-      <c r="C41" s="72"/>
-      <c r="D41" s="75"/>
+      <c r="A41" s="72"/>
+      <c r="B41" s="68"/>
+      <c r="C41" s="70"/>
+      <c r="D41" s="78"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
       <c r="H41" s="13"/>
       <c r="I41" s="11"/>
       <c r="J41" s="12"/>
-      <c r="K41" s="60"/>
-      <c r="L41" s="61"/>
-      <c r="M41" s="59"/>
+      <c r="K41" s="59"/>
+      <c r="L41" s="60"/>
+      <c r="M41" s="58"/>
       <c r="N41" s="43"/>
       <c r="O41" s="51"/>
-      <c r="P41" s="61"/>
+      <c r="P41" s="60"/>
       <c r="Q41" s="42"/>
       <c r="R41" s="43"/>
       <c r="S41" s="43"/>
       <c r="T41" s="49"/>
-      <c r="U41" s="59"/>
+      <c r="U41" s="58"/>
       <c r="V41" s="12"/>
       <c r="W41" s="12"/>
       <c r="X41" s="13"/>
@@ -3783,14 +3784,14 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="88"/>
-      <c r="B42" s="73" t="s">
+      <c r="A42" s="72"/>
+      <c r="B42" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="72">
+      <c r="C42" s="70">
         <v>4</v>
       </c>
-      <c r="D42" s="75">
+      <c r="D42" s="78">
         <v>2</v>
       </c>
       <c r="E42" s="11"/>
@@ -3798,8 +3799,8 @@
       <c r="G42" s="12"/>
       <c r="H42" s="13"/>
       <c r="I42" s="11"/>
-      <c r="J42" s="55"/>
-      <c r="K42" s="55"/>
+      <c r="J42" s="54"/>
+      <c r="K42" s="54"/>
       <c r="L42" s="49"/>
       <c r="M42" s="42"/>
       <c r="N42" s="43"/>
@@ -3843,17 +3844,17 @@
       <c r="AZ42" s="13"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A43" s="88"/>
-      <c r="B43" s="74"/>
-      <c r="C43" s="72"/>
-      <c r="D43" s="75"/>
+      <c r="A43" s="72"/>
+      <c r="B43" s="68"/>
+      <c r="C43" s="70"/>
+      <c r="D43" s="78"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
       <c r="H43" s="13"/>
       <c r="I43" s="11"/>
-      <c r="J43" s="60"/>
-      <c r="K43" s="60"/>
+      <c r="J43" s="59"/>
+      <c r="K43" s="59"/>
       <c r="L43" s="52"/>
       <c r="M43" s="42"/>
       <c r="N43" s="43"/>
@@ -3867,11 +3868,11 @@
       <c r="V43" s="12"/>
       <c r="W43" s="12"/>
       <c r="X43" s="13"/>
-      <c r="Y43" s="59"/>
+      <c r="Y43" s="58"/>
       <c r="Z43" s="12"/>
       <c r="AA43" s="12"/>
       <c r="AB43" s="13"/>
-      <c r="AC43" s="65"/>
+      <c r="AC43" s="64"/>
       <c r="AD43" s="12"/>
       <c r="AE43" s="12"/>
       <c r="AF43" s="13"/>
@@ -3897,12 +3898,12 @@
       <c r="AZ43" s="13"/>
     </row>
     <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="88"/>
-      <c r="B44" s="73" t="s">
+      <c r="A44" s="72"/>
+      <c r="B44" s="67" t="s">
         <v>46</v>
       </c>
-      <c r="C44" s="72"/>
-      <c r="D44" s="75"/>
+      <c r="C44" s="70"/>
+      <c r="D44" s="78"/>
       <c r="E44" s="11"/>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
@@ -3953,10 +3954,10 @@
       <c r="AZ44" s="13"/>
     </row>
     <row r="45" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="88"/>
-      <c r="B45" s="74"/>
-      <c r="C45" s="72"/>
-      <c r="D45" s="75"/>
+      <c r="A45" s="72"/>
+      <c r="B45" s="68"/>
+      <c r="C45" s="70"/>
+      <c r="D45" s="78"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
@@ -3972,17 +3973,17 @@
       <c r="Q45" s="11"/>
       <c r="R45" s="12"/>
       <c r="S45" s="12"/>
-      <c r="T45" s="61"/>
-      <c r="U45" s="59"/>
-      <c r="V45" s="60"/>
+      <c r="T45" s="60"/>
+      <c r="U45" s="58"/>
+      <c r="V45" s="59"/>
       <c r="W45" s="12"/>
       <c r="X45" s="13"/>
       <c r="Y45" s="11"/>
-      <c r="Z45" s="60"/>
-      <c r="AA45" s="60"/>
-      <c r="AB45" s="61"/>
-      <c r="AC45" s="59"/>
-      <c r="AD45" s="60"/>
+      <c r="Z45" s="59"/>
+      <c r="AA45" s="59"/>
+      <c r="AB45" s="60"/>
+      <c r="AC45" s="58"/>
+      <c r="AD45" s="59"/>
       <c r="AE45" s="12"/>
       <c r="AF45" s="13"/>
       <c r="AG45" s="11"/>
@@ -4007,12 +4008,12 @@
       <c r="AZ45" s="13"/>
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A46" s="88"/>
-      <c r="B46" s="73" t="s">
+      <c r="A46" s="72"/>
+      <c r="B46" s="67" t="s">
         <v>47</v>
       </c>
-      <c r="C46" s="76"/>
-      <c r="D46" s="75"/>
+      <c r="C46" s="69"/>
+      <c r="D46" s="78"/>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -4063,10 +4064,10 @@
       <c r="AZ46" s="13"/>
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A47" s="88"/>
-      <c r="B47" s="74"/>
-      <c r="C47" s="76"/>
-      <c r="D47" s="75"/>
+      <c r="A47" s="72"/>
+      <c r="B47" s="68"/>
+      <c r="C47" s="69"/>
+      <c r="D47" s="78"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -4085,8 +4086,8 @@
       <c r="T47" s="13"/>
       <c r="U47" s="11"/>
       <c r="V47" s="12"/>
-      <c r="W47" s="12"/>
-      <c r="X47" s="13"/>
+      <c r="W47" s="59"/>
+      <c r="X47" s="60"/>
       <c r="Y47" s="11"/>
       <c r="Z47" s="12"/>
       <c r="AA47" s="12"/>
@@ -4117,12 +4118,12 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="88"/>
-      <c r="B48" s="73" t="s">
+      <c r="A48" s="72"/>
+      <c r="B48" s="67" t="s">
         <v>48</v>
       </c>
-      <c r="C48" s="72"/>
-      <c r="D48" s="72"/>
+      <c r="C48" s="70"/>
+      <c r="D48" s="70"/>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4173,10 +4174,10 @@
       <c r="AZ48" s="13"/>
     </row>
     <row r="49" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A49" s="88"/>
-      <c r="B49" s="74"/>
-      <c r="C49" s="72"/>
-      <c r="D49" s="72"/>
+      <c r="A49" s="72"/>
+      <c r="B49" s="68"/>
+      <c r="C49" s="70"/>
+      <c r="D49" s="70"/>
       <c r="E49" s="11"/>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
@@ -4202,9 +4203,9 @@
       <c r="AA49" s="12"/>
       <c r="AB49" s="13"/>
       <c r="AC49" s="11"/>
-      <c r="AD49" s="12"/>
-      <c r="AE49" s="12"/>
-      <c r="AF49" s="13"/>
+      <c r="AD49" s="59"/>
+      <c r="AE49" s="59"/>
+      <c r="AF49" s="60"/>
       <c r="AG49" s="11"/>
       <c r="AH49" s="12"/>
       <c r="AI49" s="12"/>
@@ -4227,12 +4228,12 @@
       <c r="AZ49" s="13"/>
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A50" s="88"/>
-      <c r="B50" s="73" t="s">
+      <c r="A50" s="72"/>
+      <c r="B50" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="C50" s="72"/>
-      <c r="D50" s="72"/>
+      <c r="C50" s="70"/>
+      <c r="D50" s="70"/>
       <c r="E50" s="42"/>
       <c r="F50" s="43"/>
       <c r="G50" s="12"/>
@@ -4283,10 +4284,10 @@
       <c r="AZ50" s="13"/>
     </row>
     <row r="51" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A51" s="88"/>
-      <c r="B51" s="74"/>
-      <c r="C51" s="72"/>
-      <c r="D51" s="72"/>
+      <c r="A51" s="72"/>
+      <c r="B51" s="68"/>
+      <c r="C51" s="70"/>
+      <c r="D51" s="70"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4307,11 +4308,11 @@
       <c r="V51" s="12"/>
       <c r="W51" s="12"/>
       <c r="X51" s="13"/>
-      <c r="Y51" s="59"/>
-      <c r="Z51" s="60"/>
+      <c r="Y51" s="58"/>
+      <c r="Z51" s="59"/>
       <c r="AA51" s="12"/>
       <c r="AB51" s="13"/>
-      <c r="AC51" s="65"/>
+      <c r="AC51" s="64"/>
       <c r="AD51" s="12"/>
       <c r="AE51" s="12"/>
       <c r="AF51" s="13"/>
@@ -4337,14 +4338,14 @@
       <c r="AZ51" s="13"/>
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A52" s="88"/>
-      <c r="B52" s="73" t="s">
+      <c r="A52" s="72"/>
+      <c r="B52" s="67" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="72">
+      <c r="C52" s="70">
         <v>2</v>
       </c>
-      <c r="D52" s="72" t="s">
+      <c r="D52" s="70" t="s">
         <v>45</v>
       </c>
       <c r="E52" s="11"/>
@@ -4356,7 +4357,7 @@
       <c r="K52" s="12"/>
       <c r="L52" s="13"/>
       <c r="M52" s="11"/>
-      <c r="N52" s="55"/>
+      <c r="N52" s="54"/>
       <c r="O52" s="12"/>
       <c r="P52" s="13"/>
       <c r="Q52" s="11"/>
@@ -4397,10 +4398,10 @@
       <c r="AZ52" s="13"/>
     </row>
     <row r="53" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A53" s="88"/>
-      <c r="B53" s="74"/>
-      <c r="C53" s="72"/>
-      <c r="D53" s="72"/>
+      <c r="A53" s="72"/>
+      <c r="B53" s="68"/>
+      <c r="C53" s="70"/>
+      <c r="D53" s="70"/>
       <c r="E53" s="11"/>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
@@ -4410,8 +4411,8 @@
       <c r="K53" s="12"/>
       <c r="L53" s="13"/>
       <c r="M53" s="11"/>
-      <c r="N53" s="60"/>
-      <c r="O53" s="60"/>
+      <c r="N53" s="59"/>
+      <c r="O53" s="59"/>
       <c r="P53" s="13"/>
       <c r="Q53" s="11"/>
       <c r="R53" s="12"/>
@@ -4451,12 +4452,12 @@
       <c r="AZ53" s="13"/>
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A54" s="88"/>
-      <c r="B54" s="73" t="s">
+      <c r="A54" s="72"/>
+      <c r="B54" s="67" t="s">
         <v>50</v>
       </c>
-      <c r="C54" s="68"/>
-      <c r="D54" s="70"/>
+      <c r="C54" s="85"/>
+      <c r="D54" s="89"/>
       <c r="E54" s="11"/>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
@@ -4507,10 +4508,10 @@
       <c r="AZ54" s="13"/>
     </row>
     <row r="55" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A55" s="88"/>
-      <c r="B55" s="74"/>
-      <c r="C55" s="69"/>
-      <c r="D55" s="71"/>
+      <c r="A55" s="72"/>
+      <c r="B55" s="68"/>
+      <c r="C55" s="84"/>
+      <c r="D55" s="90"/>
       <c r="E55" s="11"/>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
@@ -4539,10 +4540,10 @@
       <c r="AD55" s="12"/>
       <c r="AE55" s="12"/>
       <c r="AF55" s="13"/>
-      <c r="AG55" s="59"/>
-      <c r="AH55" s="60"/>
-      <c r="AI55" s="60"/>
-      <c r="AJ55" s="61"/>
+      <c r="AG55" s="58"/>
+      <c r="AH55" s="59"/>
+      <c r="AI55" s="59"/>
+      <c r="AJ55" s="49"/>
       <c r="AK55" s="11"/>
       <c r="AL55" s="12"/>
       <c r="AM55" s="12"/>
@@ -4561,12 +4562,12 @@
       <c r="AZ55" s="13"/>
     </row>
     <row r="56" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A56" s="88"/>
-      <c r="B56" s="73" t="s">
+      <c r="A56" s="72"/>
+      <c r="B56" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="C56" s="72"/>
-      <c r="D56" s="72"/>
+      <c r="C56" s="70"/>
+      <c r="D56" s="70"/>
       <c r="E56" s="11"/>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
@@ -4617,10 +4618,10 @@
       <c r="AZ56" s="13"/>
     </row>
     <row r="57" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A57" s="88"/>
-      <c r="B57" s="74"/>
-      <c r="C57" s="72"/>
-      <c r="D57" s="72"/>
+      <c r="A57" s="72"/>
+      <c r="B57" s="68"/>
+      <c r="C57" s="70"/>
+      <c r="D57" s="70"/>
       <c r="E57" s="11"/>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
@@ -4653,9 +4654,9 @@
       <c r="AH57" s="12"/>
       <c r="AI57" s="12"/>
       <c r="AJ57" s="13"/>
-      <c r="AK57" s="59"/>
-      <c r="AL57" s="60"/>
-      <c r="AM57" s="60"/>
+      <c r="AK57" s="58"/>
+      <c r="AL57" s="59"/>
+      <c r="AM57" s="59"/>
       <c r="AN57" s="13"/>
       <c r="AO57" s="11"/>
       <c r="AP57" s="12"/>
@@ -4671,12 +4672,12 @@
       <c r="AZ57" s="13"/>
     </row>
     <row r="58" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="88"/>
-      <c r="B58" s="73" t="s">
+      <c r="A58" s="72"/>
+      <c r="B58" s="67" t="s">
         <v>44</v>
       </c>
-      <c r="C58" s="76"/>
-      <c r="D58" s="75"/>
+      <c r="C58" s="69"/>
+      <c r="D58" s="78"/>
       <c r="E58" s="11"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
@@ -4727,10 +4728,10 @@
       <c r="AZ58" s="13"/>
     </row>
     <row r="59" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="88"/>
-      <c r="B59" s="74"/>
-      <c r="C59" s="72"/>
-      <c r="D59" s="75"/>
+      <c r="A59" s="72"/>
+      <c r="B59" s="68"/>
+      <c r="C59" s="70"/>
+      <c r="D59" s="78"/>
       <c r="E59" s="11"/>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
@@ -4781,12 +4782,12 @@
       <c r="AZ59" s="13"/>
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A60" s="88"/>
-      <c r="B60" s="102" t="s">
+      <c r="A60" s="72"/>
+      <c r="B60" s="88" t="s">
         <v>26</v>
       </c>
-      <c r="C60" s="72"/>
-      <c r="D60" s="75"/>
+      <c r="C60" s="70"/>
+      <c r="D60" s="78"/>
       <c r="E60" s="11"/>
       <c r="F60" s="12"/>
       <c r="G60" s="12"/>
@@ -4837,10 +4838,10 @@
       <c r="AZ60" s="13"/>
     </row>
     <row r="61" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A61" s="88"/>
-      <c r="B61" s="102"/>
-      <c r="C61" s="72"/>
-      <c r="D61" s="75"/>
+      <c r="A61" s="72"/>
+      <c r="B61" s="88"/>
+      <c r="C61" s="70"/>
+      <c r="D61" s="78"/>
       <c r="E61" s="11"/>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
@@ -4891,12 +4892,12 @@
       <c r="AZ61" s="13"/>
     </row>
     <row r="62" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A62" s="88"/>
-      <c r="B62" s="80" t="s">
+      <c r="A62" s="72"/>
+      <c r="B62" s="75" t="s">
         <v>7</v>
       </c>
-      <c r="C62" s="72"/>
-      <c r="D62" s="75">
+      <c r="C62" s="70"/>
+      <c r="D62" s="78">
         <v>0</v>
       </c>
       <c r="E62" s="11"/>
@@ -4949,10 +4950,10 @@
       <c r="AZ62" s="13"/>
     </row>
     <row r="63" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="88"/>
-      <c r="B63" s="80"/>
-      <c r="C63" s="72"/>
-      <c r="D63" s="75"/>
+      <c r="A63" s="72"/>
+      <c r="B63" s="75"/>
+      <c r="C63" s="70"/>
+      <c r="D63" s="78"/>
       <c r="E63" s="11"/>
       <c r="F63" s="12"/>
       <c r="G63" s="12"/>
@@ -4983,8 +4984,8 @@
       <c r="AF63" s="13"/>
       <c r="AG63" s="11"/>
       <c r="AH63" s="12"/>
-      <c r="AI63" s="12"/>
-      <c r="AJ63" s="13"/>
+      <c r="AI63" s="59"/>
+      <c r="AJ63" s="60"/>
       <c r="AK63" s="11"/>
       <c r="AL63" s="12"/>
       <c r="AM63" s="12"/>
@@ -5003,14 +5004,14 @@
       <c r="AZ63" s="13"/>
     </row>
     <row r="64" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A64" s="87" t="s">
+      <c r="A64" s="71" t="s">
         <v>14</v>
       </c>
-      <c r="B64" s="103" t="s">
+      <c r="B64" s="74" t="s">
         <v>22</v>
       </c>
-      <c r="C64" s="105"/>
-      <c r="D64" s="106"/>
+      <c r="C64" s="76"/>
+      <c r="D64" s="77"/>
       <c r="E64" s="8"/>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -5061,10 +5062,10 @@
       <c r="AZ64" s="10"/>
     </row>
     <row r="65" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A65" s="88"/>
-      <c r="B65" s="80"/>
-      <c r="C65" s="72"/>
-      <c r="D65" s="75"/>
+      <c r="A65" s="72"/>
+      <c r="B65" s="75"/>
+      <c r="C65" s="70"/>
+      <c r="D65" s="78"/>
       <c r="E65" s="11"/>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
@@ -5115,12 +5116,12 @@
       <c r="AZ65" s="13"/>
     </row>
     <row r="66" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="88"/>
-      <c r="B66" s="73" t="s">
+      <c r="A66" s="72"/>
+      <c r="B66" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="C66" s="76"/>
-      <c r="D66" s="76"/>
+      <c r="C66" s="69"/>
+      <c r="D66" s="69"/>
       <c r="E66" s="11"/>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
@@ -5171,10 +5172,10 @@
       <c r="AZ66" s="13"/>
     </row>
     <row r="67" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="88"/>
-      <c r="B67" s="74"/>
-      <c r="C67" s="72"/>
-      <c r="D67" s="72"/>
+      <c r="A67" s="72"/>
+      <c r="B67" s="68"/>
+      <c r="C67" s="70"/>
+      <c r="D67" s="70"/>
       <c r="E67" s="11"/>
       <c r="F67" s="12"/>
       <c r="G67" s="12"/>
@@ -5225,12 +5226,12 @@
       <c r="AZ67" s="13"/>
     </row>
     <row r="68" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A68" s="88"/>
-      <c r="B68" s="80" t="s">
+      <c r="A68" s="72"/>
+      <c r="B68" s="75" t="s">
         <v>24</v>
       </c>
-      <c r="C68" s="72"/>
-      <c r="D68" s="75"/>
+      <c r="C68" s="70"/>
+      <c r="D68" s="78"/>
       <c r="E68" s="11"/>
       <c r="F68" s="12"/>
       <c r="G68" s="12"/>
@@ -5281,10 +5282,10 @@
       <c r="AZ68" s="13"/>
     </row>
     <row r="69" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="89"/>
-      <c r="B69" s="104"/>
-      <c r="C69" s="99"/>
-      <c r="D69" s="100"/>
+      <c r="A69" s="73"/>
+      <c r="B69" s="79"/>
+      <c r="C69" s="80"/>
+      <c r="D69" s="81"/>
       <c r="E69" s="17"/>
       <c r="F69" s="18"/>
       <c r="G69" s="18"/>
@@ -5319,8 +5320,8 @@
       <c r="AJ69" s="19"/>
       <c r="AK69" s="17"/>
       <c r="AL69" s="18"/>
-      <c r="AM69" s="66"/>
-      <c r="AN69" s="67"/>
+      <c r="AM69" s="65"/>
+      <c r="AN69" s="66"/>
       <c r="AO69" s="17"/>
       <c r="AP69" s="18"/>
       <c r="AQ69" s="18"/>
@@ -5335,14 +5336,14 @@
       <c r="AZ69" s="19"/>
     </row>
     <row r="70" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="87" t="s">
+      <c r="A70" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="B70" s="73" t="s">
+      <c r="B70" s="67" t="s">
         <v>25</v>
       </c>
-      <c r="C70" s="76"/>
-      <c r="D70" s="76"/>
+      <c r="C70" s="69"/>
+      <c r="D70" s="69"/>
       <c r="E70" s="11"/>
       <c r="F70" s="12"/>
       <c r="G70" s="12"/>
@@ -5393,10 +5394,10 @@
       <c r="AZ70" s="13"/>
     </row>
     <row r="71" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="88"/>
-      <c r="B71" s="74"/>
-      <c r="C71" s="72"/>
-      <c r="D71" s="72"/>
+      <c r="A71" s="72"/>
+      <c r="B71" s="68"/>
+      <c r="C71" s="70"/>
+      <c r="D71" s="70"/>
       <c r="E71" s="11"/>
       <c r="F71" s="12"/>
       <c r="G71" s="12"/>
@@ -5433,10 +5434,10 @@
       <c r="AL71" s="12"/>
       <c r="AM71" s="12"/>
       <c r="AN71" s="13"/>
-      <c r="AO71" s="11"/>
-      <c r="AP71" s="12"/>
-      <c r="AQ71" s="12"/>
-      <c r="AR71" s="13"/>
+      <c r="AO71" s="58"/>
+      <c r="AP71" s="59"/>
+      <c r="AQ71" s="59"/>
+      <c r="AR71" s="60"/>
       <c r="AS71" s="11"/>
       <c r="AT71" s="12"/>
       <c r="AU71" s="12"/>
@@ -5447,12 +5448,12 @@
       <c r="AZ71" s="13"/>
     </row>
     <row r="72" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="88"/>
-      <c r="B72" s="73" t="s">
+      <c r="A72" s="72"/>
+      <c r="B72" s="67" t="s">
         <v>7</v>
       </c>
-      <c r="C72" s="76"/>
-      <c r="D72" s="76">
+      <c r="C72" s="69"/>
+      <c r="D72" s="69">
         <v>0</v>
       </c>
       <c r="E72" s="11"/>
@@ -5505,10 +5506,10 @@
       <c r="AZ72" s="13"/>
     </row>
     <row r="73" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="89"/>
-      <c r="B73" s="108"/>
-      <c r="C73" s="72"/>
-      <c r="D73" s="72"/>
+      <c r="A73" s="73"/>
+      <c r="B73" s="82"/>
+      <c r="C73" s="70"/>
+      <c r="D73" s="70"/>
       <c r="E73" s="17"/>
       <c r="F73" s="18"/>
       <c r="G73" s="18"/>
@@ -5622,22 +5623,104 @@
     <row r="75" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="138">
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="D70:D71"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="C72:C73"/>
-    <mergeCell ref="D72:D73"/>
+    <mergeCell ref="D34:D35"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="D40:D41"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="D56:D57"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="D44:D45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="B52:B53"/>
+    <mergeCell ref="B56:B57"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="D50:D51"/>
+    <mergeCell ref="C52:C53"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="B54:B55"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="AS2:AV2"/>
+    <mergeCell ref="AW2:AZ2"/>
+    <mergeCell ref="AS1:AV1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="A8:A17"/>
+    <mergeCell ref="A18:A27"/>
+    <mergeCell ref="AK1:AN1"/>
+    <mergeCell ref="AO1:AR1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="Q1:T1"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="AK2:AN2"/>
+    <mergeCell ref="AO2:AR2"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="U2:X2"/>
+    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A63"/>
+    <mergeCell ref="A64:A69"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:C5"/>
     <mergeCell ref="D4:D5"/>
@@ -5662,104 +5745,22 @@
     <mergeCell ref="C32:C33"/>
     <mergeCell ref="D32:D33"/>
     <mergeCell ref="C34:C35"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AW1:AZ1"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A63"/>
-    <mergeCell ref="A64:A69"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="AS2:AV2"/>
-    <mergeCell ref="AW2:AZ2"/>
-    <mergeCell ref="AS1:AV1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A8:A17"/>
-    <mergeCell ref="A18:A27"/>
-    <mergeCell ref="AK1:AN1"/>
-    <mergeCell ref="AO1:AR1"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="M1:P1"/>
-    <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="AG2:AJ2"/>
-    <mergeCell ref="AK2:AN2"/>
-    <mergeCell ref="AO2:AR2"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="C56:C57"/>
-    <mergeCell ref="D56:D57"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="D44:D45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="B52:B53"/>
-    <mergeCell ref="B56:B57"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="D50:D51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="D34:D35"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="D40:D41"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="D52:D53"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="C72:C73"/>
+    <mergeCell ref="D72:D73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>

<commit_message>
Code ausführlich dokumentiert + Zeitplan aktualisi
</commit_message>
<xml_diff>
--- a/docs/PA_Fotostudio_Zeitplan.xlsx
+++ b/docs/PA_Fotostudio_Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E37E85-F071-4310-ADDF-65BC44DA3350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C4D215C-0B1F-42C9-9B1A-FC32AED8D300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -187,7 +187,7 @@
     <t>Installationsanleitung, Tests, Probleme, Bedienungsanleitung und Schlusswort schreiben</t>
   </si>
   <si>
-    <t>Dokumentation zu Ende schreiben</t>
+    <t>Dokumentation zu Ende schreiben ausser Journal</t>
   </si>
 </sst>
 </file>
@@ -800,7 +800,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -882,85 +882,33 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -972,8 +920,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -983,6 +931,24 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1005,23 +971,58 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Abwesenheit" xfId="5" xr:uid="{044D2A48-2EE8-4886-A796-1561124F3878}"/>
@@ -1356,162 +1357,162 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A1" s="110" t="s">
+      <c r="A1" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="104" t="s">
+      <c r="C1" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="105"/>
-      <c r="E1" s="94" t="s">
+      <c r="D1" s="95"/>
+      <c r="E1" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="95"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="94" t="s">
+      <c r="F1" s="79"/>
+      <c r="G1" s="79"/>
+      <c r="H1" s="80"/>
+      <c r="I1" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
-      <c r="L1" s="96"/>
-      <c r="M1" s="94" t="s">
+      <c r="J1" s="79"/>
+      <c r="K1" s="79"/>
+      <c r="L1" s="80"/>
+      <c r="M1" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="N1" s="95"/>
-      <c r="O1" s="95"/>
-      <c r="P1" s="96"/>
-      <c r="Q1" s="94" t="s">
+      <c r="N1" s="79"/>
+      <c r="O1" s="79"/>
+      <c r="P1" s="80"/>
+      <c r="Q1" s="78" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="95"/>
-      <c r="S1" s="95"/>
-      <c r="T1" s="96"/>
-      <c r="U1" s="94" t="s">
+      <c r="R1" s="79"/>
+      <c r="S1" s="79"/>
+      <c r="T1" s="80"/>
+      <c r="U1" s="78" t="s">
         <v>31</v>
       </c>
-      <c r="V1" s="95"/>
-      <c r="W1" s="95"/>
-      <c r="X1" s="96"/>
-      <c r="Y1" s="94" t="s">
+      <c r="V1" s="79"/>
+      <c r="W1" s="79"/>
+      <c r="X1" s="80"/>
+      <c r="Y1" s="78" t="s">
         <v>28</v>
       </c>
-      <c r="Z1" s="95"/>
-      <c r="AA1" s="95"/>
-      <c r="AB1" s="96"/>
-      <c r="AC1" s="94" t="s">
+      <c r="Z1" s="79"/>
+      <c r="AA1" s="79"/>
+      <c r="AB1" s="80"/>
+      <c r="AC1" s="78" t="s">
         <v>29</v>
       </c>
-      <c r="AD1" s="95"/>
-      <c r="AE1" s="95"/>
-      <c r="AF1" s="96"/>
-      <c r="AG1" s="94" t="s">
+      <c r="AD1" s="79"/>
+      <c r="AE1" s="79"/>
+      <c r="AF1" s="80"/>
+      <c r="AG1" s="78" t="s">
         <v>30</v>
       </c>
-      <c r="AH1" s="95"/>
-      <c r="AI1" s="95"/>
-      <c r="AJ1" s="96"/>
-      <c r="AK1" s="94" t="s">
+      <c r="AH1" s="79"/>
+      <c r="AI1" s="79"/>
+      <c r="AJ1" s="80"/>
+      <c r="AK1" s="78" t="s">
         <v>31</v>
       </c>
-      <c r="AL1" s="95"/>
-      <c r="AM1" s="95"/>
-      <c r="AN1" s="96"/>
-      <c r="AO1" s="94" t="s">
+      <c r="AL1" s="79"/>
+      <c r="AM1" s="79"/>
+      <c r="AN1" s="80"/>
+      <c r="AO1" s="78" t="s">
         <v>27</v>
       </c>
-      <c r="AP1" s="95"/>
-      <c r="AQ1" s="95"/>
-      <c r="AR1" s="96"/>
-      <c r="AS1" s="94"/>
-      <c r="AT1" s="95"/>
-      <c r="AU1" s="95"/>
-      <c r="AV1" s="96"/>
-      <c r="AW1" s="94"/>
-      <c r="AX1" s="95"/>
-      <c r="AY1" s="95"/>
-      <c r="AZ1" s="96"/>
+      <c r="AP1" s="79"/>
+      <c r="AQ1" s="79"/>
+      <c r="AR1" s="80"/>
+      <c r="AS1" s="78"/>
+      <c r="AT1" s="79"/>
+      <c r="AU1" s="79"/>
+      <c r="AV1" s="80"/>
+      <c r="AW1" s="78"/>
+      <c r="AX1" s="79"/>
+      <c r="AY1" s="79"/>
+      <c r="AZ1" s="80"/>
     </row>
     <row r="2" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A2" s="111"/>
-      <c r="B2" s="102"/>
-      <c r="C2" s="106"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="98">
+      <c r="A2" s="86"/>
+      <c r="B2" s="92"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="97"/>
+      <c r="E2" s="82">
         <v>44781</v>
       </c>
-      <c r="F2" s="99"/>
-      <c r="G2" s="99"/>
-      <c r="H2" s="100"/>
-      <c r="I2" s="98">
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="84"/>
+      <c r="I2" s="82">
         <v>44782</v>
       </c>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="100"/>
-      <c r="M2" s="98">
+      <c r="J2" s="83"/>
+      <c r="K2" s="83"/>
+      <c r="L2" s="84"/>
+      <c r="M2" s="82">
         <v>44783</v>
       </c>
-      <c r="N2" s="99"/>
-      <c r="O2" s="99"/>
-      <c r="P2" s="100"/>
-      <c r="Q2" s="98">
+      <c r="N2" s="83"/>
+      <c r="O2" s="83"/>
+      <c r="P2" s="84"/>
+      <c r="Q2" s="82">
         <v>44784</v>
       </c>
-      <c r="R2" s="99"/>
-      <c r="S2" s="99"/>
-      <c r="T2" s="100"/>
-      <c r="U2" s="98">
+      <c r="R2" s="83"/>
+      <c r="S2" s="83"/>
+      <c r="T2" s="84"/>
+      <c r="U2" s="82">
         <v>44785</v>
       </c>
-      <c r="V2" s="99"/>
-      <c r="W2" s="99"/>
-      <c r="X2" s="100"/>
-      <c r="Y2" s="98">
+      <c r="V2" s="83"/>
+      <c r="W2" s="83"/>
+      <c r="X2" s="84"/>
+      <c r="Y2" s="82">
         <v>44789</v>
       </c>
-      <c r="Z2" s="99"/>
-      <c r="AA2" s="99"/>
-      <c r="AB2" s="100"/>
-      <c r="AC2" s="98">
+      <c r="Z2" s="83"/>
+      <c r="AA2" s="83"/>
+      <c r="AB2" s="84"/>
+      <c r="AC2" s="82">
         <v>44790</v>
       </c>
-      <c r="AD2" s="99"/>
-      <c r="AE2" s="99"/>
-      <c r="AF2" s="100"/>
-      <c r="AG2" s="98">
+      <c r="AD2" s="83"/>
+      <c r="AE2" s="83"/>
+      <c r="AF2" s="84"/>
+      <c r="AG2" s="82">
         <v>44791</v>
       </c>
-      <c r="AH2" s="99"/>
-      <c r="AI2" s="99"/>
-      <c r="AJ2" s="100"/>
-      <c r="AK2" s="98">
+      <c r="AH2" s="83"/>
+      <c r="AI2" s="83"/>
+      <c r="AJ2" s="84"/>
+      <c r="AK2" s="82">
         <v>44792</v>
       </c>
-      <c r="AL2" s="99"/>
-      <c r="AM2" s="99"/>
-      <c r="AN2" s="100"/>
-      <c r="AO2" s="98">
+      <c r="AL2" s="83"/>
+      <c r="AM2" s="83"/>
+      <c r="AN2" s="84"/>
+      <c r="AO2" s="82">
         <v>44795</v>
       </c>
-      <c r="AP2" s="99"/>
-      <c r="AQ2" s="99"/>
-      <c r="AR2" s="100"/>
-      <c r="AS2" s="98"/>
-      <c r="AT2" s="99"/>
-      <c r="AU2" s="99"/>
-      <c r="AV2" s="100"/>
-      <c r="AW2" s="98"/>
-      <c r="AX2" s="99"/>
-      <c r="AY2" s="99"/>
-      <c r="AZ2" s="100"/>
+      <c r="AP2" s="83"/>
+      <c r="AQ2" s="83"/>
+      <c r="AR2" s="84"/>
+      <c r="AS2" s="82"/>
+      <c r="AT2" s="83"/>
+      <c r="AU2" s="83"/>
+      <c r="AV2" s="84"/>
+      <c r="AW2" s="82"/>
+      <c r="AX2" s="83"/>
+      <c r="AY2" s="83"/>
+      <c r="AZ2" s="84"/>
     </row>
     <row r="3" spans="1:55" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="112"/>
-      <c r="B3" s="103"/>
+      <c r="A3" s="87"/>
+      <c r="B3" s="93"/>
       <c r="C3" s="36" t="s">
         <v>3</v>
       </c>
@@ -1649,11 +1650,11 @@
     </row>
     <row r="4" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22"/>
-      <c r="B4" s="68" t="s">
+      <c r="B4" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="84"/>
-      <c r="D4" s="86"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="111"/>
       <c r="E4" s="38"/>
       <c r="F4" s="39"/>
       <c r="G4" s="39"/>
@@ -1709,9 +1710,9 @@
     </row>
     <row r="5" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="22"/>
-      <c r="B5" s="83"/>
-      <c r="C5" s="85"/>
-      <c r="D5" s="87"/>
+      <c r="B5" s="98"/>
+      <c r="C5" s="74"/>
+      <c r="D5" s="110"/>
       <c r="E5" s="40"/>
       <c r="F5" s="41"/>
       <c r="G5" s="41"/>
@@ -1767,9 +1768,9 @@
     </row>
     <row r="6" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="22"/>
-      <c r="B6" s="88"/>
-      <c r="C6" s="70"/>
-      <c r="D6" s="78"/>
+      <c r="B6" s="103"/>
+      <c r="C6" s="69"/>
+      <c r="D6" s="72"/>
       <c r="E6" s="42"/>
       <c r="F6" s="43"/>
       <c r="G6" s="43"/>
@@ -1814,9 +1815,9 @@
     </row>
     <row r="7" spans="1:55" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23"/>
-      <c r="B7" s="67"/>
-      <c r="C7" s="85"/>
-      <c r="D7" s="87"/>
+      <c r="B7" s="70"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="110"/>
       <c r="E7" s="44"/>
       <c r="F7" s="45"/>
       <c r="G7" s="45"/>
@@ -1871,16 +1872,16 @@
       <c r="BC7" s="27"/>
     </row>
     <row r="8" spans="1:55" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="71" t="s">
+      <c r="A8" s="88" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="74" t="s">
+      <c r="B8" s="104" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="76">
+      <c r="C8" s="106">
         <v>0.1</v>
       </c>
-      <c r="D8" s="92">
+      <c r="D8" s="113">
         <v>0.1</v>
       </c>
       <c r="E8" s="46"/>
@@ -1937,10 +1938,10 @@
       <c r="BC8" s="26"/>
     </row>
     <row r="9" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A9" s="72"/>
-      <c r="B9" s="75"/>
-      <c r="C9" s="70"/>
-      <c r="D9" s="93"/>
+      <c r="A9" s="89"/>
+      <c r="B9" s="81"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="114"/>
       <c r="E9" s="58"/>
       <c r="F9" s="43"/>
       <c r="G9" s="43"/>
@@ -1991,14 +1992,14 @@
       <c r="AZ9" s="13"/>
     </row>
     <row r="10" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="72"/>
-      <c r="B10" s="75" t="s">
+      <c r="A10" s="89"/>
+      <c r="B10" s="81" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="84">
+      <c r="C10" s="75">
         <v>1</v>
       </c>
-      <c r="D10" s="84">
+      <c r="D10" s="75">
         <v>1.5</v>
       </c>
       <c r="E10" s="42"/>
@@ -2051,10 +2052,10 @@
       <c r="AZ10" s="13"/>
     </row>
     <row r="11" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="72"/>
-      <c r="B11" s="75"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="70"/>
+      <c r="A11" s="89"/>
+      <c r="B11" s="81"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
       <c r="E11" s="42"/>
       <c r="F11" s="43"/>
       <c r="G11" s="43"/>
@@ -2105,12 +2106,12 @@
       <c r="AZ11" s="13"/>
     </row>
     <row r="12" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="72"/>
-      <c r="B12" s="75" t="s">
+      <c r="A12" s="89"/>
+      <c r="B12" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="84"/>
-      <c r="D12" s="84"/>
+      <c r="C12" s="75"/>
+      <c r="D12" s="75"/>
       <c r="E12" s="42"/>
       <c r="F12" s="43"/>
       <c r="G12" s="43"/>
@@ -2161,10 +2162,10 @@
       <c r="AZ12" s="13"/>
     </row>
     <row r="13" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="72"/>
-      <c r="B13" s="75"/>
-      <c r="C13" s="70"/>
-      <c r="D13" s="70"/>
+      <c r="A13" s="89"/>
+      <c r="B13" s="81"/>
+      <c r="C13" s="69"/>
+      <c r="D13" s="69"/>
       <c r="E13" s="42"/>
       <c r="F13" s="43"/>
       <c r="G13" s="43"/>
@@ -2215,14 +2216,14 @@
       <c r="AZ13" s="13"/>
     </row>
     <row r="14" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="72"/>
-      <c r="B14" s="75" t="s">
+      <c r="A14" s="89"/>
+      <c r="B14" s="81" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="84" t="s">
+      <c r="C14" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="84" t="s">
+      <c r="D14" s="75" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="42"/>
@@ -2275,10 +2276,10 @@
       <c r="AZ14" s="13"/>
     </row>
     <row r="15" spans="1:55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="72"/>
-      <c r="B15" s="75"/>
-      <c r="C15" s="70"/>
-      <c r="D15" s="70"/>
+      <c r="A15" s="89"/>
+      <c r="B15" s="81"/>
+      <c r="C15" s="69"/>
+      <c r="D15" s="69"/>
       <c r="E15" s="58"/>
       <c r="F15" s="43"/>
       <c r="G15" s="43"/>
@@ -2329,14 +2330,14 @@
       <c r="AZ15" s="13"/>
     </row>
     <row r="16" spans="1:55" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="72"/>
-      <c r="B16" s="83" t="s">
+      <c r="A16" s="89"/>
+      <c r="B16" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="70" t="s">
+      <c r="C16" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="78" t="s">
+      <c r="D16" s="72" t="s">
         <v>34</v>
       </c>
       <c r="E16" s="20"/>
@@ -2389,11 +2390,11 @@
       <c r="AZ16" s="13"/>
     </row>
     <row r="17" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="73"/>
-      <c r="B17" s="108"/>
-      <c r="C17" s="80"/>
-      <c r="D17" s="81"/>
-      <c r="E17" s="114"/>
+      <c r="A17" s="90"/>
+      <c r="B17" s="99"/>
+      <c r="C17" s="100"/>
+      <c r="D17" s="101"/>
+      <c r="E17" s="68"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
       <c r="H17" s="19"/>
@@ -2443,14 +2444,14 @@
       <c r="AZ17" s="19"/>
     </row>
     <row r="18" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="71" t="s">
+      <c r="A18" s="88" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="97" t="s">
+      <c r="B18" s="108" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="76"/>
-      <c r="D18" s="77"/>
+      <c r="C18" s="106"/>
+      <c r="D18" s="107"/>
       <c r="E18" s="8"/>
       <c r="F18" s="21"/>
       <c r="G18" s="29"/>
@@ -2501,10 +2502,10 @@
       <c r="AZ18" s="10"/>
     </row>
     <row r="19" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="72"/>
-      <c r="B19" s="82"/>
-      <c r="C19" s="70"/>
-      <c r="D19" s="78"/>
+      <c r="A19" s="89"/>
+      <c r="B19" s="109"/>
+      <c r="C19" s="69"/>
+      <c r="D19" s="72"/>
       <c r="E19" s="58"/>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -2555,12 +2556,12 @@
       <c r="AZ19" s="13"/>
     </row>
     <row r="20" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A20" s="72"/>
-      <c r="B20" s="75" t="s">
+      <c r="A20" s="89"/>
+      <c r="B20" s="81" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="70"/>
-      <c r="D20" s="78"/>
+      <c r="C20" s="69"/>
+      <c r="D20" s="72"/>
       <c r="E20" s="11"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -2600,10 +2601,10 @@
       <c r="AZ20" s="13"/>
     </row>
     <row r="21" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A21" s="72"/>
-      <c r="B21" s="75"/>
-      <c r="C21" s="70"/>
-      <c r="D21" s="78"/>
+      <c r="A21" s="89"/>
+      <c r="B21" s="81"/>
+      <c r="C21" s="69"/>
+      <c r="D21" s="72"/>
       <c r="E21" s="58"/>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -2654,14 +2655,14 @@
       <c r="AZ21" s="13"/>
     </row>
     <row r="22" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A22" s="72"/>
-      <c r="B22" s="75" t="s">
+      <c r="A22" s="89"/>
+      <c r="B22" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="C22" s="70">
+      <c r="C22" s="69">
         <v>0.1</v>
       </c>
-      <c r="D22" s="78">
+      <c r="D22" s="72">
         <v>0.1</v>
       </c>
       <c r="E22" s="11"/>
@@ -2714,10 +2715,10 @@
       <c r="AZ22" s="13"/>
     </row>
     <row r="23" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A23" s="72"/>
-      <c r="B23" s="75"/>
-      <c r="C23" s="70"/>
-      <c r="D23" s="78"/>
+      <c r="A23" s="89"/>
+      <c r="B23" s="81"/>
+      <c r="C23" s="69"/>
+      <c r="D23" s="72"/>
       <c r="E23" s="58"/>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -2768,10 +2769,10 @@
       <c r="AZ23" s="13"/>
     </row>
     <row r="24" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="72"/>
-      <c r="B24" s="83"/>
-      <c r="C24" s="85"/>
-      <c r="D24" s="89"/>
+      <c r="A24" s="89"/>
+      <c r="B24" s="98"/>
+      <c r="C24" s="74"/>
+      <c r="D24" s="76"/>
       <c r="E24" s="11"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -2822,10 +2823,10 @@
       <c r="AZ24" s="13"/>
     </row>
     <row r="25" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="72"/>
-      <c r="B25" s="68"/>
-      <c r="C25" s="84"/>
-      <c r="D25" s="90"/>
+      <c r="A25" s="89"/>
+      <c r="B25" s="71"/>
+      <c r="C25" s="75"/>
+      <c r="D25" s="77"/>
       <c r="E25" s="14"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15"/>
@@ -2876,12 +2877,12 @@
       <c r="AZ25" s="16"/>
     </row>
     <row r="26" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="72"/>
-      <c r="B26" s="75" t="s">
+      <c r="A26" s="89"/>
+      <c r="B26" s="81" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="85"/>
-      <c r="D26" s="89">
+      <c r="C26" s="74"/>
+      <c r="D26" s="76">
         <v>0</v>
       </c>
       <c r="E26" s="14"/>
@@ -2934,10 +2935,10 @@
       <c r="AZ26" s="16"/>
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="73"/>
-      <c r="B27" s="75"/>
-      <c r="C27" s="109"/>
-      <c r="D27" s="91"/>
+      <c r="A27" s="90"/>
+      <c r="B27" s="81"/>
+      <c r="C27" s="102"/>
+      <c r="D27" s="112"/>
       <c r="E27" s="17"/>
       <c r="F27" s="18"/>
       <c r="G27" s="18"/>
@@ -2988,14 +2989,14 @@
       <c r="AZ27" s="19"/>
     </row>
     <row r="28" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A28" s="71" t="s">
+      <c r="A28" s="88" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="74" t="s">
+      <c r="B28" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="C28" s="76"/>
-      <c r="D28" s="77"/>
+      <c r="C28" s="106"/>
+      <c r="D28" s="107"/>
       <c r="E28" s="8"/>
       <c r="F28" s="9"/>
       <c r="G28" s="9"/>
@@ -3046,10 +3047,10 @@
       <c r="AZ28" s="10"/>
     </row>
     <row r="29" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="72"/>
-      <c r="B29" s="79"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="81"/>
+      <c r="A29" s="89"/>
+      <c r="B29" s="105"/>
+      <c r="C29" s="100"/>
+      <c r="D29" s="101"/>
       <c r="E29" s="17"/>
       <c r="F29" s="18"/>
       <c r="G29" s="18"/>
@@ -3100,19 +3101,19 @@
       <c r="AZ29" s="19"/>
     </row>
     <row r="30" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A30" s="71" t="s">
+      <c r="A30" s="88" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="74" t="s">
+      <c r="B30" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="76">
+      <c r="C30" s="106">
         <v>2</v>
       </c>
-      <c r="D30" s="77">
+      <c r="D30" s="107">
         <v>2</v>
       </c>
-      <c r="E30" s="113"/>
+      <c r="E30" s="67"/>
       <c r="F30" s="53"/>
       <c r="G30" s="47"/>
       <c r="H30" s="48"/>
@@ -3162,10 +3163,10 @@
       <c r="AZ30" s="10"/>
     </row>
     <row r="31" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A31" s="72"/>
-      <c r="B31" s="75"/>
-      <c r="C31" s="70"/>
-      <c r="D31" s="78"/>
+      <c r="A31" s="89"/>
+      <c r="B31" s="81"/>
+      <c r="C31" s="69"/>
+      <c r="D31" s="72"/>
       <c r="E31" s="42"/>
       <c r="F31" s="59"/>
       <c r="G31" s="43"/>
@@ -3216,14 +3217,14 @@
       <c r="AZ31" s="13"/>
     </row>
     <row r="32" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="72"/>
-      <c r="B32" s="67" t="s">
+      <c r="A32" s="89"/>
+      <c r="B32" s="70" t="s">
         <v>36</v>
       </c>
-      <c r="C32" s="70">
+      <c r="C32" s="69">
         <v>4</v>
       </c>
-      <c r="D32" s="70">
+      <c r="D32" s="69">
         <v>7</v>
       </c>
       <c r="E32" s="11"/>
@@ -3276,10 +3277,10 @@
       <c r="AZ32" s="13"/>
     </row>
     <row r="33" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="72"/>
-      <c r="B33" s="68"/>
-      <c r="C33" s="70"/>
-      <c r="D33" s="70"/>
+      <c r="A33" s="89"/>
+      <c r="B33" s="71"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="69"/>
       <c r="E33" s="11"/>
       <c r="F33" s="59"/>
       <c r="G33" s="59"/>
@@ -3330,14 +3331,14 @@
       <c r="AZ33" s="13"/>
     </row>
     <row r="34" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="72"/>
-      <c r="B34" s="67" t="s">
+      <c r="A34" s="89"/>
+      <c r="B34" s="70" t="s">
         <v>37</v>
       </c>
-      <c r="C34" s="70" t="s">
+      <c r="C34" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="D34" s="70" t="s">
+      <c r="D34" s="69" t="s">
         <v>34</v>
       </c>
       <c r="E34" s="11"/>
@@ -3390,10 +3391,10 @@
       <c r="AZ34" s="13"/>
     </row>
     <row r="35" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="72"/>
-      <c r="B35" s="68"/>
-      <c r="C35" s="70"/>
-      <c r="D35" s="70"/>
+      <c r="A35" s="89"/>
+      <c r="B35" s="71"/>
+      <c r="C35" s="69"/>
+      <c r="D35" s="69"/>
       <c r="E35" s="11"/>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -3444,14 +3445,14 @@
       <c r="AZ35" s="13"/>
     </row>
     <row r="36" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="72"/>
-      <c r="B36" s="67" t="s">
+      <c r="A36" s="89"/>
+      <c r="B36" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="70">
+      <c r="C36" s="69">
         <v>1.5</v>
       </c>
-      <c r="D36" s="70">
+      <c r="D36" s="69">
         <v>2</v>
       </c>
       <c r="E36" s="11"/>
@@ -3504,10 +3505,10 @@
       <c r="AZ36" s="13"/>
     </row>
     <row r="37" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="72"/>
-      <c r="B37" s="68"/>
-      <c r="C37" s="70"/>
-      <c r="D37" s="70"/>
+      <c r="A37" s="89"/>
+      <c r="B37" s="71"/>
+      <c r="C37" s="69"/>
+      <c r="D37" s="69"/>
       <c r="E37" s="11"/>
       <c r="F37" s="12"/>
       <c r="G37" s="12"/>
@@ -3558,14 +3559,14 @@
       <c r="AZ37" s="13"/>
     </row>
     <row r="38" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="72"/>
-      <c r="B38" s="67" t="s">
+      <c r="A38" s="89"/>
+      <c r="B38" s="70" t="s">
         <v>39</v>
       </c>
-      <c r="C38" s="70">
+      <c r="C38" s="69">
         <v>7</v>
       </c>
-      <c r="D38" s="78">
+      <c r="D38" s="72">
         <v>6</v>
       </c>
       <c r="E38" s="11"/>
@@ -3618,10 +3619,10 @@
       <c r="AZ38" s="13"/>
     </row>
     <row r="39" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="72"/>
-      <c r="B39" s="68"/>
-      <c r="C39" s="70"/>
-      <c r="D39" s="78"/>
+      <c r="A39" s="89"/>
+      <c r="B39" s="71"/>
+      <c r="C39" s="69"/>
+      <c r="D39" s="72"/>
       <c r="E39" s="11"/>
       <c r="F39" s="12"/>
       <c r="G39" s="12"/>
@@ -3672,14 +3673,16 @@
       <c r="AZ39" s="13"/>
     </row>
     <row r="40" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="72"/>
-      <c r="B40" s="67" t="s">
+      <c r="A40" s="89"/>
+      <c r="B40" s="70" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="70">
+      <c r="C40" s="69">
         <v>6</v>
       </c>
-      <c r="D40" s="78"/>
+      <c r="D40" s="72">
+        <v>9</v>
+      </c>
       <c r="E40" s="11"/>
       <c r="F40" s="12"/>
       <c r="G40" s="12"/>
@@ -3730,10 +3733,10 @@
       <c r="AZ40" s="13"/>
     </row>
     <row r="41" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="72"/>
-      <c r="B41" s="68"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="78"/>
+      <c r="A41" s="89"/>
+      <c r="B41" s="71"/>
+      <c r="C41" s="69"/>
+      <c r="D41" s="72"/>
       <c r="E41" s="11"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
@@ -3784,14 +3787,14 @@
       <c r="AZ41" s="13"/>
     </row>
     <row r="42" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A42" s="72"/>
-      <c r="B42" s="67" t="s">
+      <c r="A42" s="89"/>
+      <c r="B42" s="70" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="70">
+      <c r="C42" s="69">
         <v>4</v>
       </c>
-      <c r="D42" s="78">
+      <c r="D42" s="72">
         <v>2</v>
       </c>
       <c r="E42" s="11"/>
@@ -3844,10 +3847,10 @@
       <c r="AZ42" s="13"/>
     </row>
     <row r="43" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A43" s="72"/>
-      <c r="B43" s="68"/>
-      <c r="C43" s="70"/>
-      <c r="D43" s="78"/>
+      <c r="A43" s="89"/>
+      <c r="B43" s="71"/>
+      <c r="C43" s="69"/>
+      <c r="D43" s="72"/>
       <c r="E43" s="11"/>
       <c r="F43" s="12"/>
       <c r="G43" s="12"/>
@@ -3898,12 +3901,16 @@
       <c r="AZ43" s="13"/>
     </row>
     <row r="44" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="72"/>
-      <c r="B44" s="67" t="s">
+      <c r="A44" s="89"/>
+      <c r="B44" s="70" t="s">
         <v>46</v>
       </c>
-      <c r="C44" s="70"/>
-      <c r="D44" s="78"/>
+      <c r="C44" s="69">
+        <v>6</v>
+      </c>
+      <c r="D44" s="72">
+        <v>13</v>
+      </c>
       <c r="E44" s="11"/>
       <c r="F44" s="12"/>
       <c r="G44" s="12"/>
@@ -3920,9 +3927,9 @@
       <c r="R44" s="12"/>
       <c r="S44" s="12"/>
       <c r="T44" s="13"/>
-      <c r="U44" s="11"/>
-      <c r="V44" s="12"/>
-      <c r="W44" s="12"/>
+      <c r="U44" s="56"/>
+      <c r="V44" s="54"/>
+      <c r="W44" s="54"/>
       <c r="X44" s="13"/>
       <c r="Y44" s="11"/>
       <c r="Z44" s="12"/>
@@ -3954,10 +3961,10 @@
       <c r="AZ44" s="13"/>
     </row>
     <row r="45" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="72"/>
-      <c r="B45" s="68"/>
-      <c r="C45" s="70"/>
-      <c r="D45" s="78"/>
+      <c r="A45" s="89"/>
+      <c r="B45" s="71"/>
+      <c r="C45" s="69"/>
+      <c r="D45" s="72"/>
       <c r="E45" s="11"/>
       <c r="F45" s="12"/>
       <c r="G45" s="12"/>
@@ -4008,12 +4015,16 @@
       <c r="AZ45" s="13"/>
     </row>
     <row r="46" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A46" s="72"/>
-      <c r="B46" s="67" t="s">
+      <c r="A46" s="89"/>
+      <c r="B46" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="C46" s="69"/>
-      <c r="D46" s="78"/>
+      <c r="C46" s="73">
+        <v>4</v>
+      </c>
+      <c r="D46" s="72">
+        <v>4</v>
+      </c>
       <c r="E46" s="11"/>
       <c r="F46" s="12"/>
       <c r="G46" s="12"/>
@@ -4032,8 +4043,8 @@
       <c r="T46" s="13"/>
       <c r="U46" s="11"/>
       <c r="V46" s="12"/>
-      <c r="W46" s="12"/>
-      <c r="X46" s="13"/>
+      <c r="W46" s="54"/>
+      <c r="X46" s="55"/>
       <c r="Y46" s="11"/>
       <c r="Z46" s="12"/>
       <c r="AA46" s="12"/>
@@ -4064,10 +4075,10 @@
       <c r="AZ46" s="13"/>
     </row>
     <row r="47" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A47" s="72"/>
-      <c r="B47" s="68"/>
-      <c r="C47" s="69"/>
-      <c r="D47" s="78"/>
+      <c r="A47" s="89"/>
+      <c r="B47" s="71"/>
+      <c r="C47" s="73"/>
+      <c r="D47" s="72"/>
       <c r="E47" s="11"/>
       <c r="F47" s="12"/>
       <c r="G47" s="12"/>
@@ -4118,12 +4129,16 @@
       <c r="AZ47" s="13"/>
     </row>
     <row r="48" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A48" s="72"/>
-      <c r="B48" s="67" t="s">
+      <c r="A48" s="89"/>
+      <c r="B48" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="C48" s="70"/>
-      <c r="D48" s="70"/>
+      <c r="C48" s="69">
+        <v>5</v>
+      </c>
+      <c r="D48" s="69">
+        <v>3</v>
+      </c>
       <c r="E48" s="11"/>
       <c r="F48" s="12"/>
       <c r="G48" s="12"/>
@@ -4144,9 +4159,9 @@
       <c r="V48" s="12"/>
       <c r="W48" s="12"/>
       <c r="X48" s="13"/>
-      <c r="Y48" s="11"/>
-      <c r="Z48" s="12"/>
-      <c r="AA48" s="12"/>
+      <c r="Y48" s="56"/>
+      <c r="Z48" s="54"/>
+      <c r="AA48" s="54"/>
       <c r="AB48" s="13"/>
       <c r="AC48" s="11"/>
       <c r="AD48" s="12"/>
@@ -4174,10 +4189,10 @@
       <c r="AZ48" s="13"/>
     </row>
     <row r="49" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A49" s="72"/>
-      <c r="B49" s="68"/>
-      <c r="C49" s="70"/>
-      <c r="D49" s="70"/>
+      <c r="A49" s="89"/>
+      <c r="B49" s="71"/>
+      <c r="C49" s="69"/>
+      <c r="D49" s="69"/>
       <c r="E49" s="11"/>
       <c r="F49" s="12"/>
       <c r="G49" s="12"/>
@@ -4228,12 +4243,16 @@
       <c r="AZ49" s="13"/>
     </row>
     <row r="50" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A50" s="72"/>
-      <c r="B50" s="67" t="s">
+      <c r="A50" s="89"/>
+      <c r="B50" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="C50" s="70"/>
-      <c r="D50" s="70"/>
+      <c r="C50" s="69">
+        <v>4</v>
+      </c>
+      <c r="D50" s="69">
+        <v>2</v>
+      </c>
       <c r="E50" s="42"/>
       <c r="F50" s="43"/>
       <c r="G50" s="12"/>
@@ -4257,8 +4276,8 @@
       <c r="Y50" s="11"/>
       <c r="Z50" s="12"/>
       <c r="AA50" s="12"/>
-      <c r="AB50" s="13"/>
-      <c r="AC50" s="11"/>
+      <c r="AB50" s="55"/>
+      <c r="AC50" s="56"/>
       <c r="AD50" s="12"/>
       <c r="AE50" s="12"/>
       <c r="AF50" s="13"/>
@@ -4284,10 +4303,10 @@
       <c r="AZ50" s="13"/>
     </row>
     <row r="51" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A51" s="72"/>
-      <c r="B51" s="68"/>
-      <c r="C51" s="70"/>
-      <c r="D51" s="70"/>
+      <c r="A51" s="89"/>
+      <c r="B51" s="71"/>
+      <c r="C51" s="69"/>
+      <c r="D51" s="69"/>
       <c r="E51" s="11"/>
       <c r="F51" s="12"/>
       <c r="G51" s="12"/>
@@ -4338,14 +4357,14 @@
       <c r="AZ51" s="13"/>
     </row>
     <row r="52" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A52" s="72"/>
-      <c r="B52" s="67" t="s">
+      <c r="A52" s="89"/>
+      <c r="B52" s="70" t="s">
         <v>43</v>
       </c>
-      <c r="C52" s="70">
+      <c r="C52" s="69">
         <v>2</v>
       </c>
-      <c r="D52" s="70" t="s">
+      <c r="D52" s="69" t="s">
         <v>45</v>
       </c>
       <c r="E52" s="11"/>
@@ -4358,7 +4377,7 @@
       <c r="L52" s="13"/>
       <c r="M52" s="11"/>
       <c r="N52" s="54"/>
-      <c r="O52" s="12"/>
+      <c r="O52" s="54"/>
       <c r="P52" s="13"/>
       <c r="Q52" s="11"/>
       <c r="R52" s="12"/>
@@ -4398,10 +4417,10 @@
       <c r="AZ52" s="13"/>
     </row>
     <row r="53" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A53" s="72"/>
-      <c r="B53" s="68"/>
-      <c r="C53" s="70"/>
-      <c r="D53" s="70"/>
+      <c r="A53" s="89"/>
+      <c r="B53" s="71"/>
+      <c r="C53" s="69"/>
+      <c r="D53" s="69"/>
       <c r="E53" s="11"/>
       <c r="F53" s="12"/>
       <c r="G53" s="12"/>
@@ -4412,7 +4431,7 @@
       <c r="L53" s="13"/>
       <c r="M53" s="11"/>
       <c r="N53" s="59"/>
-      <c r="O53" s="59"/>
+      <c r="O53" s="43"/>
       <c r="P53" s="13"/>
       <c r="Q53" s="11"/>
       <c r="R53" s="12"/>
@@ -4452,12 +4471,16 @@
       <c r="AZ53" s="13"/>
     </row>
     <row r="54" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A54" s="72"/>
-      <c r="B54" s="67" t="s">
+      <c r="A54" s="89"/>
+      <c r="B54" s="70" t="s">
         <v>50</v>
       </c>
-      <c r="C54" s="85"/>
-      <c r="D54" s="89"/>
+      <c r="C54" s="74">
+        <v>6</v>
+      </c>
+      <c r="D54" s="76">
+        <v>3.8</v>
+      </c>
       <c r="E54" s="11"/>
       <c r="F54" s="12"/>
       <c r="G54" s="12"/>
@@ -4483,9 +4506,9 @@
       <c r="AA54" s="12"/>
       <c r="AB54" s="13"/>
       <c r="AC54" s="11"/>
-      <c r="AD54" s="12"/>
-      <c r="AE54" s="12"/>
-      <c r="AF54" s="13"/>
+      <c r="AD54" s="54"/>
+      <c r="AE54" s="54"/>
+      <c r="AF54" s="55"/>
       <c r="AG54" s="11"/>
       <c r="AH54" s="12"/>
       <c r="AI54" s="12"/>
@@ -4508,10 +4531,10 @@
       <c r="AZ54" s="13"/>
     </row>
     <row r="55" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A55" s="72"/>
-      <c r="B55" s="68"/>
-      <c r="C55" s="84"/>
-      <c r="D55" s="90"/>
+      <c r="A55" s="89"/>
+      <c r="B55" s="71"/>
+      <c r="C55" s="75"/>
+      <c r="D55" s="77"/>
       <c r="E55" s="11"/>
       <c r="F55" s="12"/>
       <c r="G55" s="12"/>
@@ -4562,12 +4585,16 @@
       <c r="AZ55" s="13"/>
     </row>
     <row r="56" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A56" s="72"/>
-      <c r="B56" s="67" t="s">
+      <c r="A56" s="89"/>
+      <c r="B56" s="70" t="s">
         <v>51</v>
       </c>
-      <c r="C56" s="70"/>
-      <c r="D56" s="70"/>
+      <c r="C56" s="69">
+        <v>8</v>
+      </c>
+      <c r="D56" s="69">
+        <v>6</v>
+      </c>
       <c r="E56" s="11"/>
       <c r="F56" s="12"/>
       <c r="G56" s="12"/>
@@ -4596,10 +4623,10 @@
       <c r="AD56" s="12"/>
       <c r="AE56" s="12"/>
       <c r="AF56" s="13"/>
-      <c r="AG56" s="11"/>
-      <c r="AH56" s="12"/>
-      <c r="AI56" s="12"/>
-      <c r="AJ56" s="13"/>
+      <c r="AG56" s="56"/>
+      <c r="AH56" s="54"/>
+      <c r="AI56" s="54"/>
+      <c r="AJ56" s="55"/>
       <c r="AK56" s="11"/>
       <c r="AL56" s="12"/>
       <c r="AM56" s="12"/>
@@ -4618,10 +4645,10 @@
       <c r="AZ56" s="13"/>
     </row>
     <row r="57" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A57" s="72"/>
-      <c r="B57" s="68"/>
-      <c r="C57" s="70"/>
-      <c r="D57" s="70"/>
+      <c r="A57" s="89"/>
+      <c r="B57" s="71"/>
+      <c r="C57" s="69"/>
+      <c r="D57" s="69"/>
       <c r="E57" s="11"/>
       <c r="F57" s="12"/>
       <c r="G57" s="12"/>
@@ -4672,12 +4699,16 @@
       <c r="AZ57" s="13"/>
     </row>
     <row r="58" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="72"/>
-      <c r="B58" s="67" t="s">
+      <c r="A58" s="89"/>
+      <c r="B58" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="C58" s="69"/>
-      <c r="D58" s="78"/>
+      <c r="C58" s="73">
+        <v>2</v>
+      </c>
+      <c r="D58" s="72">
+        <v>1.5</v>
+      </c>
       <c r="E58" s="11"/>
       <c r="F58" s="12"/>
       <c r="G58" s="12"/>
@@ -4710,7 +4741,7 @@
       <c r="AH58" s="12"/>
       <c r="AI58" s="12"/>
       <c r="AJ58" s="13"/>
-      <c r="AK58" s="11"/>
+      <c r="AK58" s="56"/>
       <c r="AL58" s="12"/>
       <c r="AM58" s="12"/>
       <c r="AN58" s="13"/>
@@ -4728,10 +4759,10 @@
       <c r="AZ58" s="13"/>
     </row>
     <row r="59" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="72"/>
-      <c r="B59" s="68"/>
-      <c r="C59" s="70"/>
-      <c r="D59" s="78"/>
+      <c r="A59" s="89"/>
+      <c r="B59" s="71"/>
+      <c r="C59" s="69"/>
+      <c r="D59" s="72"/>
       <c r="E59" s="11"/>
       <c r="F59" s="12"/>
       <c r="G59" s="12"/>
@@ -4767,7 +4798,7 @@
       <c r="AK59" s="11"/>
       <c r="AL59" s="12"/>
       <c r="AM59" s="12"/>
-      <c r="AN59" s="13"/>
+      <c r="AN59" s="60"/>
       <c r="AO59" s="11"/>
       <c r="AP59" s="12"/>
       <c r="AQ59" s="12"/>
@@ -4782,12 +4813,16 @@
       <c r="AZ59" s="13"/>
     </row>
     <row r="60" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A60" s="72"/>
-      <c r="B60" s="88" t="s">
+      <c r="A60" s="89"/>
+      <c r="B60" s="103" t="s">
         <v>26</v>
       </c>
-      <c r="C60" s="70"/>
-      <c r="D60" s="78"/>
+      <c r="C60" s="69">
+        <v>2</v>
+      </c>
+      <c r="D60" s="72">
+        <v>0.5</v>
+      </c>
       <c r="E60" s="11"/>
       <c r="F60" s="12"/>
       <c r="G60" s="12"/>
@@ -4820,8 +4855,8 @@
       <c r="AH60" s="12"/>
       <c r="AI60" s="12"/>
       <c r="AJ60" s="13"/>
-      <c r="AK60" s="11"/>
-      <c r="AL60" s="12"/>
+      <c r="AK60" s="56"/>
+      <c r="AL60" s="54"/>
       <c r="AM60" s="12"/>
       <c r="AN60" s="13"/>
       <c r="AO60" s="11"/>
@@ -4838,10 +4873,10 @@
       <c r="AZ60" s="13"/>
     </row>
     <row r="61" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A61" s="72"/>
-      <c r="B61" s="88"/>
-      <c r="C61" s="70"/>
-      <c r="D61" s="78"/>
+      <c r="A61" s="89"/>
+      <c r="B61" s="103"/>
+      <c r="C61" s="69"/>
+      <c r="D61" s="72"/>
       <c r="E61" s="11"/>
       <c r="F61" s="12"/>
       <c r="G61" s="12"/>
@@ -4874,7 +4909,7 @@
       <c r="AH61" s="12"/>
       <c r="AI61" s="12"/>
       <c r="AJ61" s="13"/>
-      <c r="AK61" s="11"/>
+      <c r="AK61" s="58"/>
       <c r="AL61" s="12"/>
       <c r="AM61" s="12"/>
       <c r="AN61" s="13"/>
@@ -4892,12 +4927,12 @@
       <c r="AZ61" s="13"/>
     </row>
     <row r="62" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A62" s="72"/>
-      <c r="B62" s="75" t="s">
+      <c r="A62" s="89"/>
+      <c r="B62" s="81" t="s">
         <v>7</v>
       </c>
-      <c r="C62" s="70"/>
-      <c r="D62" s="78">
+      <c r="C62" s="69"/>
+      <c r="D62" s="72">
         <v>0</v>
       </c>
       <c r="E62" s="11"/>
@@ -4950,10 +4985,10 @@
       <c r="AZ62" s="13"/>
     </row>
     <row r="63" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="72"/>
-      <c r="B63" s="75"/>
-      <c r="C63" s="70"/>
-      <c r="D63" s="78"/>
+      <c r="A63" s="89"/>
+      <c r="B63" s="81"/>
+      <c r="C63" s="69"/>
+      <c r="D63" s="72"/>
       <c r="E63" s="11"/>
       <c r="F63" s="12"/>
       <c r="G63" s="12"/>
@@ -4984,8 +5019,8 @@
       <c r="AF63" s="13"/>
       <c r="AG63" s="11"/>
       <c r="AH63" s="12"/>
-      <c r="AI63" s="59"/>
-      <c r="AJ63" s="60"/>
+      <c r="AI63" s="43"/>
+      <c r="AJ63" s="49"/>
       <c r="AK63" s="11"/>
       <c r="AL63" s="12"/>
       <c r="AM63" s="12"/>
@@ -5004,14 +5039,18 @@
       <c r="AZ63" s="13"/>
     </row>
     <row r="64" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A64" s="71" t="s">
+      <c r="A64" s="88" t="s">
         <v>14</v>
       </c>
-      <c r="B64" s="74" t="s">
+      <c r="B64" s="104" t="s">
         <v>22</v>
       </c>
-      <c r="C64" s="76"/>
-      <c r="D64" s="77"/>
+      <c r="C64" s="106">
+        <v>5</v>
+      </c>
+      <c r="D64" s="107">
+        <v>4</v>
+      </c>
       <c r="E64" s="8"/>
       <c r="F64" s="9"/>
       <c r="G64" s="9"/>
@@ -5046,8 +5085,8 @@
       <c r="AJ64" s="10"/>
       <c r="AK64" s="8"/>
       <c r="AL64" s="9"/>
-      <c r="AM64" s="9"/>
-      <c r="AN64" s="10"/>
+      <c r="AM64" s="53"/>
+      <c r="AN64" s="115"/>
       <c r="AO64" s="8"/>
       <c r="AP64" s="9"/>
       <c r="AQ64" s="9"/>
@@ -5062,10 +5101,10 @@
       <c r="AZ64" s="10"/>
     </row>
     <row r="65" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A65" s="72"/>
-      <c r="B65" s="75"/>
-      <c r="C65" s="70"/>
-      <c r="D65" s="78"/>
+      <c r="A65" s="89"/>
+      <c r="B65" s="81"/>
+      <c r="C65" s="69"/>
+      <c r="D65" s="72"/>
       <c r="E65" s="11"/>
       <c r="F65" s="12"/>
       <c r="G65" s="12"/>
@@ -5096,8 +5135,8 @@
       <c r="AF65" s="13"/>
       <c r="AG65" s="11"/>
       <c r="AH65" s="12"/>
-      <c r="AI65" s="12"/>
-      <c r="AJ65" s="13"/>
+      <c r="AI65" s="59"/>
+      <c r="AJ65" s="60"/>
       <c r="AK65" s="11"/>
       <c r="AL65" s="12"/>
       <c r="AM65" s="12"/>
@@ -5116,12 +5155,16 @@
       <c r="AZ65" s="13"/>
     </row>
     <row r="66" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="72"/>
-      <c r="B66" s="67" t="s">
+      <c r="A66" s="89"/>
+      <c r="B66" s="70" t="s">
         <v>23</v>
       </c>
-      <c r="C66" s="69"/>
-      <c r="D66" s="69"/>
+      <c r="C66" s="73">
+        <v>6</v>
+      </c>
+      <c r="D66" s="73">
+        <v>3</v>
+      </c>
       <c r="E66" s="11"/>
       <c r="F66" s="12"/>
       <c r="G66" s="12"/>
@@ -5158,10 +5201,10 @@
       <c r="AL66" s="12"/>
       <c r="AM66" s="12"/>
       <c r="AN66" s="13"/>
-      <c r="AO66" s="11"/>
-      <c r="AP66" s="12"/>
-      <c r="AQ66" s="12"/>
-      <c r="AR66" s="13"/>
+      <c r="AO66" s="56"/>
+      <c r="AP66" s="54"/>
+      <c r="AQ66" s="54"/>
+      <c r="AR66" s="55"/>
       <c r="AS66" s="11"/>
       <c r="AT66" s="12"/>
       <c r="AU66" s="12"/>
@@ -5172,10 +5215,10 @@
       <c r="AZ66" s="13"/>
     </row>
     <row r="67" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="72"/>
-      <c r="B67" s="68"/>
-      <c r="C67" s="70"/>
-      <c r="D67" s="70"/>
+      <c r="A67" s="89"/>
+      <c r="B67" s="71"/>
+      <c r="C67" s="69"/>
+      <c r="D67" s="69"/>
       <c r="E67" s="11"/>
       <c r="F67" s="12"/>
       <c r="G67" s="12"/>
@@ -5214,8 +5257,8 @@
       <c r="AN67" s="13"/>
       <c r="AO67" s="11"/>
       <c r="AP67" s="12"/>
-      <c r="AQ67" s="12"/>
-      <c r="AR67" s="13"/>
+      <c r="AQ67" s="59"/>
+      <c r="AR67" s="60"/>
       <c r="AS67" s="11"/>
       <c r="AT67" s="12"/>
       <c r="AU67" s="12"/>
@@ -5226,12 +5269,16 @@
       <c r="AZ67" s="13"/>
     </row>
     <row r="68" spans="1:52" x14ac:dyDescent="0.25">
-      <c r="A68" s="72"/>
-      <c r="B68" s="75" t="s">
+      <c r="A68" s="89"/>
+      <c r="B68" s="81" t="s">
         <v>24</v>
       </c>
-      <c r="C68" s="70"/>
-      <c r="D68" s="78"/>
+      <c r="C68" s="69">
+        <v>4.5</v>
+      </c>
+      <c r="D68" s="72">
+        <v>4</v>
+      </c>
       <c r="E68" s="11"/>
       <c r="F68" s="12"/>
       <c r="G68" s="12"/>
@@ -5270,8 +5317,8 @@
       <c r="AN68" s="13"/>
       <c r="AO68" s="11"/>
       <c r="AP68" s="12"/>
-      <c r="AQ68" s="12"/>
-      <c r="AR68" s="13"/>
+      <c r="AQ68" s="54"/>
+      <c r="AR68" s="55"/>
       <c r="AS68" s="11"/>
       <c r="AT68" s="12"/>
       <c r="AU68" s="12"/>
@@ -5282,10 +5329,10 @@
       <c r="AZ68" s="13"/>
     </row>
     <row r="69" spans="1:52" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="73"/>
-      <c r="B69" s="79"/>
-      <c r="C69" s="80"/>
-      <c r="D69" s="81"/>
+      <c r="A69" s="90"/>
+      <c r="B69" s="105"/>
+      <c r="C69" s="100"/>
+      <c r="D69" s="101"/>
       <c r="E69" s="17"/>
       <c r="F69" s="18"/>
       <c r="G69" s="18"/>
@@ -5336,14 +5383,18 @@
       <c r="AZ69" s="19"/>
     </row>
     <row r="70" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="71" t="s">
+      <c r="A70" s="88" t="s">
         <v>15</v>
       </c>
-      <c r="B70" s="67" t="s">
+      <c r="B70" s="70" t="s">
         <v>25</v>
       </c>
-      <c r="C70" s="69"/>
-      <c r="D70" s="69"/>
+      <c r="C70" s="73">
+        <v>1.5</v>
+      </c>
+      <c r="D70" s="73">
+        <v>0.5</v>
+      </c>
       <c r="E70" s="11"/>
       <c r="F70" s="12"/>
       <c r="G70" s="12"/>
@@ -5383,7 +5434,7 @@
       <c r="AO70" s="11"/>
       <c r="AP70" s="12"/>
       <c r="AQ70" s="12"/>
-      <c r="AR70" s="13"/>
+      <c r="AR70" s="55"/>
       <c r="AS70" s="11"/>
       <c r="AT70" s="12"/>
       <c r="AU70" s="12"/>
@@ -5394,10 +5445,10 @@
       <c r="AZ70" s="13"/>
     </row>
     <row r="71" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="72"/>
-      <c r="B71" s="68"/>
-      <c r="C71" s="70"/>
-      <c r="D71" s="70"/>
+      <c r="A71" s="89"/>
+      <c r="B71" s="71"/>
+      <c r="C71" s="69"/>
+      <c r="D71" s="69"/>
       <c r="E71" s="11"/>
       <c r="F71" s="12"/>
       <c r="G71" s="12"/>
@@ -5448,12 +5499,12 @@
       <c r="AZ71" s="13"/>
     </row>
     <row r="72" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="72"/>
-      <c r="B72" s="67" t="s">
+      <c r="A72" s="89"/>
+      <c r="B72" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="C72" s="69"/>
-      <c r="D72" s="69">
+      <c r="C72" s="73"/>
+      <c r="D72" s="73">
         <v>0</v>
       </c>
       <c r="E72" s="11"/>
@@ -5506,10 +5557,10 @@
       <c r="AZ72" s="13"/>
     </row>
     <row r="73" spans="1:52" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="73"/>
-      <c r="B73" s="82"/>
-      <c r="C73" s="70"/>
-      <c r="D73" s="70"/>
+      <c r="A73" s="90"/>
+      <c r="B73" s="109"/>
+      <c r="C73" s="69"/>
+      <c r="D73" s="69"/>
       <c r="E73" s="17"/>
       <c r="F73" s="18"/>
       <c r="G73" s="18"/>
@@ -5565,11 +5616,11 @@
       </c>
       <c r="C74" s="5">
         <f>SUM(C4:C73)</f>
-        <v>27.7</v>
+        <v>81.7</v>
       </c>
       <c r="D74" s="5">
         <f>SUM(D4:D73)</f>
-        <v>20.7</v>
+        <v>75</v>
       </c>
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
@@ -5623,6 +5674,120 @@
     <row r="75" spans="1:52" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="138">
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="D66:D67"/>
+    <mergeCell ref="D70:D71"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="B70:B71"/>
+    <mergeCell ref="B64:B65"/>
+    <mergeCell ref="C64:C65"/>
+    <mergeCell ref="D64:D65"/>
+    <mergeCell ref="B68:B69"/>
+    <mergeCell ref="C68:C69"/>
+    <mergeCell ref="D68:D69"/>
+    <mergeCell ref="B72:B73"/>
+    <mergeCell ref="C72:C73"/>
+    <mergeCell ref="D72:D73"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="D42:D43"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="A30:A63"/>
+    <mergeCell ref="A64:A69"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="D62:D63"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="C62:C63"/>
+    <mergeCell ref="B58:B59"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="D58:D59"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="A8:A17"/>
+    <mergeCell ref="A18:A27"/>
+    <mergeCell ref="AK1:AN1"/>
+    <mergeCell ref="AO1:AR1"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="Q1:T1"/>
+    <mergeCell ref="AG2:AJ2"/>
+    <mergeCell ref="AK2:AN2"/>
+    <mergeCell ref="AO2:AR2"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="U2:X2"/>
+    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="AC2:AF2"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="I2:L2"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="AC1:AF1"/>
+    <mergeCell ref="AG1:AJ1"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="D54:D55"/>
+    <mergeCell ref="U1:X1"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="AS2:AV2"/>
+    <mergeCell ref="AW2:AZ2"/>
+    <mergeCell ref="AS1:AV1"/>
+    <mergeCell ref="AW1:AZ1"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
     <mergeCell ref="D34:D35"/>
     <mergeCell ref="B40:B41"/>
     <mergeCell ref="C40:C41"/>
@@ -5647,120 +5812,6 @@
     <mergeCell ref="C52:C53"/>
     <mergeCell ref="C46:C47"/>
     <mergeCell ref="B54:B55"/>
-    <mergeCell ref="C54:C55"/>
-    <mergeCell ref="D54:D55"/>
-    <mergeCell ref="U1:X1"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="AS2:AV2"/>
-    <mergeCell ref="AW2:AZ2"/>
-    <mergeCell ref="AS1:AV1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="A8:A17"/>
-    <mergeCell ref="A18:A27"/>
-    <mergeCell ref="AK1:AN1"/>
-    <mergeCell ref="AO1:AR1"/>
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="M1:P1"/>
-    <mergeCell ref="Q1:T1"/>
-    <mergeCell ref="AG2:AJ2"/>
-    <mergeCell ref="AK2:AN2"/>
-    <mergeCell ref="AO2:AR2"/>
-    <mergeCell ref="M2:P2"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="Y2:AB2"/>
-    <mergeCell ref="AC2:AF2"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="I2:L2"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="A30:A63"/>
-    <mergeCell ref="A64:A69"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:D2"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="D62:D63"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="C62:C63"/>
-    <mergeCell ref="B58:B59"/>
-    <mergeCell ref="C58:C59"/>
-    <mergeCell ref="D58:D59"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="Y1:AB1"/>
-    <mergeCell ref="AC1:AF1"/>
-    <mergeCell ref="AG1:AJ1"/>
-    <mergeCell ref="AW1:AZ1"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="D42:D43"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
-    <mergeCell ref="D66:D67"/>
-    <mergeCell ref="D70:D71"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="B70:B71"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="C64:C65"/>
-    <mergeCell ref="D64:D65"/>
-    <mergeCell ref="B68:B69"/>
-    <mergeCell ref="C68:C69"/>
-    <mergeCell ref="D68:D69"/>
-    <mergeCell ref="B72:B73"/>
-    <mergeCell ref="C72:C73"/>
-    <mergeCell ref="D72:D73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" scale="59" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>